<commit_message>
[ADD] Opt-models No smote
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4.xlsx
+++ b/results/metrics_modelling4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH87"/>
+  <dimension ref="A1:DH92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34528,6 +34528,1956 @@
       </c>
       <c r="DH87" t="n">
         <v>4.196248604251576e-17</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>LogisticRegression_splashing_opt-model</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.552828000398145, 'class_weight': 'balanced', 'penalty': 'l2'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.552828000398145, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.8478260869565217</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.8297872340425533</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0.886574074074074</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.7720364741641338</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.7766203703703703</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0.6896551724137931</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.835016835016835</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0.9440993788819876</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="R88" t="n">
+        <v>0.8611898016997168</v>
+      </c>
+      <c r="S88" t="n">
+        <v>0.9174355158730159</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0.828935149812514</v>
+      </c>
+      <c r="U88" t="n">
+        <v>0.8529761904761904</v>
+      </c>
+      <c r="V88" t="n">
+        <v>0.7058823529411765</v>
+      </c>
+      <c r="W88" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="X88" t="n">
+        <v>0.7966804979253113</v>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>0.010000228881835938, 0.009027719497680664, 0.007972478866577148, 0.008032798767089844, 0.00700831413269043, 0.0070002079010009766, 0.0069963932037353516</t>
+        </is>
+      </c>
+      <c r="Z88" t="n">
+        <v>0.008005448750087194</v>
+      </c>
+      <c r="AA88" t="n">
+        <v>0.007972478866577148</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>0.001072313919758811</v>
+      </c>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>0.020000934600830078, 0.016000032424926758, 0.015268802642822266, 0.016999006271362305, 0.015991687774658203, 0.015967845916748047, 0.014999628067016602</t>
+        </is>
+      </c>
+      <c r="AD88" t="n">
+        <v>0.01646113395690918</v>
+      </c>
+      <c r="AE88" t="n">
+        <v>0.0159916877746582</v>
+      </c>
+      <c r="AF88" t="n">
+        <v>0.00156083659277844</v>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.8113207547169812, 0.8490566037735849, 0.8113207547169812, 0.8113207547169812, 0.7547169811320755, 0.7547169811320755</t>
+        </is>
+      </c>
+      <c r="AH88" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.8166666666666667, 0.8707430340557275, 0.8413312693498451, 0.818111455108359, 0.7856037151702786, 0.7507739938080495</t>
+        </is>
+      </c>
+      <c r="AI88" t="n">
+        <v>0.8288610180914471</v>
+      </c>
+      <c r="AJ88" t="n">
+        <v>0.818111455108359</v>
+      </c>
+      <c r="AK88" t="n">
+        <v>0.05103377431461123</v>
+      </c>
+      <c r="AL88" t="n">
+        <v>0.816911250873515</v>
+      </c>
+      <c r="AM88" t="n">
+        <v>0.8113207547169812</v>
+      </c>
+      <c r="AN88" t="n">
+        <v>0.05444202474588818</v>
+      </c>
+      <c r="AO88" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8484848484848486, 0.8709677419354839, 0.8333333333333333, 0.84375, 0.7796610169491526, 0.7999999999999999</t>
+        </is>
+      </c>
+      <c r="AP88" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.7499999999999999, 0.8181818181818181, 0.782608695652174, 0.761904761904762, 0.7234042553191489, 0.6829268292682926</t>
+        </is>
+      </c>
+      <c r="AQ88" t="n">
+        <v>0.7733947432044941</v>
+      </c>
+      <c r="AR88" t="n">
+        <v>0.761904761904762</v>
+      </c>
+      <c r="AS88" t="n">
+        <v>0.06344571355692517</v>
+      </c>
+      <c r="AT88" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.7992424242424243, 0.8445747800586509, 0.8079710144927537, 0.8028273809523809, 0.7515326361341508, 0.7414634146341463</t>
+        </is>
+      </c>
+      <c r="AU88" t="n">
+        <v>0.8094869489993871</v>
+      </c>
+      <c r="AV88" t="n">
+        <v>0.8028273809523809</v>
+      </c>
+      <c r="AW88" t="n">
+        <v>0.05518455178911399</v>
+      </c>
+      <c r="AX88" t="n">
+        <v>0.8455791547942801</v>
+      </c>
+      <c r="AY88" t="n">
+        <v>0.84375</v>
+      </c>
+      <c r="AZ88" t="n">
+        <v>0.04883206875705084</v>
+      </c>
+      <c r="BA88" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.9032258064516129, 0.9642857142857143, 0.9615384615384616, 0.9, 0.92, 0.8387096774193549</t>
+        </is>
+      </c>
+      <c r="BB88" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.6818181818181818, 0.72, 0.6666666666666666, 0.6956521739130435, 0.6071428571428571, 0.6363636363636364</t>
+        </is>
+      </c>
+      <c r="BC88" t="n">
+        <v>0.7003400511442355</v>
+      </c>
+      <c r="BD88" t="n">
+        <v>0.6818181818181818</v>
+      </c>
+      <c r="BE88" t="n">
+        <v>0.08656480413235169</v>
+      </c>
+      <c r="BF88" t="n">
+        <v>0.9186595432217552</v>
+      </c>
+      <c r="BG88" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="BH88" t="n">
+        <v>0.04050754709259869</v>
+      </c>
+      <c r="BI88" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8, 0.7941176470588235, 0.7352941176470589, 0.7941176470588235, 0.6764705882352942, 0.7647058823529411</t>
+        </is>
+      </c>
+      <c r="BJ88" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8333333333333334, 0.9473684210526315, 0.9473684210526315, 0.8421052631578947, 0.8947368421052632, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="BK88" t="n">
+        <v>0.8709273182957392</v>
+      </c>
+      <c r="BL88" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM88" t="n">
+        <v>0.06870551459585363</v>
+      </c>
+      <c r="BN88" t="n">
+        <v>0.7867947178871548</v>
+      </c>
+      <c r="BO88" t="n">
+        <v>0.7941176470588235</v>
+      </c>
+      <c r="BP88" t="n">
+        <v>0.07554445485019097</v>
+      </c>
+      <c r="BQ88" t="inlineStr">
+        <is>
+          <t>0.9578947368421052, 0.8682539682539683, 0.9504643962848298, 0.8715170278637772, 0.936532507739938, 0.8297213622291021, 0.8668730650154799</t>
+        </is>
+      </c>
+      <c r="BR88" t="n">
+        <v>0.8973224377470286</v>
+      </c>
+      <c r="BS88" t="n">
+        <v>0.8715170278637772</v>
+      </c>
+      <c r="BT88" t="n">
+        <v>0.04635032065320189</v>
+      </c>
+      <c r="BU88" t="inlineStr">
+        <is>
+          <t>0.8081761006289309, 0.8181818181818182, 0.8244514106583072, 0.8244514106583072, 0.8275862068965517, 0.8275862068965517, 0.8432601880877743</t>
+        </is>
+      </c>
+      <c r="BV88" t="inlineStr">
+        <is>
+          <t>0.8234189510036694, 0.8332263585793753, 0.8401065383624022, 0.8321161611822321, 0.8405361285333792, 0.8445313171234642, 0.8486768622733911</t>
+        </is>
+      </c>
+      <c r="BW88" t="n">
+        <v>0.8375160452939875</v>
+      </c>
+      <c r="BX88" t="n">
+        <v>0.8401065383624022</v>
+      </c>
+      <c r="BY88" t="n">
+        <v>0.007891203597854857</v>
+      </c>
+      <c r="BZ88" t="n">
+        <v>0.8248133345726059</v>
+      </c>
+      <c r="CA88" t="n">
+        <v>0.8244514106583072</v>
+      </c>
+      <c r="CB88" t="n">
+        <v>0.009832167231209065</v>
+      </c>
+      <c r="CC88" t="inlineStr">
+        <is>
+          <t>0.8381962864721485, 0.8465608465608465, 0.8526315789473684, 0.8556701030927835, 0.8563968668407311, 0.8548812664907651, 0.8724489795918366</t>
+        </is>
+      </c>
+      <c r="CD88" t="inlineStr">
+        <is>
+          <t>0.7644787644787645, 0.7769230769230769, 0.7829457364341085, 0.776, 0.7843137254901961, 0.7876447876447877, 0.7967479674796748</t>
+        </is>
+      </c>
+      <c r="CE88" t="n">
+        <v>0.7812934369215155</v>
+      </c>
+      <c r="CF88" t="n">
+        <v>0.7829457364341085</v>
+      </c>
+      <c r="CG88" t="n">
+        <v>0.009417977776689589</v>
+      </c>
+      <c r="CH88" t="inlineStr">
+        <is>
+          <t>0.8013375254754564, 0.8117419617419617, 0.8177886576907385, 0.8158350515463917, 0.8203552961654637, 0.8212630270677764, 0.8345984735357557</t>
+        </is>
+      </c>
+      <c r="CI88" t="n">
+        <v>0.817559999031935</v>
+      </c>
+      <c r="CJ88" t="n">
+        <v>0.8177886576907385</v>
+      </c>
+      <c r="CK88" t="n">
+        <v>0.009349420539145593</v>
+      </c>
+      <c r="CL88" t="n">
+        <v>0.8538265611423543</v>
+      </c>
+      <c r="CM88" t="n">
+        <v>0.8548812664907651</v>
+      </c>
+      <c r="CN88" t="n">
+        <v>0.009683830910175054</v>
+      </c>
+      <c r="CO88" t="inlineStr">
+        <is>
+          <t>0.9186046511627907, 0.9248554913294798, 0.9310344827586207, 0.9120879120879121, 0.9265536723163842, 0.9364161849710982, 0.9193548387096774</t>
+        </is>
+      </c>
+      <c r="CP88" t="inlineStr">
+        <is>
+          <t>0.678082191780822, 0.6917808219178082, 0.696551724137931, 0.708029197080292, 0.704225352112676, 0.6986301369863014, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="CQ88" t="n">
+        <v>0.7020202184684268</v>
+      </c>
+      <c r="CR88" t="n">
+        <v>0.6986301369863014</v>
+      </c>
+      <c r="CS88" t="n">
+        <v>0.01678777482237482</v>
+      </c>
+      <c r="CT88" t="n">
+        <v>0.9241296047622803</v>
+      </c>
+      <c r="CU88" t="n">
+        <v>0.9248554913294798</v>
+      </c>
+      <c r="CV88" t="n">
+        <v>0.007591031115589147</v>
+      </c>
+      <c r="CW88" t="inlineStr">
+        <is>
+          <t>0.7707317073170732, 0.7804878048780488, 0.7864077669902912, 0.8058252427184466, 0.7961165048543689, 0.7864077669902912, 0.8300970873786407</t>
+        </is>
+      </c>
+      <c r="CX88" t="inlineStr">
+        <is>
+          <t>0.8761061946902655, 0.8859649122807017, 0.8938053097345132, 0.8584070796460177, 0.8849557522123894, 0.9026548672566371, 0.8672566371681416</t>
+        </is>
+      </c>
+      <c r="CY88" t="n">
+        <v>0.8813072504269523</v>
+      </c>
+      <c r="CZ88" t="n">
+        <v>0.8849557522123894</v>
+      </c>
+      <c r="DA88" t="n">
+        <v>0.01412098815595993</v>
+      </c>
+      <c r="DB88" t="n">
+        <v>0.793724840161023</v>
+      </c>
+      <c r="DC88" t="n">
+        <v>0.7864077669902912</v>
+      </c>
+      <c r="DD88" t="n">
+        <v>0.01807153464251965</v>
+      </c>
+      <c r="DE88" t="inlineStr">
+        <is>
+          <t>0.9004748543060652, 0.9134788189987163, 0.9035784861242375, 0.9139745682618782, 0.9036214451413351, 0.9203110232837873, 0.9124280436463613</t>
+        </is>
+      </c>
+      <c r="DF88" t="n">
+        <v>0.9096953199660545</v>
+      </c>
+      <c r="DG88" t="n">
+        <v>0.9124280436463613</v>
+      </c>
+      <c r="DH88" t="n">
+        <v>0.00667738577131045</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>LogisticRegression_no_fragmentation_opt-model</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 3.6236985622991797, 'class_weight': None, 'penalty': 'l2'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 3.6236985622991797, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.6296296296296297</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.723404255319149</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0.9436363636363636</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0.7985953315430696</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.8340909090909091</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0.8737864077669902</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0.8653198653198653</v>
+      </c>
+      <c r="P89" t="n">
+        <v>0.693069306930693</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0.8860759493670886</v>
+      </c>
+      <c r="R89" t="n">
+        <v>0.7777777777777777</v>
+      </c>
+      <c r="S89" t="n">
+        <v>0.937231448147718</v>
+      </c>
+      <c r="T89" t="n">
+        <v>0.8405797101449275</v>
+      </c>
+      <c r="U89" t="n">
+        <v>0.8719370572523516</v>
+      </c>
+      <c r="V89" t="n">
+        <v>0.9540816326530612</v>
+      </c>
+      <c r="W89" t="n">
+        <v>0.8577981651376146</v>
+      </c>
+      <c r="X89" t="n">
+        <v>0.9033816425120772</v>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>0.00800013542175293, 0.0069997310638427734, 0.0069997310638427734, 0.006999969482421875, 0.007001161575317383, 0.007002353668212891, 0.008000850677490234</t>
+        </is>
+      </c>
+      <c r="Z89" t="n">
+        <v>0.007286276136125837</v>
+      </c>
+      <c r="AA89" t="n">
+        <v>0.007001161575317383</v>
+      </c>
+      <c r="AB89" t="n">
+        <v>0.0004517113161977159</v>
+      </c>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>0.014000415802001953, 0.014000177383422852, 0.01300048828125, 0.01399993896484375, 0.012998580932617188, 0.013000011444091797, 0.012981653213500977</t>
+        </is>
+      </c>
+      <c r="AD89" t="n">
+        <v>0.01342589514596122</v>
+      </c>
+      <c r="AE89" t="n">
+        <v>0.01300048828125</v>
+      </c>
+      <c r="AF89" t="n">
+        <v>0.0004973783610121497</v>
+      </c>
+      <c r="AG89" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7169811320754716, 0.8867924528301887, 0.8490566037735849, 0.8867924528301887, 0.8867924528301887, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH89" t="inlineStr">
+        <is>
+          <t>0.882051282051282, 0.7161172161172161, 0.9001831501831502, 0.8745421245421245, 0.9001831501831502, 0.8543956043956045, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="AI89" t="n">
+        <v>0.8643642072213501</v>
+      </c>
+      <c r="AJ89" t="n">
+        <v>0.882051282051282</v>
+      </c>
+      <c r="AK89" t="n">
+        <v>0.06381462257831934</v>
+      </c>
+      <c r="AL89" t="n">
+        <v>0.8574423480083857</v>
+      </c>
+      <c r="AM89" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN89" t="n">
+        <v>0.05883909467264655</v>
+      </c>
+      <c r="AO89" t="inlineStr">
+        <is>
+          <t>0.8125, 0.5714285714285714, 0.8125000000000001, 0.7647058823529412, 0.8125000000000001, 0.7857142857142857, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="AP89" t="inlineStr">
+        <is>
+          <t>0.9210526315789475, 0.7887323943661971, 0.9189189189189189, 0.8888888888888888, 0.9189189189189189, 0.9230769230769231, 0.9166666666666666</t>
+        </is>
+      </c>
+      <c r="AQ89" t="n">
+        <v>0.8966079060593516</v>
+      </c>
+      <c r="AR89" t="n">
+        <v>0.9189189189189189</v>
+      </c>
+      <c r="AS89" t="n">
+        <v>0.04534436361805354</v>
+      </c>
+      <c r="AT89" t="inlineStr">
+        <is>
+          <t>0.8667763157894737, 0.6800804828973843, 0.8657094594594594, 0.826797385620915, 0.8657094594594594, 0.8543956043956045, 0.8700980392156863</t>
+        </is>
+      </c>
+      <c r="AU89" t="n">
+        <v>0.8327952495482832</v>
+      </c>
+      <c r="AV89" t="n">
+        <v>0.8657094594594594</v>
+      </c>
+      <c r="AW89" t="n">
+        <v>0.06384943344918412</v>
+      </c>
+      <c r="AX89" t="n">
+        <v>0.7689825930372149</v>
+      </c>
+      <c r="AY89" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="AZ89" t="n">
+        <v>0.08279275400268954</v>
+      </c>
+      <c r="BA89" t="inlineStr">
+        <is>
+          <t>0.7647058823529411, 0.47619047619047616, 0.7222222222222222, 0.65, 0.7222222222222222, 0.7857142857142857, 0.7</t>
+        </is>
+      </c>
+      <c r="BB89" t="inlineStr">
+        <is>
+          <t>0.9459459459459459, 0.875, 0.9714285714285714, 0.9696969696969697, 0.9714285714285714, 0.9230769230769231, 1.0</t>
+        </is>
+      </c>
+      <c r="BC89" t="n">
+        <v>0.9509395687967117</v>
+      </c>
+      <c r="BD89" t="n">
+        <v>0.9696969696969697</v>
+      </c>
+      <c r="BE89" t="n">
+        <v>0.03810970229068961</v>
+      </c>
+      <c r="BF89" t="n">
+        <v>0.6887221555288783</v>
+      </c>
+      <c r="BG89" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="BH89" t="n">
+        <v>0.09578384804489491</v>
+      </c>
+      <c r="BI89" t="inlineStr">
+        <is>
+          <t>0.8666666666666667, 0.7142857142857143, 0.9285714285714286, 0.9285714285714286, 0.9285714285714286, 0.7857142857142857, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ89" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.717948717948718, 0.8717948717948718, 0.8205128205128205, 0.8717948717948718, 0.9230769230769231, 0.8461538461538461</t>
+        </is>
+      </c>
+      <c r="BK89" t="n">
+        <v>0.8498168498168497</v>
+      </c>
+      <c r="BL89" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="BM89" t="n">
+        <v>0.061947012913142</v>
+      </c>
+      <c r="BN89" t="n">
+        <v>0.8789115646258504</v>
+      </c>
+      <c r="BO89" t="n">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="BP89" t="n">
+        <v>0.09102437378872236</v>
+      </c>
+      <c r="BQ89" t="inlineStr">
+        <is>
+          <t>0.9384615384615385, 0.9010989010989012, 0.9688644688644688, 0.924908424908425, 0.8772893772893773, 0.9413919413919414, 0.9945054945054945</t>
+        </is>
+      </c>
+      <c r="BR89" t="n">
+        <v>0.9352171637885923</v>
+      </c>
+      <c r="BS89" t="n">
+        <v>0.9384615384615385</v>
+      </c>
+      <c r="BT89" t="n">
+        <v>0.0364923779487796</v>
+      </c>
+      <c r="BU89" t="inlineStr">
+        <is>
+          <t>0.8584905660377359, 0.8808777429467085, 0.8495297805642633, 0.8557993730407524, 0.8589341692789969, 0.8652037617554859, 0.8526645768025078</t>
+        </is>
+      </c>
+      <c r="BV89" t="inlineStr">
+        <is>
+          <t>0.8656898656898657, 0.8888386123680241, 0.8562342885872298, 0.8605077928607341, 0.8588989441930618, 0.8744092508798391, 0.8546254399195575</t>
+        </is>
+      </c>
+      <c r="BW89" t="n">
+        <v>0.8656005992140445</v>
+      </c>
+      <c r="BX89" t="n">
+        <v>0.8605077928607341</v>
+      </c>
+      <c r="BY89" t="n">
+        <v>0.01131772516824489</v>
+      </c>
+      <c r="BZ89" t="n">
+        <v>0.860214281489493</v>
+      </c>
+      <c r="CA89" t="n">
+        <v>0.8584905660377359</v>
+      </c>
+      <c r="CB89" t="n">
+        <v>0.009614954516208677</v>
+      </c>
+      <c r="CC89" t="inlineStr">
+        <is>
+          <t>0.766839378238342, 0.8020833333333333, 0.7551020408163265, 0.7628865979381444, 0.7643979057591622, 0.7794871794871796, 0.7564766839378239</t>
+        </is>
+      </c>
+      <c r="CD89" t="inlineStr">
+        <is>
+          <t>0.8984198645598194, 0.914798206278027, 0.8914027149321265, 0.8963963963963965, 0.8993288590604026, 0.9029345372460497, 0.89438202247191</t>
+        </is>
+      </c>
+      <c r="CE89" t="n">
+        <v>0.8996660858492473</v>
+      </c>
+      <c r="CF89" t="n">
+        <v>0.8984198645598194</v>
+      </c>
+      <c r="CG89" t="n">
+        <v>0.007053126220958513</v>
+      </c>
+      <c r="CH89" t="inlineStr">
+        <is>
+          <t>0.8326296213990807, 0.8584407698056802, 0.8232523778742264, 0.8296414971672704, 0.8318633824097824, 0.8412108583666147, 0.8254293532048669</t>
+        </is>
+      </c>
+      <c r="CI89" t="n">
+        <v>0.8346382657467888</v>
+      </c>
+      <c r="CJ89" t="n">
+        <v>0.8318633824097824</v>
+      </c>
+      <c r="CK89" t="n">
+        <v>0.01108991183758527</v>
+      </c>
+      <c r="CL89" t="n">
+        <v>0.7696104456443302</v>
+      </c>
+      <c r="CM89" t="n">
+        <v>0.7643979057591622</v>
+      </c>
+      <c r="CN89" t="n">
+        <v>0.01518969259578258</v>
+      </c>
+      <c r="CO89" t="inlineStr">
+        <is>
+          <t>0.6788990825688074, 0.719626168224299, 0.6666666666666666, 0.6788990825688074, 0.6886792452830188, 0.6909090909090909, 0.6759259259259259</t>
+        </is>
+      </c>
+      <c r="CP89" t="inlineStr">
+        <is>
+          <t>0.9521531100478469, 0.9622641509433962, 0.9471153846153846, 0.9476190476190476, 0.9436619718309859, 0.9569377990430622, 0.943127962085308</t>
+        </is>
+      </c>
+      <c r="CQ89" t="n">
+        <v>0.9504113465978615</v>
+      </c>
+      <c r="CR89" t="n">
+        <v>0.9476190476190476</v>
+      </c>
+      <c r="CS89" t="n">
+        <v>0.006583305085779567</v>
+      </c>
+      <c r="CT89" t="n">
+        <v>0.6856578945923736</v>
+      </c>
+      <c r="CU89" t="n">
+        <v>0.6788990825688074</v>
+      </c>
+      <c r="CV89" t="n">
+        <v>0.01575385788795243</v>
+      </c>
+      <c r="CW89" t="inlineStr">
+        <is>
+          <t>0.8809523809523809, 0.9058823529411765, 0.8705882352941177, 0.8705882352941177, 0.8588235294117647, 0.8941176470588236, 0.8588235294117647</t>
+        </is>
+      </c>
+      <c r="CX89" t="inlineStr">
+        <is>
+          <t>0.8504273504273504, 0.8717948717948718, 0.8418803418803419, 0.8504273504273504, 0.8589743589743589, 0.8547008547008547, 0.8504273504273504</t>
+        </is>
+      </c>
+      <c r="CY89" t="n">
+        <v>0.8540903540903539</v>
+      </c>
+      <c r="CZ89" t="n">
+        <v>0.8504273504273504</v>
+      </c>
+      <c r="DA89" t="n">
+        <v>0.008676843958212391</v>
+      </c>
+      <c r="DB89" t="n">
+        <v>0.877110844337735</v>
+      </c>
+      <c r="DC89" t="n">
+        <v>0.8705882352941177</v>
+      </c>
+      <c r="DD89" t="n">
+        <v>0.01641310052344333</v>
+      </c>
+      <c r="DE89" t="inlineStr">
+        <is>
+          <t>0.9384411884411885, 0.9471593765711412, 0.9345399698340874, 0.9425339366515838, 0.9405731523378582, 0.9429361488185017, 0.929462041226747</t>
+        </is>
+      </c>
+      <c r="DF89" t="n">
+        <v>0.939377973411587</v>
+      </c>
+      <c r="DG89" t="n">
+        <v>0.9405731523378582</v>
+      </c>
+      <c r="DH89" t="n">
+        <v>0.005440705833764539</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_splashing_opt-model</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'distance', 'p': 2}, 'base_estimator_params': {'n_neighbors': 3, 'weights': 'distance', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.8627450980392157</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.888888888888889</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0.8811728395061729</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0.8366013071895425</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0.8287037037037037</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="M90" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0.7843137254901961</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P90" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0.9947916666666666</v>
+      </c>
+      <c r="R90" t="n">
+        <v>0.9973890339425587</v>
+      </c>
+      <c r="S90" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="T90" t="n">
+        <v>0.996324848724834</v>
+      </c>
+      <c r="U90" t="n">
+        <v>0.9973958333333333</v>
+      </c>
+      <c r="V90" t="n">
+        <v>0.9905660377358491</v>
+      </c>
+      <c r="W90" t="n">
+        <v>1</v>
+      </c>
+      <c r="X90" t="n">
+        <v>0.9952606635071091</v>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>0.010028839111328125, 0.006996870040893555, 0.006000995635986328, 0.006015300750732422, 0.006010293960571289, 0.0059702396392822266, 0.006994485855102539</t>
+        </is>
+      </c>
+      <c r="Z90" t="n">
+        <v>0.00685957499912807</v>
+      </c>
+      <c r="AA90" t="n">
+        <v>0.006015300750732422</v>
+      </c>
+      <c r="AB90" t="n">
+        <v>0.001365045215079156</v>
+      </c>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>0.01797008514404297, 0.015841007232666016, 0.015000104904174805, 0.015995264053344727, 0.015989065170288086, 0.016028881072998047, 0.014969587326049805</t>
+        </is>
+      </c>
+      <c r="AD90" t="n">
+        <v>0.01597057070050921</v>
+      </c>
+      <c r="AE90" t="n">
+        <v>0.01598906517028809</v>
+      </c>
+      <c r="AF90" t="n">
+        <v>0.0009229586112470226</v>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.8301886792452831, 0.9056603773584906, 0.9056603773584906, 0.8867924528301887, 0.8867924528301887, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH90" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.830952380952381, 0.914860681114551, 0.903250773993808, 0.8769349845201238, 0.8769349845201238, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AI90" t="n">
+        <v>0.885845917314294</v>
+      </c>
+      <c r="AJ90" t="n">
+        <v>0.8769349845201238</v>
+      </c>
+      <c r="AK90" t="n">
+        <v>0.02837456805923068</v>
+      </c>
+      <c r="AL90" t="n">
+        <v>0.8923330338424679</v>
+      </c>
+      <c r="AM90" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN90" t="n">
+        <v>0.03167885777043797</v>
+      </c>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t>0.958904109589041, 0.8656716417910447, 0.923076923076923, 0.9253731343283583, 0.9117647058823528, 0.9117647058823528, 0.9117647058823528</t>
+        </is>
+      </c>
+      <c r="AP90" t="inlineStr">
+        <is>
+          <t>0.9142857142857143, 0.7692307692307692, 0.8780487804878049, 0.8717948717948718, 0.8421052631578947, 0.8421052631578947, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="AQ90" t="n">
+        <v>0.8513822750389777</v>
+      </c>
+      <c r="AR90" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="AS90" t="n">
+        <v>0.04156179228075492</v>
+      </c>
+      <c r="AT90" t="inlineStr">
+        <is>
+          <t>0.9365949119373776, 0.8174512055109069, 0.900562851782364, 0.898584003061615, 0.8769349845201238, 0.8769349845201238, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AU90" t="n">
+        <v>0.8834282751218049</v>
+      </c>
+      <c r="AV90" t="n">
+        <v>0.8769349845201238</v>
+      </c>
+      <c r="AW90" t="n">
+        <v>0.03344386183262089</v>
+      </c>
+      <c r="AX90" t="n">
+        <v>0.9154742752046323</v>
+      </c>
+      <c r="AY90" t="n">
+        <v>0.9117647058823528</v>
+      </c>
+      <c r="AZ90" t="n">
+        <v>0.02553295682580002</v>
+      </c>
+      <c r="BA90" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.90625, 0.967741935483871, 0.9393939393939394, 0.9117647058823529, 0.9117647058823529, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BB90" t="inlineStr">
+        <is>
+          <t>1.0, 0.7142857142857143, 0.8181818181818182, 0.85, 0.8421052631578947, 0.8421052631578947, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BC90" t="n">
+        <v>0.8441119031344595</v>
+      </c>
+      <c r="BD90" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BE90" t="n">
+        <v>0.07734436617924688</v>
+      </c>
+      <c r="BF90" t="n">
+        <v>0.9242475177291167</v>
+      </c>
+      <c r="BG90" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BH90" t="n">
+        <v>0.02043371926778044</v>
+      </c>
+      <c r="BI90" t="inlineStr">
+        <is>
+          <t>1.0, 0.8285714285714286, 0.8823529411764706, 0.9117647058823529, 0.9117647058823529, 0.9117647058823529, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BJ90" t="inlineStr">
+        <is>
+          <t>0.8421052631578947, 0.8333333333333334, 0.9473684210526315, 0.8947368421052632, 0.8421052631578947, 0.8421052631578947, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BK90" t="n">
+        <v>0.8634085213032581</v>
+      </c>
+      <c r="BL90" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BM90" t="n">
+        <v>0.03918921245892704</v>
+      </c>
+      <c r="BN90" t="n">
+        <v>0.9082833133253302</v>
+      </c>
+      <c r="BO90" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BP90" t="n">
+        <v>0.04703615594400541</v>
+      </c>
+      <c r="BQ90" t="inlineStr">
+        <is>
+          <t>0.9443609022556392, 0.8563492063492063, 0.9473684210526316, 0.956656346749226, 0.8831269349845201, 0.9411764705882353, 0.945046439628483</t>
+        </is>
+      </c>
+      <c r="BR90" t="n">
+        <v>0.9248692459439918</v>
+      </c>
+      <c r="BS90" t="n">
+        <v>0.9443609022556392</v>
+      </c>
+      <c r="BT90" t="n">
+        <v>0.0358708365325814</v>
+      </c>
+      <c r="BU90" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV90" t="inlineStr">
+        <is>
+          <t>0.9975609756097561, 1.0, 0.9975728155339806, 0.9975728155339806, 0.9975728155339806, 1.0, 0.9975728155339806</t>
+        </is>
+      </c>
+      <c r="BW90" t="n">
+        <v>0.9982646053922398</v>
+      </c>
+      <c r="BX90" t="n">
+        <v>0.9975728155339806</v>
+      </c>
+      <c r="BY90" t="n">
+        <v>0.001097567218380571</v>
+      </c>
+      <c r="BZ90" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA90" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB90" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC90" t="inlineStr">
+        <is>
+          <t>0.9975550122249389, 1.0, 0.9975669099756691, 0.9975669099756691, 0.9975669099756691, 1.0, 0.9975669099756691</t>
+        </is>
+      </c>
+      <c r="CD90" t="inlineStr">
+        <is>
+          <t>0.9955947136563876, 1.0, 0.9955947136563876, 0.9955947136563876, 0.9955947136563876, 1.0, 0.9955947136563876</t>
+        </is>
+      </c>
+      <c r="CE90" t="n">
+        <v>0.9968533668974198</v>
+      </c>
+      <c r="CF90" t="n">
+        <v>0.9955947136563876</v>
+      </c>
+      <c r="CG90" t="n">
+        <v>0.001990105513007176</v>
+      </c>
+      <c r="CH90" t="inlineStr">
+        <is>
+          <t>0.9965748629406632, 1.0, 0.9965808118160284, 0.9965808118160284, 0.9965808118160284, 1.0, 0.9965808118160284</t>
+        </is>
+      </c>
+      <c r="CI90" t="n">
+        <v>0.9975568728863966</v>
+      </c>
+      <c r="CJ90" t="n">
+        <v>0.9965808118160284</v>
+      </c>
+      <c r="CK90" t="n">
+        <v>0.001545170567206118</v>
+      </c>
+      <c r="CL90" t="n">
+        <v>0.9982603788753737</v>
+      </c>
+      <c r="CM90" t="n">
+        <v>0.9975669099756691</v>
+      </c>
+      <c r="CN90" t="n">
+        <v>0.001100240355913701</v>
+      </c>
+      <c r="CO90" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP90" t="inlineStr">
+        <is>
+          <t>0.9912280701754386, 1.0, 0.9912280701754386, 0.9912280701754386, 0.9912280701754386, 1.0, 0.9912280701754386</t>
+        </is>
+      </c>
+      <c r="CQ90" t="n">
+        <v>0.9937343358395989</v>
+      </c>
+      <c r="CR90" t="n">
+        <v>0.9912280701754386</v>
+      </c>
+      <c r="CS90" t="n">
+        <v>0.003962753960110763</v>
+      </c>
+      <c r="CT90" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU90" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV90" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW90" t="inlineStr">
+        <is>
+          <t>0.9951219512195122, 1.0, 0.9951456310679612, 0.9951456310679612, 0.9951456310679612, 1.0, 0.9951456310679612</t>
+        </is>
+      </c>
+      <c r="CX90" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY90" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ90" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA90" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB90" t="n">
+        <v>0.9965292107844796</v>
+      </c>
+      <c r="DC90" t="n">
+        <v>0.9951456310679612</v>
+      </c>
+      <c r="DD90" t="n">
+        <v>0.002195134436761142</v>
+      </c>
+      <c r="DE90" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 1.0, 0.9999785204914512, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914512</t>
+        </is>
+      </c>
+      <c r="DF90" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="DG90" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="DH90" t="n">
+        <v>9.712984233443666e-06</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_no_fragmentation_opt-model</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 5, 'weights': 'distance', 'p': 1}, 'base_estimator_params': {'n_neighbors': 5, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0.9727272727272727</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0.8903508771929824</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.865909090909091</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0.9152542372881356</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0.9818181818181818</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0.9473684210526316</v>
+      </c>
+      <c r="O91" t="n">
+        <v>1</v>
+      </c>
+      <c r="P91" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>1</v>
+      </c>
+      <c r="R91" t="n">
+        <v>1</v>
+      </c>
+      <c r="S91" t="n">
+        <v>1</v>
+      </c>
+      <c r="T91" t="n">
+        <v>1</v>
+      </c>
+      <c r="U91" t="n">
+        <v>1</v>
+      </c>
+      <c r="V91" t="n">
+        <v>1</v>
+      </c>
+      <c r="W91" t="n">
+        <v>1</v>
+      </c>
+      <c r="X91" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>0.008001327514648438, 0.00699925422668457, 0.004000425338745117, 0.00500178337097168, 0.005002498626708984, 0.006001710891723633, 0.004999876022338867</t>
+        </is>
+      </c>
+      <c r="Z91" t="n">
+        <v>0.005715267998831612</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>0.005002498626708984</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>0.001277626694582705</v>
+      </c>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>0.01999688148498535, 0.014000892639160156, 0.01456141471862793, 0.014660358428955078, 0.013967752456665039, 0.012997865676879883, 0.015000581741333008</t>
+        </is>
+      </c>
+      <c r="AD91" t="n">
+        <v>0.01502653530665806</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>0.01456141471862793</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>0.002116057717912368</v>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.8301886792452831, 0.9056603773584906, 0.8679245283018868, 0.8490566037735849, 0.9245283018867925, 0.8490566037735849</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>0.8410256410256409, 0.7930402930402931, 0.8443223443223443, 0.8415750915750916, 0.7371794871794872, 0.88003663003663, 0.8516483516483516</t>
+        </is>
+      </c>
+      <c r="AI91" t="n">
+        <v>0.826975405546834</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>0.8415750915750916</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>0.04367186551670905</v>
+      </c>
+      <c r="AL91" t="n">
+        <v>0.8736148547469302</v>
+      </c>
+      <c r="AM91" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="AN91" t="n">
+        <v>0.03157037185529663</v>
+      </c>
+      <c r="AO91" t="inlineStr">
+        <is>
+          <t>0.7857142857142856, 0.689655172413793, 0.8, 0.7586206896551724, 0.6363636363636364, 0.8461538461538461, 0.75</t>
+        </is>
+      </c>
+      <c r="AP91" t="inlineStr">
+        <is>
+          <t>0.9249999999999999, 0.8831168831168831, 0.9382716049382716, 0.9090909090909091, 0.9047619047619048, 0.9500000000000001, 0.8918918918918919</t>
+        </is>
+      </c>
+      <c r="AQ91" t="n">
+        <v>0.914590456257123</v>
+      </c>
+      <c r="AR91" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="AS91" t="n">
+        <v>0.02253773745095227</v>
+      </c>
+      <c r="AT91" t="inlineStr">
+        <is>
+          <t>0.8553571428571427, 0.7863860277653381, 0.8691358024691358, 0.8338557993730407, 0.7705627705627706, 0.8980769230769231, 0.8209459459459459</t>
+        </is>
+      </c>
+      <c r="AU91" t="n">
+        <v>0.8334743445786138</v>
+      </c>
+      <c r="AV91" t="n">
+        <v>0.8338557993730407</v>
+      </c>
+      <c r="AW91" t="n">
+        <v>0.04184387921364716</v>
+      </c>
+      <c r="AX91" t="n">
+        <v>0.7523582329001048</v>
+      </c>
+      <c r="AY91" t="n">
+        <v>0.7586206896551724</v>
+      </c>
+      <c r="AZ91" t="n">
+        <v>0.06503974734665487</v>
+      </c>
+      <c r="BA91" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.6666666666666666, 0.9090909090909091, 0.7333333333333333, 0.875, 0.9166666666666666, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="BB91" t="inlineStr">
+        <is>
+          <t>0.9024390243902439, 0.8947368421052632, 0.9047619047619048, 0.9210526315789473, 0.8444444444444444, 0.926829268292683, 0.9428571428571428</t>
+        </is>
+      </c>
+      <c r="BC91" t="n">
+        <v>0.9053030369186613</v>
+      </c>
+      <c r="BD91" t="n">
+        <v>0.9047619047619048</v>
+      </c>
+      <c r="BE91" t="n">
+        <v>0.02914409370333505</v>
+      </c>
+      <c r="BF91" t="n">
+        <v>0.801939726939727</v>
+      </c>
+      <c r="BG91" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="BH91" t="n">
+        <v>0.1022886512962076</v>
+      </c>
+      <c r="BI91" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.7142857142857143, 0.7142857142857143, 0.7857142857142857, 0.5, 0.7857142857142857, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="BJ91" t="inlineStr">
+        <is>
+          <t>0.9487179487179487, 0.8717948717948718, 0.9743589743589743, 0.8974358974358975, 0.9743589743589743, 0.9743589743589743, 0.8461538461538461</t>
+        </is>
+      </c>
+      <c r="BK91" t="n">
+        <v>0.9267399267399267</v>
+      </c>
+      <c r="BL91" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="BM91" t="n">
+        <v>0.05022457582711386</v>
+      </c>
+      <c r="BN91" t="n">
+        <v>0.7272108843537415</v>
+      </c>
+      <c r="BO91" t="n">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="BP91" t="n">
+        <v>0.1040082441013137</v>
+      </c>
+      <c r="BQ91" t="inlineStr">
+        <is>
+          <t>0.9384615384615385, 0.8663003663003662, 0.9395604395604396, 0.9468864468864469, 0.9670329670329672, 0.8946886446886446, 0.9688644688644689</t>
+        </is>
+      </c>
+      <c r="BR91" t="n">
+        <v>0.9316849816849818</v>
+      </c>
+      <c r="BS91" t="n">
+        <v>0.9395604395604396</v>
+      </c>
+      <c r="BT91" t="n">
+        <v>0.03508092749628462</v>
+      </c>
+      <c r="BU91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BV91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BW91" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX91" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY91" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CD91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CE91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CI91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV91" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY91" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ91" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB91" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC91" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD91" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE91" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="DF91" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG91" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>SVC_splashing_opt-model</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 18.041415988066607, 'class_weight': None, 'coef0': 0.06653734510998605, 'degree': 2, 'gamma': 'scale'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 18.041415988066607, 'class_weight': None, 'coef0': 0.06653734510998605, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.8799999999999999</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0.8989197530864197</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0.8101851851851851</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0.8260869565217391</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0.927461139896373</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0.9322916666666666</v>
+      </c>
+      <c r="R92" t="n">
+        <v>0.9298701298701298</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0.9624751984126985</v>
+      </c>
+      <c r="T92" t="n">
+        <v>0.9003417634996582</v>
+      </c>
+      <c r="U92" t="n">
+        <v>0.8994791666666666</v>
+      </c>
+      <c r="V92" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="W92" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="X92" t="n">
+        <v>0.8708133971291866</v>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>0.01703166961669922, 0.01800060272216797, 0.014998435974121094, 0.019999027252197266, 0.016000032424926758, 0.014002799987792969, 0.014002084732055664</t>
+        </is>
+      </c>
+      <c r="Z92" t="n">
+        <v>0.01629066467285156</v>
+      </c>
+      <c r="AA92" t="n">
+        <v>0.01600003242492676</v>
+      </c>
+      <c r="AB92" t="n">
+        <v>0.002051172993857287</v>
+      </c>
+      <c r="AC92" t="inlineStr">
+        <is>
+          <t>0.016968965530395508, 0.02397298812866211, 0.020013093948364258, 0.016998767852783203, 0.016031980514526367, 0.014997720718383789, 0.0149688720703125</t>
+        </is>
+      </c>
+      <c r="AD92" t="n">
+        <v>0.01770748410906111</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>0.01696896553039551</v>
+      </c>
+      <c r="AF92" t="n">
+        <v>0.003006426250579327</v>
+      </c>
+      <c r="AG92" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.8301886792452831, 0.9056603773584906, 0.8679245283018868, 0.9245283018867925, 0.8490566037735849, 0.8490566037735849</t>
+        </is>
+      </c>
+      <c r="AH92" t="inlineStr">
+        <is>
+          <t>0.9067669172932331, 0.803968253968254, 0.891640866873065, 0.8738390092879257, 0.9179566563467492, 0.8243034055727554, 0.8126934984520124</t>
+        </is>
+      </c>
+      <c r="AI92" t="n">
+        <v>0.8615955153991421</v>
+      </c>
+      <c r="AJ92" t="n">
+        <v>0.8738390092879257</v>
+      </c>
+      <c r="AK92" t="n">
+        <v>0.04370791040306145</v>
+      </c>
+      <c r="AL92" t="n">
+        <v>0.8789058600379356</v>
+      </c>
+      <c r="AM92" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="AN92" t="n">
+        <v>0.03641822060368381</v>
+      </c>
+      <c r="AO92" t="inlineStr">
+        <is>
+          <t>0.9444444444444445, 0.8732394366197184, 0.9275362318840579, 0.8923076923076922, 0.9411764705882353, 0.8857142857142858, 0.8888888888888888</t>
+        </is>
+      </c>
+      <c r="AP92" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7428571428571428, 0.8648648648648649, 0.8292682926829269, 0.8947368421052632, 0.7777777777777778, 0.7647058823529413</t>
+        </is>
+      </c>
+      <c r="AQ92" t="n">
+        <v>0.8232999559328293</v>
+      </c>
+      <c r="AR92" t="n">
+        <v>0.8292682926829269</v>
+      </c>
+      <c r="AS92" t="n">
+        <v>0.05750152776680204</v>
+      </c>
+      <c r="AT92" t="inlineStr">
+        <is>
+          <t>0.9166666666666667, 0.8080482897384306, 0.8962005483744614, 0.8607879924953096, 0.9179566563467492, 0.8317460317460318, 0.8267973856209151</t>
+        </is>
+      </c>
+      <c r="AU92" t="n">
+        <v>0.8654576529983663</v>
+      </c>
+      <c r="AV92" t="n">
+        <v>0.8607879924953096</v>
+      </c>
+      <c r="AW92" t="n">
+        <v>0.04187117052825106</v>
+      </c>
+      <c r="AX92" t="n">
+        <v>0.9076153500639033</v>
+      </c>
+      <c r="AY92" t="n">
+        <v>0.8923076923076922</v>
+      </c>
+      <c r="AZ92" t="n">
+        <v>0.02706061269267544</v>
+      </c>
+      <c r="BA92" t="inlineStr">
+        <is>
+          <t>0.918918918918919, 0.8611111111111112, 0.9142857142857143, 0.9354838709677419, 0.9411764705882353, 0.8611111111111112, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BB92" t="inlineStr">
+        <is>
+          <t>0.9411764705882353, 0.7647058823529411, 0.8888888888888888, 0.7727272727272727, 0.8947368421052632, 0.8235294117647058, 0.8666666666666667</t>
+        </is>
+      </c>
+      <c r="BC92" t="n">
+        <v>0.8503473478705674</v>
+      </c>
+      <c r="BD92" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="BE92" t="n">
+        <v>0.06100429219131633</v>
+      </c>
+      <c r="BF92" t="n">
+        <v>0.8963132085915325</v>
+      </c>
+      <c r="BG92" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="BH92" t="n">
+        <v>0.03741267709229684</v>
+      </c>
+      <c r="BI92" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.8857142857142857, 0.9411764705882353, 0.8529411764705882, 0.9411764705882353, 0.9117647058823529, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="BJ92" t="inlineStr">
+        <is>
+          <t>0.8421052631578947, 0.7222222222222222, 0.8421052631578947, 0.8947368421052632, 0.8947368421052632, 0.7368421052631579, 0.6842105263157895</t>
+        </is>
+      </c>
+      <c r="BK92" t="n">
+        <v>0.802422723475355</v>
+      </c>
+      <c r="BL92" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BM92" t="n">
+        <v>0.08008946992652823</v>
+      </c>
+      <c r="BN92" t="n">
+        <v>0.9207683073229292</v>
+      </c>
+      <c r="BO92" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="BP92" t="n">
+        <v>0.03727563488458872</v>
+      </c>
+      <c r="BQ92" t="inlineStr">
+        <is>
+          <t>0.9804511278195489, 0.8666666666666666, 0.9489164086687306, 0.9396284829721362, 0.9674922600619195, 0.9396284829721362, 0.9040247678018576</t>
+        </is>
+      </c>
+      <c r="BR92" t="n">
+        <v>0.9352583138518564</v>
+      </c>
+      <c r="BS92" t="n">
+        <v>0.9396284829721362</v>
+      </c>
+      <c r="BT92" t="n">
+        <v>0.03582996849273579</v>
+      </c>
+      <c r="BU92" t="inlineStr">
+        <is>
+          <t>0.8962264150943396, 0.9247648902821317, 0.9059561128526645, 0.9153605015673981, 0.9028213166144201, 0.9059561128526645, 0.9247648902821317</t>
+        </is>
+      </c>
+      <c r="BV92" t="inlineStr">
+        <is>
+          <t>0.8857543708180444, 0.9161531878476679, 0.895222957298737, 0.9045021049918378, 0.8927957728327176, 0.8932253630036945, 0.9157788469799811</t>
+        </is>
+      </c>
+      <c r="BW92" t="n">
+        <v>0.9004903719675258</v>
+      </c>
+      <c r="BX92" t="n">
+        <v>0.895222957298737</v>
+      </c>
+      <c r="BY92" t="n">
+        <v>0.01103266493917355</v>
+      </c>
+      <c r="BZ92" t="n">
+        <v>0.9108357485065357</v>
+      </c>
+      <c r="CA92" t="n">
+        <v>0.9059561128526645</v>
+      </c>
+      <c r="CB92" t="n">
+        <v>0.01023858807929395</v>
+      </c>
+      <c r="CC92" t="inlineStr">
+        <is>
+          <t>0.9197080291970803, 0.9417475728155339, 0.927536231884058, 0.9349397590361446, 0.9249394673123488, 0.9278846153846153, 0.9420289855072463</t>
+        </is>
+      </c>
+      <c r="CD92" t="inlineStr">
+        <is>
+          <t>0.8533333333333332, 0.8938053097345132, 0.8660714285714286, 0.8789237668161435, 0.8622222222222222, 0.8648648648648649, 0.8928571428571428</t>
+        </is>
+      </c>
+      <c r="CE92" t="n">
+        <v>0.8731540097713785</v>
+      </c>
+      <c r="CF92" t="n">
+        <v>0.8660714285714286</v>
+      </c>
+      <c r="CG92" t="n">
+        <v>0.01453673088192685</v>
+      </c>
+      <c r="CH92" t="inlineStr">
+        <is>
+          <t>0.8865206812652067, 0.9177764412750236, 0.8968038302277432, 0.906931762926144, 0.8935808447672855, 0.8963747401247402, 0.9174430641821946</t>
+        </is>
+      </c>
+      <c r="CI92" t="n">
+        <v>0.902204480681191</v>
+      </c>
+      <c r="CJ92" t="n">
+        <v>0.8968038302277432</v>
+      </c>
+      <c r="CK92" t="n">
+        <v>0.01121573602481712</v>
+      </c>
+      <c r="CL92" t="n">
+        <v>0.9312549515910039</v>
+      </c>
+      <c r="CM92" t="n">
+        <v>0.9278846153846153</v>
+      </c>
+      <c r="CN92" t="n">
+        <v>0.007911632608703652</v>
+      </c>
+      <c r="CO92" t="inlineStr">
+        <is>
+          <t>0.9174757281553398, 0.9371980676328503, 0.9230769230769231, 0.9282296650717703, 0.9227053140096618, 0.919047619047619, 0.9375</t>
+        </is>
+      </c>
+      <c r="CP92" t="inlineStr">
+        <is>
+          <t>0.8571428571428571, 0.9017857142857143, 0.8738738738738738, 0.8909090909090909, 0.8660714285714286, 0.8807339449541285, 0.9009009009009009</t>
+        </is>
+      </c>
+      <c r="CQ92" t="n">
+        <v>0.8816311158054277</v>
+      </c>
+      <c r="CR92" t="n">
+        <v>0.8807339449541285</v>
+      </c>
+      <c r="CS92" t="n">
+        <v>0.01588517582355774</v>
+      </c>
+      <c r="CT92" t="n">
+        <v>0.9264619024277377</v>
+      </c>
+      <c r="CU92" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="CV92" t="n">
+        <v>0.007573664841642884</v>
+      </c>
+      <c r="CW92" t="inlineStr">
+        <is>
+          <t>0.9219512195121952, 0.9463414634146341, 0.9320388349514563, 0.941747572815534, 0.9271844660194175, 0.9368932038834952, 0.9466019417475728</t>
+        </is>
+      </c>
+      <c r="CX92" t="inlineStr">
+        <is>
+          <t>0.8495575221238938, 0.8859649122807017, 0.8584070796460177, 0.8672566371681416, 0.8584070796460177, 0.8495575221238938, 0.8849557522123894</t>
+        </is>
+      </c>
+      <c r="CY92" t="n">
+        <v>0.864872357885865</v>
+      </c>
+      <c r="CZ92" t="n">
+        <v>0.8584070796460177</v>
+      </c>
+      <c r="DA92" t="n">
+        <v>0.01417548890837029</v>
+      </c>
+      <c r="DB92" t="n">
+        <v>0.9361083860491864</v>
+      </c>
+      <c r="DC92" t="n">
+        <v>0.9368932038834952</v>
+      </c>
+      <c r="DD92" t="n">
+        <v>0.008814516510296494</v>
+      </c>
+      <c r="DE92" t="inlineStr">
+        <is>
+          <t>0.957500539607166, 0.9679931536157467, 0.9661268150184723, 0.9622605034796803, 0.9604132657444797, 0.9692413437580547, 0.9713678151043904</t>
+        </is>
+      </c>
+      <c r="DF92" t="n">
+        <v>0.9649862051897128</v>
+      </c>
+      <c r="DG92" t="n">
+        <v>0.9661268150184723</v>
+      </c>
+      <c r="DH92" t="n">
+        <v>0.004683562337012314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] Opt SVC no_fragmentation with 2500 iters
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4.xlsx
+++ b/results/metrics_modelling4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH92"/>
+  <dimension ref="A1:DH93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36173,31 +36173,31 @@
       </c>
       <c r="Y92" t="inlineStr">
         <is>
-          <t>0.01703166961669922, 0.01800060272216797, 0.014998435974121094, 0.019999027252197266, 0.016000032424926758, 0.014002799987792969, 0.014002084732055664</t>
+          <t>0.03385305404663086, 0.016930818557739258, 0.015964508056640625, 0.018526554107666016, 0.016786813735961914, 0.014027833938598633, 0.014509916305541992</t>
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>0.01629066467285156</v>
+        <v>0.01865707124982561</v>
       </c>
       <c r="AA92" t="n">
-        <v>0.01600003242492676</v>
+        <v>0.01678681373596191</v>
       </c>
       <c r="AB92" t="n">
-        <v>0.002051172993857287</v>
+        <v>0.006361618933384177</v>
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>0.016968965530395508, 0.02397298812866211, 0.020013093948364258, 0.016998767852783203, 0.016031980514526367, 0.014997720718383789, 0.0149688720703125</t>
+          <t>0.029328107833862305, 0.015465497970581055, 0.015213727951049805, 0.015401363372802734, 0.014502525329589844, 0.016023635864257812, 0.01510477066040039</t>
         </is>
       </c>
       <c r="AD92" t="n">
-        <v>0.01770748410906111</v>
+        <v>0.01729137556893485</v>
       </c>
       <c r="AE92" t="n">
-        <v>0.01696896553039551</v>
+        <v>0.01540136337280273</v>
       </c>
       <c r="AF92" t="n">
-        <v>0.003006426250579327</v>
+        <v>0.004931989007485197</v>
       </c>
       <c r="AG92" t="inlineStr">
         <is>
@@ -36478,6 +36478,396 @@
       </c>
       <c r="DH92" t="n">
         <v>0.004683562337012314</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SVC_no_fragmentation_opt-model</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 5.737910803667096, 'class_weight': None, 'coef0': 0.8535469624679377, 'degree': 2, 'gamma': 'scale'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 5.737910803667096, 'class_weight': None, 'coef0': 0.8535469624679377, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.7368421052631577</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0.9345454545454545</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.8237781954887217</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0.8136363636363636</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0.9272727272727272</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0.9107142857142856</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.9259259259259259</v>
+      </c>
+      <c r="P93" t="n">
+        <v>0.8352941176470589</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0.8987341772151899</v>
+      </c>
+      <c r="R93" t="n">
+        <v>0.8658536585365854</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0.9734641737312739</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0.9073454339194555</v>
+      </c>
+      <c r="U93" t="n">
+        <v>0.9172569968644757</v>
+      </c>
+      <c r="V93" t="n">
+        <v>0.9622641509433962</v>
+      </c>
+      <c r="W93" t="n">
+        <v>0.9357798165137615</v>
+      </c>
+      <c r="X93" t="n">
+        <v>0.9488372093023256</v>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>0.012425422668457031, 0.009999275207519531, 0.010129451751708984, 0.010998725891113281, 0.011511564254760742, 0.011305809020996094, 0.011202335357666016</t>
+        </is>
+      </c>
+      <c r="Z93" t="n">
+        <v>0.01108179773603167</v>
+      </c>
+      <c r="AA93" t="n">
+        <v>0.01120233535766602</v>
+      </c>
+      <c r="AB93" t="n">
+        <v>0.0007690863246816449</v>
+      </c>
+      <c r="AC93" t="inlineStr">
+        <is>
+          <t>0.01711130142211914, 0.014055728912353516, 0.012678384780883789, 0.014551162719726562, 0.015752315521240234, 0.014023542404174805, 0.01426076889038086</t>
+        </is>
+      </c>
+      <c r="AD93" t="n">
+        <v>0.01463331495012556</v>
+      </c>
+      <c r="AE93" t="n">
+        <v>0.01426076889038086</v>
+      </c>
+      <c r="AF93" t="n">
+        <v>0.001312864857834909</v>
+      </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.7735849056603774, 0.9433962264150944, 0.9245283018867925, 0.9056603773584906, 0.9056603773584906, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="AH93" t="inlineStr">
+        <is>
+          <t>0.8948717948717949, 0.7545787545787546, 0.9157509157509157, 0.9487179487179487, 0.8672161172161172, 0.8901098901098901, 0.9258241758241759</t>
+        </is>
+      </c>
+      <c r="AI93" t="n">
+        <v>0.8852956567242282</v>
+      </c>
+      <c r="AJ93" t="n">
+        <v>0.8948717948717949</v>
+      </c>
+      <c r="AK93" t="n">
+        <v>0.05870157980935895</v>
+      </c>
+      <c r="AL93" t="n">
+        <v>0.8978236997104921</v>
+      </c>
+      <c r="AM93" t="n">
+        <v>0.9074074074074074</v>
+      </c>
+      <c r="AN93" t="n">
+        <v>0.05230826099520123</v>
+      </c>
+      <c r="AO93" t="inlineStr">
+        <is>
+          <t>0.8387096774193549, 0.6250000000000001, 0.888888888888889, 0.8750000000000001, 0.8148148148148148, 0.8275862068965518, 0.8666666666666666</t>
+        </is>
+      </c>
+      <c r="AP93" t="inlineStr">
+        <is>
+          <t>0.935064935064935, 0.8378378378378378, 0.9620253164556962, 0.945945945945946, 0.9367088607594937, 0.935064935064935, 0.9473684210526315</t>
+        </is>
+      </c>
+      <c r="AQ93" t="n">
+        <v>0.9285737503116395</v>
+      </c>
+      <c r="AR93" t="n">
+        <v>0.9367088607594937</v>
+      </c>
+      <c r="AS93" t="n">
+        <v>0.0380929256656181</v>
+      </c>
+      <c r="AT93" t="inlineStr">
+        <is>
+          <t>0.886887306242145, 0.731418918918919, 0.9254571026722926, 0.910472972972973, 0.8757618377871542, 0.8813255709807435, 0.9070175438596491</t>
+        </is>
+      </c>
+      <c r="AU93" t="n">
+        <v>0.8740487504905536</v>
+      </c>
+      <c r="AV93" t="n">
+        <v>0.886887306242145</v>
+      </c>
+      <c r="AW93" t="n">
+        <v>0.06049848657632026</v>
+      </c>
+      <c r="AX93" t="n">
+        <v>0.819523750669468</v>
+      </c>
+      <c r="AY93" t="n">
+        <v>0.8387096774193549</v>
+      </c>
+      <c r="AZ93" t="n">
+        <v>0.08315764530247687</v>
+      </c>
+      <c r="BA93" t="inlineStr">
+        <is>
+          <t>0.8125, 0.5555555555555556, 0.9230769230769231, 0.7777777777777778, 0.8461538461538461, 0.8, 0.8125</t>
+        </is>
+      </c>
+      <c r="BB93" t="inlineStr">
+        <is>
+          <t>0.9473684210526315, 0.8857142857142857, 0.95, 1.0, 0.925, 0.9473684210526315, 0.972972972972973</t>
+        </is>
+      </c>
+      <c r="BC93" t="n">
+        <v>0.946917728684646</v>
+      </c>
+      <c r="BD93" t="n">
+        <v>0.9473684210526315</v>
+      </c>
+      <c r="BE93" t="n">
+        <v>0.03323672278137914</v>
+      </c>
+      <c r="BF93" t="n">
+        <v>0.7896520146520147</v>
+      </c>
+      <c r="BG93" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="BH93" t="n">
+        <v>0.1049407686566827</v>
+      </c>
+      <c r="BI93" t="inlineStr">
+        <is>
+          <t>0.8666666666666667, 0.7142857142857143, 0.8571428571428571, 1.0, 0.7857142857142857, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ93" t="inlineStr">
+        <is>
+          <t>0.9230769230769231, 0.7948717948717948, 0.9743589743589743, 0.8974358974358975, 0.9487179487179487, 0.9230769230769231, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="BK93" t="n">
+        <v>0.9120879120879122</v>
+      </c>
+      <c r="BL93" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="BM93" t="n">
+        <v>0.0528285901166885</v>
+      </c>
+      <c r="BN93" t="n">
+        <v>0.8585034013605443</v>
+      </c>
+      <c r="BO93" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP93" t="n">
+        <v>0.08543849378950347</v>
+      </c>
+      <c r="BQ93" t="inlineStr">
+        <is>
+          <t>0.9658119658119659, 0.9175824175824177, 0.9725274725274725, 0.9597069597069597, 0.9597069597069597, 0.9505494505494505, 0.9853479853479854</t>
+        </is>
+      </c>
+      <c r="BR93" t="n">
+        <v>0.9587476016047445</v>
+      </c>
+      <c r="BS93" t="n">
+        <v>0.9597069597069597</v>
+      </c>
+      <c r="BT93" t="n">
+        <v>0.01967955172195972</v>
+      </c>
+      <c r="BU93" t="inlineStr">
+        <is>
+          <t>0.9182389937106918, 0.9310344827586207, 0.9184952978056427, 0.9184952978056427, 0.9184952978056427, 0.9090909090909091, 0.9184952978056427</t>
+        </is>
+      </c>
+      <c r="BV93" t="inlineStr">
+        <is>
+          <t>0.9024725274725275, 0.919281045751634, 0.9182252388134741, 0.9182252388134741, 0.9069884364002011, 0.8968325791855204, 0.9032428355957768</t>
+        </is>
+      </c>
+      <c r="BW93" t="n">
+        <v>0.9093239860046584</v>
+      </c>
+      <c r="BX93" t="n">
+        <v>0.9069884364002011</v>
+      </c>
+      <c r="BY93" t="n">
+        <v>0.008477032436672459</v>
+      </c>
+      <c r="BZ93" t="n">
+        <v>0.9189065109689702</v>
+      </c>
+      <c r="CA93" t="n">
+        <v>0.9184952978056427</v>
+      </c>
+      <c r="CB93" t="n">
+        <v>0.005910713086204811</v>
+      </c>
+      <c r="CC93" t="inlineStr">
+        <is>
+          <t>0.8488372093023256, 0.8735632183908046, 0.8571428571428571, 0.8571428571428571, 0.8522727272727273, 0.8361581920903954, 0.8505747126436781</t>
+        </is>
+      </c>
+      <c r="CD93" t="inlineStr">
+        <is>
+          <t>0.9439655172413793, 0.9525862068965517, 0.9429824561403509, 0.9429824561403509, 0.9437229437229437, 0.9370932754880693, 0.9439655172413793</t>
+        </is>
+      </c>
+      <c r="CE93" t="n">
+        <v>0.9438997675530036</v>
+      </c>
+      <c r="CF93" t="n">
+        <v>0.9437229437229437</v>
+      </c>
+      <c r="CG93" t="n">
+        <v>0.004200431880255032</v>
+      </c>
+      <c r="CH93" t="inlineStr">
+        <is>
+          <t>0.8964013632718525, 0.9130747126436782, 0.900062656641604, 0.900062656641604, 0.8979978354978355, 0.8866257337892324, 0.8972701149425287</t>
+        </is>
+      </c>
+      <c r="CI93" t="n">
+        <v>0.8987850104897622</v>
+      </c>
+      <c r="CJ93" t="n">
+        <v>0.8979978354978355</v>
+      </c>
+      <c r="CK93" t="n">
+        <v>0.00721015834928851</v>
+      </c>
+      <c r="CL93" t="n">
+        <v>0.8536702534265208</v>
+      </c>
+      <c r="CM93" t="n">
+        <v>0.8522727272727273</v>
+      </c>
+      <c r="CN93" t="n">
+        <v>0.01042945052687042</v>
+      </c>
+      <c r="CO93" t="inlineStr">
+        <is>
+          <t>0.8295454545454546, 0.8539325842696629, 0.8041237113402062, 0.8041237113402062, 0.8241758241758241, 0.8043478260869565, 0.8314606741573034</t>
+        </is>
+      </c>
+      <c r="CP93" t="inlineStr">
+        <is>
+          <t>0.9521739130434783, 0.9608695652173913, 0.9684684684684685, 0.9684684684684685, 0.956140350877193, 0.9515418502202643, 0.9521739130434783</t>
+        </is>
+      </c>
+      <c r="CQ93" t="n">
+        <v>0.9585480756198204</v>
+      </c>
+      <c r="CR93" t="n">
+        <v>0.956140350877193</v>
+      </c>
+      <c r="CS93" t="n">
+        <v>0.006952511698038863</v>
+      </c>
+      <c r="CT93" t="n">
+        <v>0.8216728265593732</v>
+      </c>
+      <c r="CU93" t="n">
+        <v>0.8241758241758241</v>
+      </c>
+      <c r="CV93" t="n">
+        <v>0.01740622108788583</v>
+      </c>
+      <c r="CW93" t="inlineStr">
+        <is>
+          <t>0.8690476190476191, 0.8941176470588236, 0.9176470588235294, 0.9176470588235294, 0.8823529411764706, 0.8705882352941177, 0.8705882352941177</t>
+        </is>
+      </c>
+      <c r="CX93" t="inlineStr">
+        <is>
+          <t>0.9358974358974359, 0.9444444444444444, 0.9188034188034188, 0.9188034188034188, 0.9316239316239316, 0.9230769230769231, 0.9358974358974359</t>
+        </is>
+      </c>
+      <c r="CY93" t="n">
+        <v>0.9297924297924298</v>
+      </c>
+      <c r="CZ93" t="n">
+        <v>0.9316239316239316</v>
+      </c>
+      <c r="DA93" t="n">
+        <v>0.009096254228175426</v>
+      </c>
+      <c r="DB93" t="n">
+        <v>0.8888555422168868</v>
+      </c>
+      <c r="DC93" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="DD93" t="n">
+        <v>0.01995573404663581</v>
+      </c>
+      <c r="DE93" t="inlineStr">
+        <is>
+          <t>0.9701872201872203, 0.9768225238813475, 0.9674710910005028, 0.9717948717948718, 0.9693564605329311, 0.9747611865258924, 0.963298139768728</t>
+        </is>
+      </c>
+      <c r="DF93" t="n">
+        <v>0.970527356241642</v>
+      </c>
+      <c r="DG93" t="n">
+        <v>0.9701872201872203</v>
+      </c>
+      <c r="DH93" t="n">
+        <v>0.004179030432633732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] opt-models without ensembles for SMOTE
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4.xlsx
+++ b/results/metrics_modelling4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH93"/>
+  <dimension ref="A1:DH99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36868,6 +36868,2346 @@
       </c>
       <c r="DH93" t="n">
         <v>0.004179030432633732</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LogisticRegression_splashing_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 0.47129737561107793, 'class_weight': None, 'penalty': 'l2'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 0.47129737561107793, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>0.7733333333333333</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.8444444444444444</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.8172043010752689</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0.8865740740740741</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0.7594793435200906</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0.7662037037037037</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0.7017543859649122</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.8383838383838383</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0.796875</v>
+      </c>
+      <c r="R94" t="n">
+        <v>0.8644067796610169</v>
+      </c>
+      <c r="S94" t="n">
+        <v>0.9173859126984127</v>
+      </c>
+      <c r="T94" t="n">
+        <v>0.8322033898305085</v>
+      </c>
+      <c r="U94" t="n">
+        <v>0.8555803571428571</v>
+      </c>
+      <c r="V94" t="n">
+        <v>0.7111111111111111</v>
+      </c>
+      <c r="W94" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="X94" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>0.011999845504760742, 0.011874675750732422, 0.011998891830444336, 0.011457443237304688, 0.010410308837890625, 0.01091313362121582, 0.01103830337524414</t>
+        </is>
+      </c>
+      <c r="Z94" t="n">
+        <v>0.01138465745108468</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>0.01145744323730469</v>
+      </c>
+      <c r="AB94" t="n">
+        <v>0.0005723144748496659</v>
+      </c>
+      <c r="AC94" t="inlineStr">
+        <is>
+          <t>0.017076492309570312, 0.014981508255004883, 0.015033721923828125, 0.015428781509399414, 0.014036893844604492, 0.014475345611572266, 0.015532970428466797</t>
+        </is>
+      </c>
+      <c r="AD94" t="n">
+        <v>0.01522367341177804</v>
+      </c>
+      <c r="AE94" t="n">
+        <v>0.01503372192382812</v>
+      </c>
+      <c r="AF94" t="n">
+        <v>0.000897125378465606</v>
+      </c>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.8113207547169812, 0.8301886792452831, 0.7924528301886793, 0.8113207547169812, 0.7735849056603774, 0.7735849056603774</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.8166666666666667, 0.8560371517027863, 0.8150154798761611, 0.818111455108359, 0.8119195046439629, 0.7654798761609907</t>
+        </is>
+      </c>
+      <c r="AI94" t="n">
+        <v>0.8288610180914471</v>
+      </c>
+      <c r="AJ94" t="n">
+        <v>0.8166666666666667</v>
+      </c>
+      <c r="AK94" t="n">
+        <v>0.04405704094412394</v>
+      </c>
+      <c r="AL94" t="n">
+        <v>0.816911250873515</v>
+      </c>
+      <c r="AM94" t="n">
+        <v>0.8113207547169812</v>
+      </c>
+      <c r="AN94" t="n">
+        <v>0.04851443893604541</v>
+      </c>
+      <c r="AO94" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8484848484848486, 0.8524590163934426, 0.819672131147541, 0.84375, 0.7931034482758621, 0.8181818181818182</t>
+        </is>
+      </c>
+      <c r="AP94" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.7499999999999999, 0.7999999999999999, 0.7555555555555555, 0.761904761904762, 0.75, 0.7</t>
+        </is>
+      </c>
+      <c r="AQ94" t="n">
+        <v>0.7731710227950829</v>
+      </c>
+      <c r="AR94" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="AS94" t="n">
+        <v>0.05652188821857555</v>
+      </c>
+      <c r="AT94" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.7992424242424243, 0.8262295081967213, 0.7876138433515483, 0.8028273809523809, 0.771551724137931, 0.759090909090909</t>
+        </is>
+      </c>
+      <c r="AU94" t="n">
+        <v>0.8093361117790167</v>
+      </c>
+      <c r="AV94" t="n">
+        <v>0.7992424242424243</v>
+      </c>
+      <c r="AW94" t="n">
+        <v>0.04904140326572431</v>
+      </c>
+      <c r="AX94" t="n">
+        <v>0.8455012007629508</v>
+      </c>
+      <c r="AY94" t="n">
+        <v>0.84375</v>
+      </c>
+      <c r="AZ94" t="n">
+        <v>0.04423568934815662</v>
+      </c>
+      <c r="BA94" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.9032258064516129, 0.9629629629629629, 0.9259259259259259, 0.9, 0.9583333333333334, 0.84375</t>
+        </is>
+      </c>
+      <c r="BB94" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.6818181818181818, 0.6923076923076923, 0.6538461538461539, 0.6956521739130435, 0.6206896551724138, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="BC94" t="n">
+        <v>0.7008167665470593</v>
+      </c>
+      <c r="BD94" t="n">
+        <v>0.6818181818181818</v>
+      </c>
+      <c r="BE94" t="n">
+        <v>0.08268515244525924</v>
+      </c>
+      <c r="BF94" t="n">
+        <v>0.9195793102187111</v>
+      </c>
+      <c r="BG94" t="n">
+        <v>0.9259259259259259</v>
+      </c>
+      <c r="BH94" t="n">
+        <v>0.03848380627638249</v>
+      </c>
+      <c r="BI94" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8, 0.7647058823529411, 0.7352941176470589, 0.7941176470588235, 0.6764705882352942, 0.7941176470588235</t>
+        </is>
+      </c>
+      <c r="BJ94" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8333333333333334, 0.9473684210526315, 0.8947368421052632, 0.8421052631578947, 0.9473684210526315, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="BK94" t="n">
+        <v>0.8709273182957393</v>
+      </c>
+      <c r="BL94" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM94" t="n">
+        <v>0.06870551459585363</v>
+      </c>
+      <c r="BN94" t="n">
+        <v>0.7867947178871548</v>
+      </c>
+      <c r="BO94" t="n">
+        <v>0.7941176470588235</v>
+      </c>
+      <c r="BP94" t="n">
+        <v>0.07554445485019097</v>
+      </c>
+      <c r="BQ94" t="inlineStr">
+        <is>
+          <t>0.962406015037594, 0.8650793650793651, 0.9473684210526316, 0.8684210526315789, 0.9380804953560372, 0.8359133126934984, 0.8668730650154799</t>
+        </is>
+      </c>
+      <c r="BR94" t="n">
+        <v>0.897734532409455</v>
+      </c>
+      <c r="BS94" t="n">
+        <v>0.8684210526315789</v>
+      </c>
+      <c r="BT94" t="n">
+        <v>0.04625033392956519</v>
+      </c>
+      <c r="BU94" t="inlineStr">
+        <is>
+          <t>0.8144654088050315, 0.8244514106583072, 0.8181818181818182, 0.8213166144200627, 0.8213166144200627, 0.8213166144200627, 0.8432601880877743</t>
+        </is>
+      </c>
+      <c r="BV94" t="inlineStr">
+        <is>
+          <t>0.8322685085257933, 0.8419982884039368, 0.8352521694303634, 0.8356817596013404, 0.8336841653062979, 0.8376793538963828, 0.8466792679783486</t>
+        </is>
+      </c>
+      <c r="BW94" t="n">
+        <v>0.8376062161632091</v>
+      </c>
+      <c r="BX94" t="n">
+        <v>0.8356817596013404</v>
+      </c>
+      <c r="BY94" t="n">
+        <v>0.004701589271750212</v>
+      </c>
+      <c r="BZ94" t="n">
+        <v>0.823472666999017</v>
+      </c>
+      <c r="CA94" t="n">
+        <v>0.8213166144200627</v>
+      </c>
+      <c r="CB94" t="n">
+        <v>0.008582152573283645</v>
+      </c>
+      <c r="CC94" t="inlineStr">
+        <is>
+          <t>0.8426666666666668, 0.8510638297872339, 0.8465608465608466, 0.8503937007874015, 0.8511749347258485, 0.8496042216358839, 0.8730964467005077</t>
+        </is>
+      </c>
+      <c r="CD94" t="inlineStr">
+        <is>
+          <t>0.7739463601532568, 0.7862595419847328, 0.7769230769230768, 0.7782101167315174, 0.776470588235294, 0.7799227799227799, 0.7950819672131147</t>
+        </is>
+      </c>
+      <c r="CE94" t="n">
+        <v>0.7809734901662532</v>
+      </c>
+      <c r="CF94" t="n">
+        <v>0.7782101167315174</v>
+      </c>
+      <c r="CG94" t="n">
+        <v>0.00678016247829866</v>
+      </c>
+      <c r="CH94" t="inlineStr">
+        <is>
+          <t>0.8083065134099618, 0.8186616858859834, 0.8117419617419617, 0.8143019087594594, 0.8138227614805713, 0.8147635007793319, 0.8340892069568112</t>
+        </is>
+      </c>
+      <c r="CI94" t="n">
+        <v>0.8165267912877258</v>
+      </c>
+      <c r="CJ94" t="n">
+        <v>0.8143019087594594</v>
+      </c>
+      <c r="CK94" t="n">
+        <v>0.007735214967265304</v>
+      </c>
+      <c r="CL94" t="n">
+        <v>0.8520800924091985</v>
+      </c>
+      <c r="CM94" t="n">
+        <v>0.8503937007874015</v>
+      </c>
+      <c r="CN94" t="n">
+        <v>0.009036337434249156</v>
+      </c>
+      <c r="CO94" t="inlineStr">
+        <is>
+          <t>0.9294117647058824, 0.935672514619883, 0.9302325581395349, 0.9257142857142857, 0.9209039548022598, 0.930635838150289, 0.9148936170212766</t>
+        </is>
+      </c>
+      <c r="CP94" t="inlineStr">
+        <is>
+          <t>0.6824324324324325, 0.6959459459459459, 0.6870748299319728, 0.6944444444444444, 0.6971830985915493, 0.6917808219178082, 0.7404580152671756</t>
+        </is>
+      </c>
+      <c r="CQ94" t="n">
+        <v>0.6984742269330468</v>
+      </c>
+      <c r="CR94" t="n">
+        <v>0.6944444444444444</v>
+      </c>
+      <c r="CS94" t="n">
+        <v>0.01780458985936085</v>
+      </c>
+      <c r="CT94" t="n">
+        <v>0.9267806475933446</v>
+      </c>
+      <c r="CU94" t="n">
+        <v>0.9294117647058824</v>
+      </c>
+      <c r="CV94" t="n">
+        <v>0.006433621494772158</v>
+      </c>
+      <c r="CW94" t="inlineStr">
+        <is>
+          <t>0.7707317073170732, 0.7804878048780488, 0.7766990291262136, 0.7864077669902912, 0.7912621359223301, 0.7815533980582524, 0.8349514563106796</t>
+        </is>
+      </c>
+      <c r="CX94" t="inlineStr">
+        <is>
+          <t>0.8938053097345132, 0.9035087719298246, 0.8938053097345132, 0.8849557522123894, 0.8761061946902655, 0.8938053097345132, 0.8584070796460177</t>
+        </is>
+      </c>
+      <c r="CY94" t="n">
+        <v>0.8863419610974338</v>
+      </c>
+      <c r="CZ94" t="n">
+        <v>0.8938053097345132</v>
+      </c>
+      <c r="DA94" t="n">
+        <v>0.01388140690435868</v>
+      </c>
+      <c r="DB94" t="n">
+        <v>0.7888704712289841</v>
+      </c>
+      <c r="DC94" t="n">
+        <v>0.7815533980582524</v>
+      </c>
+      <c r="DD94" t="n">
+        <v>0.01977086446669224</v>
+      </c>
+      <c r="DE94" t="inlineStr">
+        <is>
+          <t>0.9009497086121303, 0.9152332049636286, 0.9052109287739497, 0.9146619125354412, 0.9054686828765358, 0.9215138757625225, 0.9120843715095799</t>
+        </is>
+      </c>
+      <c r="DF94" t="n">
+        <v>0.9107318121476841</v>
+      </c>
+      <c r="DG94" t="n">
+        <v>0.9120843715095799</v>
+      </c>
+      <c r="DH94" t="n">
+        <v>0.006629595672810654</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>LogisticRegression_no_fragmentation_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'newton-cholesky', 'C': 6.5706235157060515, 'class_weight': 'balanced', 'penalty': 'l2'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'newton-cholesky', 'C': 6.5706235157060515, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0.6206896551724138</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.7346938775510204</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0.9509090909090909</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0.8029905031319459</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0.9565217391304348</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0.8712871287128713</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.8316498316498316</v>
+      </c>
+      <c r="P95" t="n">
+        <v>0.6260869565217392</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0.9113924050632911</v>
+      </c>
+      <c r="R95" t="n">
+        <v>0.7422680412371135</v>
+      </c>
+      <c r="S95" t="n">
+        <v>0.9458831726860992</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0.8086340206185567</v>
+      </c>
+      <c r="U95" t="n">
+        <v>0.8570723493206364</v>
+      </c>
+      <c r="V95" t="n">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="W95" t="n">
+        <v>0.8027522935779816</v>
+      </c>
+      <c r="X95" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>0.009731769561767578, 0.010012388229370117, 0.009104728698730469, 0.009039163589477539, 0.010002613067626953, 0.008647680282592773, 0.008929014205932617</t>
+        </is>
+      </c>
+      <c r="Z95" t="n">
+        <v>0.009352479662214006</v>
+      </c>
+      <c r="AA95" t="n">
+        <v>0.009104728698730469</v>
+      </c>
+      <c r="AB95" t="n">
+        <v>0.0005123651389478475</v>
+      </c>
+      <c r="AC95" t="inlineStr">
+        <is>
+          <t>0.01586008071899414, 0.01587843894958496, 0.014185667037963867, 0.013430356979370117, 0.013245820999145508, 0.013036012649536133, 0.01393437385559082</t>
+        </is>
+      </c>
+      <c r="AD95" t="n">
+        <v>0.01422439302716936</v>
+      </c>
+      <c r="AE95" t="n">
+        <v>0.01393437385559082</v>
+      </c>
+      <c r="AF95" t="n">
+        <v>0.001101771128809612</v>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7169811320754716, 0.8490566037735849, 0.8113207547169812, 0.8301886792452831, 0.8679245283018868, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr">
+        <is>
+          <t>0.9025641025641026, 0.7161172161172161, 0.8745421245421245, 0.848901098901099, 0.8617216117216118, 0.8644688644688645, 0.9102564102564102</t>
+        </is>
+      </c>
+      <c r="AI95" t="n">
+        <v>0.8540816326530614</v>
+      </c>
+      <c r="AJ95" t="n">
+        <v>0.8644688644688645</v>
+      </c>
+      <c r="AK95" t="n">
+        <v>0.05994291246177208</v>
+      </c>
+      <c r="AL95" t="n">
+        <v>0.8331835879005691</v>
+      </c>
+      <c r="AM95" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="AN95" t="n">
+        <v>0.05312903801593512</v>
+      </c>
+      <c r="AO95" t="inlineStr">
+        <is>
+          <t>0.8235294117647058, 0.5714285714285714, 0.7647058823529412, 0.7222222222222223, 0.742857142857143, 0.7741935483870968, 0.8</t>
+        </is>
+      </c>
+      <c r="AP95" t="inlineStr">
+        <is>
+          <t>0.9189189189189189, 0.7887323943661971, 0.8888888888888888, 0.8571428571428572, 0.8732394366197183, 0.9066666666666667, 0.9014084507042254</t>
+        </is>
+      </c>
+      <c r="AQ95" t="n">
+        <v>0.876428230472496</v>
+      </c>
+      <c r="AR95" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="AS95" t="n">
+        <v>0.04065842864681587</v>
+      </c>
+      <c r="AT95" t="inlineStr">
+        <is>
+          <t>0.8712241653418124, 0.6800804828973843, 0.826797385620915, 0.7896825396825398, 0.8080482897384307, 0.8404301075268817, 0.8507042253521127</t>
+        </is>
+      </c>
+      <c r="AU95" t="n">
+        <v>0.8095667423085823</v>
+      </c>
+      <c r="AV95" t="n">
+        <v>0.826797385620915</v>
+      </c>
+      <c r="AW95" t="n">
+        <v>0.05844136413827328</v>
+      </c>
+      <c r="AX95" t="n">
+        <v>0.7427052541446686</v>
+      </c>
+      <c r="AY95" t="n">
+        <v>0.7647058823529412</v>
+      </c>
+      <c r="AZ95" t="n">
+        <v>0.0765749421739622</v>
+      </c>
+      <c r="BA95" t="inlineStr">
+        <is>
+          <t>0.7368421052631579, 0.47619047619047616, 0.65, 0.5909090909090909, 0.6190476190476191, 0.7058823529411765, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="BB95" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.875, 0.9696969696969697, 0.967741935483871, 0.96875, 0.9444444444444444, 1.0</t>
+        </is>
+      </c>
+      <c r="BC95" t="n">
+        <v>0.9567231315791224</v>
+      </c>
+      <c r="BD95" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="BE95" t="n">
+        <v>0.03655319758017286</v>
+      </c>
+      <c r="BF95" t="n">
+        <v>0.6350769015740267</v>
+      </c>
+      <c r="BG95" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="BH95" t="n">
+        <v>0.07932105676016318</v>
+      </c>
+      <c r="BI95" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.7142857142857143, 0.9285714285714286, 0.9285714285714286, 0.9285714285714286, 0.8571428571428571, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ95" t="inlineStr">
+        <is>
+          <t>0.8717948717948718, 0.717948717948718, 0.8205128205128205, 0.7692307692307693, 0.7948717948717948, 0.8717948717948718, 0.8205128205128205</t>
+        </is>
+      </c>
+      <c r="BK95" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="BL95" t="n">
+        <v>0.8205128205128205</v>
+      </c>
+      <c r="BM95" t="n">
+        <v>0.05101973727906271</v>
+      </c>
+      <c r="BN95" t="n">
+        <v>0.8986394557823129</v>
+      </c>
+      <c r="BO95" t="n">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="BP95" t="n">
+        <v>0.08440858432242775</v>
+      </c>
+      <c r="BQ95" t="inlineStr">
+        <is>
+          <t>0.9555555555555555, 0.8974358974358975, 0.9706959706959708, 0.9395604395604396, 0.9212454212454213, 0.9432234432234432, 1.0</t>
+        </is>
+      </c>
+      <c r="BR95" t="n">
+        <v>0.946816675388104</v>
+      </c>
+      <c r="BS95" t="n">
+        <v>0.9432234432234432</v>
+      </c>
+      <c r="BT95" t="n">
+        <v>0.03078257701345802</v>
+      </c>
+      <c r="BU95" t="inlineStr">
+        <is>
+          <t>0.8207547169811321, 0.8495297805642633, 0.8307210031347962, 0.8432601880877743, 0.8526645768025078, 0.8307210031347962, 0.8307210031347962</t>
+        </is>
+      </c>
+      <c r="BV95" t="inlineStr">
+        <is>
+          <t>0.8438644688644689, 0.8712166918049271, 0.85465057817999, 0.8631975867269985, 0.8621166415284063, 0.85465057817999, 0.8509049773755657</t>
+        </is>
+      </c>
+      <c r="BW95" t="n">
+        <v>0.8572287889514781</v>
+      </c>
+      <c r="BX95" t="n">
+        <v>0.85465057817999</v>
+      </c>
+      <c r="BY95" t="n">
+        <v>0.008341540297438091</v>
+      </c>
+      <c r="BZ95" t="n">
+        <v>0.8369103245485808</v>
+      </c>
+      <c r="CA95" t="n">
+        <v>0.8307210031347962</v>
+      </c>
+      <c r="CB95" t="n">
+        <v>0.01084761103219961</v>
+      </c>
+      <c r="CC95" t="inlineStr">
+        <is>
+          <t>0.7246376811594203, 0.7647058823529411, 0.7403846153846153, 0.7549019607843137, 0.7614213197969542, 0.7403846153846153, 0.7378640776699029</t>
+        </is>
+      </c>
+      <c r="CD95" t="inlineStr">
+        <is>
+          <t>0.8671328671328672, 0.8894009216589861, 0.8744186046511628, 0.8847926267281105, 0.8934240362811792, 0.8744186046511628, 0.875</t>
+        </is>
+      </c>
+      <c r="CE95" t="n">
+        <v>0.8797982373004957</v>
+      </c>
+      <c r="CF95" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="CG95" t="n">
+        <v>0.008816651843155495</v>
+      </c>
+      <c r="CH95" t="inlineStr">
+        <is>
+          <t>0.7958852741461437, 0.8270534020059637, 0.8074016100178891, 0.8198472937562121, 0.8274226780390667, 0.8074016100178891, 0.8064320388349515</t>
+        </is>
+      </c>
+      <c r="CI95" t="n">
+        <v>0.8130634152597308</v>
+      </c>
+      <c r="CJ95" t="n">
+        <v>0.8074016100178891</v>
+      </c>
+      <c r="CK95" t="n">
+        <v>0.01102662315087141</v>
+      </c>
+      <c r="CL95" t="n">
+        <v>0.7463285932189662</v>
+      </c>
+      <c r="CM95" t="n">
+        <v>0.7403846153846153</v>
+      </c>
+      <c r="CN95" t="n">
+        <v>0.01337280405112217</v>
+      </c>
+      <c r="CO95" t="inlineStr">
+        <is>
+          <t>0.6097560975609756, 0.6554621848739496, 0.6260162601626016, 0.6470588235294118, 0.6696428571428571, 0.6260162601626016, 0.628099173553719</t>
+        </is>
+      </c>
+      <c r="CP95" t="inlineStr">
+        <is>
+          <t>0.9538461538461539, 0.965, 0.9591836734693877, 0.96, 0.9516908212560387, 0.9591836734693877, 0.9545454545454546</t>
+        </is>
+      </c>
+      <c r="CQ95" t="n">
+        <v>0.9576356823694889</v>
+      </c>
+      <c r="CR95" t="n">
+        <v>0.9591836734693877</v>
+      </c>
+      <c r="CS95" t="n">
+        <v>0.004206578742255173</v>
+      </c>
+      <c r="CT95" t="n">
+        <v>0.6374359509980165</v>
+      </c>
+      <c r="CU95" t="n">
+        <v>0.628099173553719</v>
+      </c>
+      <c r="CV95" t="n">
+        <v>0.01915723646869028</v>
+      </c>
+      <c r="CW95" t="inlineStr">
+        <is>
+          <t>0.8928571428571429, 0.9176470588235294, 0.9058823529411765, 0.9058823529411765, 0.8823529411764706, 0.9058823529411765, 0.8941176470588236</t>
+        </is>
+      </c>
+      <c r="CX95" t="inlineStr">
+        <is>
+          <t>0.7948717948717948, 0.8247863247863247, 0.8034188034188035, 0.8205128205128205, 0.8418803418803419, 0.8034188034188035, 0.8076923076923077</t>
+        </is>
+      </c>
+      <c r="CY95" t="n">
+        <v>0.8137973137973137</v>
+      </c>
+      <c r="CZ95" t="n">
+        <v>0.8076923076923077</v>
+      </c>
+      <c r="DA95" t="n">
+        <v>0.01495414983384113</v>
+      </c>
+      <c r="DB95" t="n">
+        <v>0.9006602641056424</v>
+      </c>
+      <c r="DC95" t="n">
+        <v>0.9058823529411765</v>
+      </c>
+      <c r="DD95" t="n">
+        <v>0.01075183998923873</v>
+      </c>
+      <c r="DE95" t="inlineStr">
+        <is>
+          <t>0.9463268213268213, 0.9540975364504777, 0.9437405731523378, 0.9492709904474611, 0.9479135243841126, 0.9507792860734038, 0.9380593262946205</t>
+        </is>
+      </c>
+      <c r="DF95" t="n">
+        <v>0.9471697225898907</v>
+      </c>
+      <c r="DG95" t="n">
+        <v>0.9479135243841126</v>
+      </c>
+      <c r="DH95" t="n">
+        <v>0.004802692551476039</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_splashing_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 2, 'weights': 'distance', 'p': 1}, 'base_estimator_params': {'n_neighbors': 2, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.8910891089108911</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0.8800154320987654</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0.8332996564962618</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0.8206018518518519</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0.8636363636363636</v>
+      </c>
+      <c r="M96" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0.7755102040816326</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P96" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0.9947916666666666</v>
+      </c>
+      <c r="R96" t="n">
+        <v>0.9973890339425587</v>
+      </c>
+      <c r="S96" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0.996324848724834</v>
+      </c>
+      <c r="U96" t="n">
+        <v>0.9973958333333333</v>
+      </c>
+      <c r="V96" t="n">
+        <v>0.9905660377358491</v>
+      </c>
+      <c r="W96" t="n">
+        <v>1</v>
+      </c>
+      <c r="X96" t="n">
+        <v>0.9952606635071091</v>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>0.011987924575805664, 0.009905338287353516, 0.008966207504272461, 0.009542465209960938, 0.009782791137695312, 0.009510040283203125, 0.009002685546875</t>
+        </is>
+      </c>
+      <c r="Z96" t="n">
+        <v>0.009813921792166573</v>
+      </c>
+      <c r="AA96" t="n">
+        <v>0.009542465209960938</v>
+      </c>
+      <c r="AB96" t="n">
+        <v>0.0009470533703167229</v>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>0.019345521926879883, 0.016130924224853516, 0.01617574691772461, 0.015309572219848633, 0.0145721435546875, 0.015524625778198242, 0.014997482299804688</t>
+        </is>
+      </c>
+      <c r="AD96" t="n">
+        <v>0.01600800241742815</v>
+      </c>
+      <c r="AE96" t="n">
+        <v>0.01552462577819824</v>
+      </c>
+      <c r="AF96" t="n">
+        <v>0.001463195317602059</v>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.8113207547169812, 0.8867924528301887, 0.9245283018867925, 0.9056603773584906, 0.9056603773584906, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8166666666666667, 0.8769349845201238, 0.9295665634674922, 0.891640866873065, 0.914860681114551, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AI96" t="n">
+        <v>0.885905941323898</v>
+      </c>
+      <c r="AJ96" t="n">
+        <v>0.891640866873065</v>
+      </c>
+      <c r="AK96" t="n">
+        <v>0.03340345223601217</v>
+      </c>
+      <c r="AL96" t="n">
+        <v>0.8923829489867227</v>
+      </c>
+      <c r="AM96" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="AN96" t="n">
+        <v>0.03614380377193017</v>
+      </c>
+      <c r="AO96" t="inlineStr">
+        <is>
+          <t>0.945945945945946, 0.8484848484848486, 0.9117647058823528, 0.9393939393939394, 0.9275362318840579, 0.923076923076923, 0.9117647058823528</t>
+        </is>
+      </c>
+      <c r="AP96" t="inlineStr">
+        <is>
+          <t>0.8823529411764706, 0.7499999999999999, 0.8421052631578947, 0.9, 0.8648648648648649, 0.8780487804878049, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="AQ96" t="n">
+        <v>0.8513538732635614</v>
+      </c>
+      <c r="AR96" t="n">
+        <v>0.8648648648648649</v>
+      </c>
+      <c r="AS96" t="n">
+        <v>0.04577309569572132</v>
+      </c>
+      <c r="AT96" t="inlineStr">
+        <is>
+          <t>0.9141494435612083, 0.7992424242424243, 0.8769349845201238, 0.9196969696969697, 0.8962005483744614, 0.900562851782364, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AU96" t="n">
+        <v>0.8833888866710965</v>
+      </c>
+      <c r="AV96" t="n">
+        <v>0.8962005483744614</v>
+      </c>
+      <c r="AW96" t="n">
+        <v>0.03758325111698525</v>
+      </c>
+      <c r="AX96" t="n">
+        <v>0.9154239000786316</v>
+      </c>
+      <c r="AY96" t="n">
+        <v>0.923076923076923</v>
+      </c>
+      <c r="AZ96" t="n">
+        <v>0.02980664222256574</v>
+      </c>
+      <c r="BA96" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.9032258064516129, 0.9117647058823529, 0.96875, 0.9142857142857143, 0.967741935483871, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BB96" t="inlineStr">
+        <is>
+          <t>1.0, 0.6818181818181818, 0.8421052631578947, 0.8571428571428571, 0.8888888888888888, 0.8181818181818182, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BC96" t="n">
+        <v>0.8471774674782193</v>
+      </c>
+      <c r="BD96" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BE96" t="n">
+        <v>0.08736603921685659</v>
+      </c>
+      <c r="BF96" t="n">
+        <v>0.9249955379174003</v>
+      </c>
+      <c r="BG96" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BH96" t="n">
+        <v>0.02787721190074099</v>
+      </c>
+      <c r="BI96" t="inlineStr">
+        <is>
+          <t>1.0, 0.8, 0.9117647058823529, 0.9117647058823529, 0.9411764705882353, 0.8823529411764706, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BJ96" t="inlineStr">
+        <is>
+          <t>0.7894736842105263, 0.8333333333333334, 0.8421052631578947, 0.9473684210526315, 0.8421052631578947, 0.9473684210526315, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BK96" t="n">
+        <v>0.8634085213032582</v>
+      </c>
+      <c r="BL96" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BM96" t="n">
+        <v>0.05584531317082</v>
+      </c>
+      <c r="BN96" t="n">
+        <v>0.9084033613445379</v>
+      </c>
+      <c r="BO96" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BP96" t="n">
+        <v>0.0559691623709133</v>
+      </c>
+      <c r="BQ96" t="inlineStr">
+        <is>
+          <t>0.9165413533834588, 0.8603174603174604, 0.9489164086687306, 0.9613003095975232, 0.8893188854489165, 0.9458204334365325, 0.9109907120743034</t>
+        </is>
+      </c>
+      <c r="BR96" t="n">
+        <v>0.9190293661324179</v>
+      </c>
+      <c r="BS96" t="n">
+        <v>0.9165413533834588</v>
+      </c>
+      <c r="BT96" t="n">
+        <v>0.03337758010073159</v>
+      </c>
+      <c r="BU96" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV96" t="inlineStr">
+        <is>
+          <t>0.9975609756097561, 1.0, 0.9975728155339806, 0.9975728155339806, 0.9975728155339806, 1.0, 0.9975728155339806</t>
+        </is>
+      </c>
+      <c r="BW96" t="n">
+        <v>0.9982646053922398</v>
+      </c>
+      <c r="BX96" t="n">
+        <v>0.9975728155339806</v>
+      </c>
+      <c r="BY96" t="n">
+        <v>0.001097567218380571</v>
+      </c>
+      <c r="BZ96" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA96" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB96" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC96" t="inlineStr">
+        <is>
+          <t>0.9975550122249389, 1.0, 0.9975669099756691, 0.9975669099756691, 0.9975669099756691, 1.0, 0.9975669099756691</t>
+        </is>
+      </c>
+      <c r="CD96" t="inlineStr">
+        <is>
+          <t>0.9955947136563876, 1.0, 0.9955947136563876, 0.9955947136563876, 0.9955947136563876, 1.0, 0.9955947136563876</t>
+        </is>
+      </c>
+      <c r="CE96" t="n">
+        <v>0.9968533668974198</v>
+      </c>
+      <c r="CF96" t="n">
+        <v>0.9955947136563876</v>
+      </c>
+      <c r="CG96" t="n">
+        <v>0.001990105513007176</v>
+      </c>
+      <c r="CH96" t="inlineStr">
+        <is>
+          <t>0.9965748629406632, 1.0, 0.9965808118160284, 0.9965808118160284, 0.9965808118160284, 1.0, 0.9965808118160284</t>
+        </is>
+      </c>
+      <c r="CI96" t="n">
+        <v>0.9975568728863966</v>
+      </c>
+      <c r="CJ96" t="n">
+        <v>0.9965808118160284</v>
+      </c>
+      <c r="CK96" t="n">
+        <v>0.001545170567206118</v>
+      </c>
+      <c r="CL96" t="n">
+        <v>0.9982603788753737</v>
+      </c>
+      <c r="CM96" t="n">
+        <v>0.9975669099756691</v>
+      </c>
+      <c r="CN96" t="n">
+        <v>0.001100240355913701</v>
+      </c>
+      <c r="CO96" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP96" t="inlineStr">
+        <is>
+          <t>0.9912280701754386, 1.0, 0.9912280701754386, 0.9912280701754386, 0.9912280701754386, 1.0, 0.9912280701754386</t>
+        </is>
+      </c>
+      <c r="CQ96" t="n">
+        <v>0.9937343358395989</v>
+      </c>
+      <c r="CR96" t="n">
+        <v>0.9912280701754386</v>
+      </c>
+      <c r="CS96" t="n">
+        <v>0.003962753960110763</v>
+      </c>
+      <c r="CT96" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU96" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV96" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW96" t="inlineStr">
+        <is>
+          <t>0.9951219512195122, 1.0, 0.9951456310679612, 0.9951456310679612, 0.9951456310679612, 1.0, 0.9951456310679612</t>
+        </is>
+      </c>
+      <c r="CX96" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY96" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ96" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA96" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB96" t="n">
+        <v>0.9965292107844796</v>
+      </c>
+      <c r="DC96" t="n">
+        <v>0.9951456310679612</v>
+      </c>
+      <c r="DD96" t="n">
+        <v>0.002195134436761142</v>
+      </c>
+      <c r="DE96" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 1.0, 0.9999785204914512, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914512</t>
+        </is>
+      </c>
+      <c r="DF96" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="DG96" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="DH96" t="n">
+        <v>9.712984233443666e-06</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_no_fragmentation_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'base_estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.7391304347826088</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0.9031818181818182</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0.8118729096989967</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0.8431818181818181</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.9387755102040817</v>
+      </c>
+      <c r="M97" t="n">
+        <v>0.8363636363636363</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0.8846153846153846</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0.9427609427609428</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0.8369565217391305</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0.9746835443037974</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0.9005847953216375</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0.9932934618511207</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0.9301978350130646</v>
+      </c>
+      <c r="U97" t="n">
+        <v>0.9529381024271281</v>
+      </c>
+      <c r="V97" t="n">
+        <v>0.9902439024390244</v>
+      </c>
+      <c r="W97" t="n">
+        <v>0.9311926605504587</v>
+      </c>
+      <c r="X97" t="n">
+        <v>0.9598108747044918</v>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>0.010000467300415039, 0.008997917175292969, 0.008598804473876953, 0.007999181747436523, 0.009029865264892578, 0.007953166961669922, 0.0070002079010009766</t>
+        </is>
+      </c>
+      <c r="Z97" t="n">
+        <v>0.008511372974940709</v>
+      </c>
+      <c r="AA97" t="n">
+        <v>0.008598804473876953</v>
+      </c>
+      <c r="AB97" t="n">
+        <v>0.0008934811036678975</v>
+      </c>
+      <c r="AC97" t="inlineStr">
+        <is>
+          <t>0.019122600555419922, 0.016436338424682617, 0.01525115966796875, 0.016414403915405273, 0.015381813049316406, 0.016277074813842773, 0.016347169876098633</t>
+        </is>
+      </c>
+      <c r="AD97" t="n">
+        <v>0.01646150861467634</v>
+      </c>
+      <c r="AE97" t="n">
+        <v>0.01634716987609863</v>
+      </c>
+      <c r="AF97" t="n">
+        <v>0.00118092209546679</v>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>0.8518518518518519, 0.7358490566037735, 0.9245283018867925, 0.8867924528301887, 0.9056603773584906, 0.9056603773584906, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr">
+        <is>
+          <t>0.8564102564102565, 0.728937728937729, 0.9029304029304028, 0.9001831501831502, 0.8672161172161172, 0.8901098901098901, 0.8873626373626373</t>
+        </is>
+      </c>
+      <c r="AI97" t="n">
+        <v>0.8618785975928832</v>
+      </c>
+      <c r="AJ97" t="n">
+        <v>0.8873626373626373</v>
+      </c>
+      <c r="AK97" t="n">
+        <v>0.05648084132895018</v>
+      </c>
+      <c r="AL97" t="n">
+        <v>0.868323849455925</v>
+      </c>
+      <c r="AM97" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN97" t="n">
+        <v>0.05868696535610506</v>
+      </c>
+      <c r="AO97" t="inlineStr">
+        <is>
+          <t>0.7647058823529413, 0.588235294117647, 0.8571428571428571, 0.8125000000000001, 0.8148148148148148, 0.8275862068965518, 0.7878787878787878</t>
+        </is>
+      </c>
+      <c r="AP97" t="inlineStr">
+        <is>
+          <t>0.8918918918918919, 0.8055555555555556, 0.9487179487179487, 0.9189189189189189, 0.9367088607594937, 0.935064935064935, 0.9041095890410958</t>
+        </is>
+      </c>
+      <c r="AQ97" t="n">
+        <v>0.9058525285642629</v>
+      </c>
+      <c r="AR97" t="n">
+        <v>0.9189189189189189</v>
+      </c>
+      <c r="AS97" t="n">
+        <v>0.04483473261585094</v>
+      </c>
+      <c r="AT97" t="inlineStr">
+        <is>
+          <t>0.8282988871224166, 0.6968954248366013, 0.9029304029304028, 0.8657094594594594, 0.8757618377871542, 0.8813255709807435, 0.8459941884599418</t>
+        </is>
+      </c>
+      <c r="AU97" t="n">
+        <v>0.8424165387966743</v>
+      </c>
+      <c r="AV97" t="n">
+        <v>0.8657094594594594</v>
+      </c>
+      <c r="AW97" t="n">
+        <v>0.06349219516686723</v>
+      </c>
+      <c r="AX97" t="n">
+        <v>0.7789805490290858</v>
+      </c>
+      <c r="AY97" t="n">
+        <v>0.8125000000000001</v>
+      </c>
+      <c r="AZ97" t="n">
+        <v>0.08241549925206183</v>
+      </c>
+      <c r="BA97" t="inlineStr">
+        <is>
+          <t>0.6842105263157895, 0.5, 0.8571428571428571, 0.7222222222222222, 0.8461538461538461, 0.8, 0.6842105263157895</t>
+        </is>
+      </c>
+      <c r="BB97" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8787878787878788, 0.9487179487179487, 0.9714285714285714, 0.925, 0.9473684210526315, 0.9705882352941176</t>
+        </is>
+      </c>
+      <c r="BC97" t="n">
+        <v>0.9406783140197559</v>
+      </c>
+      <c r="BD97" t="n">
+        <v>0.9473684210526315</v>
+      </c>
+      <c r="BE97" t="n">
+        <v>0.02935146085031867</v>
+      </c>
+      <c r="BF97" t="n">
+        <v>0.7277057111643578</v>
+      </c>
+      <c r="BG97" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="BH97" t="n">
+        <v>0.1144390176954305</v>
+      </c>
+      <c r="BI97" t="inlineStr">
+        <is>
+          <t>0.8666666666666667, 0.7142857142857143, 0.8571428571428571, 0.9285714285714286, 0.7857142857142857, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ97" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.7435897435897436, 0.9487179487179487, 0.8717948717948718, 0.9487179487179487, 0.9230769230769231, 0.8461538461538461</t>
+        </is>
+      </c>
+      <c r="BK97" t="n">
+        <v>0.8754578754578753</v>
+      </c>
+      <c r="BL97" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="BM97" t="n">
+        <v>0.0677408132194393</v>
+      </c>
+      <c r="BN97" t="n">
+        <v>0.8482993197278912</v>
+      </c>
+      <c r="BO97" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP97" t="n">
+        <v>0.07097034751425839</v>
+      </c>
+      <c r="BQ97" t="inlineStr">
+        <is>
+          <t>0.9128205128205128, 0.7884615384615384, 0.934981684981685, 0.9532967032967032, 0.9597069597069597, 0.8965201465201466, 0.9267399267399267</t>
+        </is>
+      </c>
+      <c r="BR97" t="n">
+        <v>0.9103610675039248</v>
+      </c>
+      <c r="BS97" t="n">
+        <v>0.9267399267399267</v>
+      </c>
+      <c r="BT97" t="n">
+        <v>0.0537321968905618</v>
+      </c>
+      <c r="BU97" t="inlineStr">
+        <is>
+          <t>0.949685534591195, 0.9435736677115988, 0.9435736677115988, 0.9404388714733543, 0.9373040752351097, 0.9498432601880877, 0.9529780564263323</t>
+        </is>
+      </c>
+      <c r="BV97" t="inlineStr">
+        <is>
+          <t>0.9543650793650793, 0.9465560583207642, 0.9503016591251885, 0.944419306184012, 0.9385369532428356, 0.9620663650075415, 0.9567119155354449</t>
+        </is>
+      </c>
+      <c r="BW97" t="n">
+        <v>0.950422476682981</v>
+      </c>
+      <c r="BX97" t="n">
+        <v>0.9503016591251885</v>
+      </c>
+      <c r="BY97" t="n">
+        <v>0.007396416155549377</v>
+      </c>
+      <c r="BZ97" t="n">
+        <v>0.9453424476196108</v>
+      </c>
+      <c r="CA97" t="n">
+        <v>0.9435736677115988</v>
+      </c>
+      <c r="CB97" t="n">
+        <v>0.005241863005903344</v>
+      </c>
+      <c r="CC97" t="inlineStr">
+        <is>
+          <t>0.9101123595505619, 0.9, 0.9010989010989011, 0.8950276243093922, 0.8888888888888888, 0.9130434782608696, 0.9162011173184357</t>
+        </is>
+      </c>
+      <c r="CD97" t="inlineStr">
+        <is>
+          <t>0.9650655021834061, 0.9606986899563319, 0.9605263157894737, 0.9584245076586433, 0.9563318777292577, 0.9647577092511014, 0.9673202614379085</t>
+        </is>
+      </c>
+      <c r="CE97" t="n">
+        <v>0.9618749805723031</v>
+      </c>
+      <c r="CF97" t="n">
+        <v>0.9606986899563319</v>
+      </c>
+      <c r="CG97" t="n">
+        <v>0.003664013124936622</v>
+      </c>
+      <c r="CH97" t="inlineStr">
+        <is>
+          <t>0.937588930866984, 0.9303493449781659, 0.9308126084441875, 0.9267260659840177, 0.9226103833090733, 0.9389005937559856, 0.941760689378172</t>
+        </is>
+      </c>
+      <c r="CI97" t="n">
+        <v>0.9326783738166552</v>
+      </c>
+      <c r="CJ97" t="n">
+        <v>0.9308126084441875</v>
+      </c>
+      <c r="CK97" t="n">
+        <v>0.0064477892626383</v>
+      </c>
+      <c r="CL97" t="n">
+        <v>0.9034817670610069</v>
+      </c>
+      <c r="CM97" t="n">
+        <v>0.9010989010989011</v>
+      </c>
+      <c r="CN97" t="n">
+        <v>0.009253557801305483</v>
+      </c>
+      <c r="CO97" t="inlineStr">
+        <is>
+          <t>0.8617021276595744, 0.8526315789473684, 0.845360824742268, 0.84375, 0.8421052631578947, 0.8484848484848485, 0.8723404255319149</t>
+        </is>
+      </c>
+      <c r="CP97" t="inlineStr">
+        <is>
+          <t>0.9866071428571429, 0.9821428571428571, 0.9864864864864865, 0.9820627802690582, 0.9776785714285714, 0.9954545454545455, 0.9866666666666667</t>
+        </is>
+      </c>
+      <c r="CQ97" t="n">
+        <v>0.9852998643293326</v>
+      </c>
+      <c r="CR97" t="n">
+        <v>0.9864864864864865</v>
+      </c>
+      <c r="CS97" t="n">
+        <v>0.005163501853603294</v>
+      </c>
+      <c r="CT97" t="n">
+        <v>0.8523392955034099</v>
+      </c>
+      <c r="CU97" t="n">
+        <v>0.8484848484848485</v>
+      </c>
+      <c r="CV97" t="n">
+        <v>0.01021106185390729</v>
+      </c>
+      <c r="CW97" t="inlineStr">
+        <is>
+          <t>0.9642857142857143, 0.9529411764705882, 0.9647058823529412, 0.9529411764705882, 0.9411764705882353, 0.9882352941176471, 0.9647058823529412</t>
+        </is>
+      </c>
+      <c r="CX97" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.9401709401709402, 0.9358974358974359, 0.9358974358974359, 0.9358974358974359, 0.9358974358974359, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="CY97" t="n">
+        <v>0.9395604395604397</v>
+      </c>
+      <c r="CZ97" t="n">
+        <v>0.9358974358974359</v>
+      </c>
+      <c r="DA97" t="n">
+        <v>0.004807086614170807</v>
+      </c>
+      <c r="DB97" t="n">
+        <v>0.9612845138055223</v>
+      </c>
+      <c r="DC97" t="n">
+        <v>0.9642857142857143</v>
+      </c>
+      <c r="DD97" t="n">
+        <v>0.0136398536179124</v>
+      </c>
+      <c r="DE97" t="inlineStr">
+        <is>
+          <t>0.99239417989418, 0.9927099044746104, 0.9914781297134239, 0.9908748114630468, 0.989693313222725, 0.9942433383609854, 0.9935897435897436</t>
+        </is>
+      </c>
+      <c r="DF97" t="n">
+        <v>0.9921404886741022</v>
+      </c>
+      <c r="DG97" t="n">
+        <v>0.99239417989418</v>
+      </c>
+      <c r="DH97" t="n">
+        <v>0.001460931018726838</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>SVC_splashing_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 8.080278139769582, 'class_weight': 'balanced', 'coef0': 0.48875906950513137, 'degree': 2, 'gamma': 'auto'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 8.080278139769582, 'class_weight': 'balanced', 'coef0': 0.48875906950513137, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.8431372549019608</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.8686868686868686</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0.8927469135802468</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0.8068924539512775</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0.7997685185185186</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0.7450980392156864</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0.9057239057239057</v>
+      </c>
+      <c r="P98" t="n">
+        <v>0.9408602150537635</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0.9114583333333334</v>
+      </c>
+      <c r="R98" t="n">
+        <v>0.9259259259259259</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0.9553323412698412</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0.8981481481481481</v>
+      </c>
+      <c r="U98" t="n">
+        <v>0.9033482142857143</v>
+      </c>
+      <c r="V98" t="n">
+        <v>0.8468468468468469</v>
+      </c>
+      <c r="W98" t="n">
+        <v>0.8952380952380953</v>
+      </c>
+      <c r="X98" t="n">
+        <v>0.8703703703703703</v>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>0.019130468368530273, 0.017958402633666992, 0.01714777946472168, 0.0182952880859375, 0.0179290771484375, 0.01857900619506836, 0.016715526580810547</t>
+        </is>
+      </c>
+      <c r="Z98" t="n">
+        <v>0.01796507835388184</v>
+      </c>
+      <c r="AA98" t="n">
+        <v>0.01795840263366699</v>
+      </c>
+      <c r="AB98" t="n">
+        <v>0.0007629620386935909</v>
+      </c>
+      <c r="AC98" t="inlineStr">
+        <is>
+          <t>0.014995336532592773, 0.015069723129272461, 0.013968467712402344, 0.015926599502563477, 0.014991998672485352, 0.014536142349243164, 0.01496744155883789</t>
+        </is>
+      </c>
+      <c r="AD98" t="n">
+        <v>0.01492224420819964</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>0.01499199867248535</v>
+      </c>
+      <c r="AF98" t="n">
+        <v>0.0005479174615344102</v>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.7735849056603774, 0.9056603773584906, 0.8490566037735849, 0.9056603773584906, 0.9056603773584906, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr">
+        <is>
+          <t>0.9067669172932331, 0.7746031746031746, 0.914860681114551, 0.8707430340557275, 0.903250773993808, 0.903250773993808, 0.8738390092879257</t>
+        </is>
+      </c>
+      <c r="AI98" t="n">
+        <v>0.8781877663346039</v>
+      </c>
+      <c r="AJ98" t="n">
+        <v>0.903250773993808</v>
+      </c>
+      <c r="AK98" t="n">
+        <v>0.04507467236953443</v>
+      </c>
+      <c r="AL98" t="n">
+        <v>0.8762104422481781</v>
+      </c>
+      <c r="AM98" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="AN98" t="n">
+        <v>0.04842005697919719</v>
+      </c>
+      <c r="AO98" t="inlineStr">
+        <is>
+          <t>0.9444444444444445, 0.8181818181818182, 0.923076923076923, 0.8709677419354839, 0.9253731343283583, 0.9253731343283583, 0.8923076923076922</t>
+        </is>
+      </c>
+      <c r="AP98" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7000000000000001, 0.8780487804878049, 0.8181818181818181, 0.8717948717948718, 0.8717948717948718, 0.8292682926829269</t>
+        </is>
+      </c>
+      <c r="AQ98" t="n">
+        <v>0.8368539319758831</v>
+      </c>
+      <c r="AR98" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="AS98" t="n">
+        <v>0.06092334679157772</v>
+      </c>
+      <c r="AT98" t="inlineStr">
+        <is>
+          <t>0.9166666666666667, 0.7590909090909091, 0.900562851782364, 0.8445747800586509, 0.898584003061615, 0.898584003061615, 0.8607879924953096</t>
+        </is>
+      </c>
+      <c r="AU98" t="n">
+        <v>0.8684073151738756</v>
+      </c>
+      <c r="AV98" t="n">
+        <v>0.898584003061615</v>
+      </c>
+      <c r="AW98" t="n">
+        <v>0.05037052563869247</v>
+      </c>
+      <c r="AX98" t="n">
+        <v>0.8999606983718683</v>
+      </c>
+      <c r="AY98" t="n">
+        <v>0.923076923076923</v>
+      </c>
+      <c r="AZ98" t="n">
+        <v>0.04034085589719612</v>
+      </c>
+      <c r="BA98" t="inlineStr">
+        <is>
+          <t>0.918918918918919, 0.8709677419354839, 0.967741935483871, 0.9642857142857143, 0.9393939393939394, 0.9393939393939394, 0.9354838709677419</t>
+        </is>
+      </c>
+      <c r="BB98" t="inlineStr">
+        <is>
+          <t>0.9411764705882353, 0.6363636363636364, 0.8181818181818182, 0.72, 0.85, 0.85, 0.7727272727272727</t>
+        </is>
+      </c>
+      <c r="BC98" t="n">
+        <v>0.798349885408709</v>
+      </c>
+      <c r="BD98" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="BE98" t="n">
+        <v>0.09193396338834088</v>
+      </c>
+      <c r="BF98" t="n">
+        <v>0.9337408657685157</v>
+      </c>
+      <c r="BG98" t="n">
+        <v>0.9393939393939394</v>
+      </c>
+      <c r="BH98" t="n">
+        <v>0.03003847115866569</v>
+      </c>
+      <c r="BI98" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.7714285714285715, 0.8823529411764706, 0.7941176470588235, 0.9117647058823529, 0.9117647058823529, 0.8529411764705882</t>
+        </is>
+      </c>
+      <c r="BJ98" t="inlineStr">
+        <is>
+          <t>0.8421052631578947, 0.7777777777777778, 0.9473684210526315, 0.9473684210526315, 0.8947368421052632, 0.8947368421052632, 0.8947368421052632</t>
+        </is>
+      </c>
+      <c r="BK98" t="n">
+        <v>0.8855472013366749</v>
+      </c>
+      <c r="BL98" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM98" t="n">
+        <v>0.05528953085304691</v>
+      </c>
+      <c r="BN98" t="n">
+        <v>0.870828331332533</v>
+      </c>
+      <c r="BO98" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="BP98" t="n">
+        <v>0.06512580147218698</v>
+      </c>
+      <c r="BQ98" t="inlineStr">
+        <is>
+          <t>0.9789473684210526, 0.8809523809523809, 0.956656346749226, 0.9272445820433437, 0.9690402476780186, 0.911764705882353, 0.9148606811145511</t>
+        </is>
+      </c>
+      <c r="BR98" t="n">
+        <v>0.9342094732629895</v>
+      </c>
+      <c r="BS98" t="n">
+        <v>0.9272445820433437</v>
+      </c>
+      <c r="BT98" t="n">
+        <v>0.03269227774760999</v>
+      </c>
+      <c r="BU98" t="inlineStr">
+        <is>
+          <t>0.8962264150943396, 0.9028213166144201, 0.896551724137931, 0.8996865203761756, 0.896551724137931, 0.9059561128526645, 0.9028213166144201</t>
+        </is>
+      </c>
+      <c r="BV98" t="inlineStr">
+        <is>
+          <t>0.8996546514137708, 0.9088147197261447, 0.8959317810808489, 0.9023541541369533, 0.8959317810808489, 0.9052109287739496, 0.912771715783143</t>
+        </is>
+      </c>
+      <c r="BW98" t="n">
+        <v>0.9029528188565228</v>
+      </c>
+      <c r="BX98" t="n">
+        <v>0.9023541541369533</v>
+      </c>
+      <c r="BY98" t="n">
+        <v>0.005924500339170411</v>
+      </c>
+      <c r="BZ98" t="n">
+        <v>0.9000878756896975</v>
+      </c>
+      <c r="CA98" t="n">
+        <v>0.8996865203761756</v>
+      </c>
+      <c r="CB98" t="n">
+        <v>0.00357491869218305</v>
+      </c>
+      <c r="CC98" t="inlineStr">
+        <is>
+          <t>0.9168765743073047, 0.9215189873417722, 0.9181141439205956, 0.92, 0.9181141439205956, 0.9257425742574257, 0.921119592875318</t>
+        </is>
+      </c>
+      <c r="CD98" t="inlineStr">
+        <is>
+          <t>0.8619246861924685, 0.8724279835390947, 0.8595744680851064, 0.8655462184873949, 0.8595744680851064, 0.8717948717948718, 0.8734693877551021</t>
+        </is>
+      </c>
+      <c r="CE98" t="n">
+        <v>0.866330297705592</v>
+      </c>
+      <c r="CF98" t="n">
+        <v>0.8655462184873949</v>
+      </c>
+      <c r="CG98" t="n">
+        <v>0.005723592902356963</v>
+      </c>
+      <c r="CH98" t="inlineStr">
+        <is>
+          <t>0.8894006302498867, 0.8969734854404334, 0.888844306002851, 0.8927731092436975, 0.888844306002851, 0.8987687230261487, 0.89729449031521</t>
+        </is>
+      </c>
+      <c r="CI98" t="n">
+        <v>0.893271292897297</v>
+      </c>
+      <c r="CJ98" t="n">
+        <v>0.8927731092436975</v>
+      </c>
+      <c r="CK98" t="n">
+        <v>0.004045115702416007</v>
+      </c>
+      <c r="CL98" t="n">
+        <v>0.9202122880890017</v>
+      </c>
+      <c r="CM98" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="CN98" t="n">
+        <v>0.002753989329424617</v>
+      </c>
+      <c r="CO98" t="inlineStr">
+        <is>
+          <t>0.9479166666666666, 0.9578947368421052, 0.9390862944162437, 0.9484536082474226, 0.9390862944162437, 0.9444444444444444, 0.9679144385026738</t>
+        </is>
+      </c>
+      <c r="CP98" t="inlineStr">
+        <is>
+          <t>0.8174603174603174, 0.8217054263565892, 0.8278688524590164, 0.824, 0.8278688524590164, 0.8429752066115702, 0.8106060606060606</t>
+        </is>
+      </c>
+      <c r="CQ98" t="n">
+        <v>0.82464067370751</v>
+      </c>
+      <c r="CR98" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="CS98" t="n">
+        <v>0.009369794886213419</v>
+      </c>
+      <c r="CT98" t="n">
+        <v>0.9492566405051143</v>
+      </c>
+      <c r="CU98" t="n">
+        <v>0.9479166666666666</v>
+      </c>
+      <c r="CV98" t="n">
+        <v>0.009674706604636844</v>
+      </c>
+      <c r="CW98" t="inlineStr">
+        <is>
+          <t>0.8878048780487805, 0.8878048780487805, 0.8980582524271845, 0.8932038834951457, 0.8980582524271845, 0.9077669902912622, 0.8786407766990292</t>
+        </is>
+      </c>
+      <c r="CX98" t="inlineStr">
+        <is>
+          <t>0.911504424778761, 0.9298245614035088, 0.8938053097345132, 0.911504424778761, 0.8938053097345132, 0.9026548672566371, 0.9469026548672567</t>
+        </is>
+      </c>
+      <c r="CY98" t="n">
+        <v>0.9128573646505646</v>
+      </c>
+      <c r="CZ98" t="n">
+        <v>0.911504424778761</v>
+      </c>
+      <c r="DA98" t="n">
+        <v>0.01805025124600332</v>
+      </c>
+      <c r="DB98" t="n">
+        <v>0.893048273062481</v>
+      </c>
+      <c r="DC98" t="n">
+        <v>0.8932038834951457</v>
+      </c>
+      <c r="DD98" t="n">
+        <v>0.008696690437331071</v>
+      </c>
+      <c r="DE98" t="inlineStr">
+        <is>
+          <t>0.9574573710338873, 0.9635002139495079, 0.9559884869834178, 0.965912019932984, 0.9544849213849987, 0.9612939255949824, 0.9649669215568348</t>
+        </is>
+      </c>
+      <c r="DF98" t="n">
+        <v>0.9605148372052303</v>
+      </c>
+      <c r="DG98" t="n">
+        <v>0.9612939255949824</v>
+      </c>
+      <c r="DH98" t="n">
+        <v>0.004220120513062114</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>SVC_no_fragmentation_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 28.682610859801468, 'class_weight': None, 'coef0': 0.49963292619423594, 'degree': 2, 'gamma': 'auto'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 28.682610859801468, 'class_weight': None, 'coef0': 0.49963292619423594, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.7727272727272727</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0.9490909090909091</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0.8391938250428816</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0.8613636363636363</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="M99" t="n">
+        <v>0.8727272727272727</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0.9056603773584905</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0.9158249158249159</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0.78125</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0.9493670886075949</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0.978341656021368</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0.8987384930105694</v>
+      </c>
+      <c r="U99" t="n">
+        <v>0.9265184066891186</v>
+      </c>
+      <c r="V99" t="n">
+        <v>0.9800995024875622</v>
+      </c>
+      <c r="W99" t="n">
+        <v>0.9036697247706422</v>
+      </c>
+      <c r="X99" t="n">
+        <v>0.9403341288782816</v>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>0.022585391998291016, 0.019678592681884766, 0.018721342086791992, 0.019030094146728516, 0.021327733993530273, 0.01943683624267578, 0.018349647521972656</t>
+        </is>
+      </c>
+      <c r="Z99" t="n">
+        <v>0.01987566266741072</v>
+      </c>
+      <c r="AA99" t="n">
+        <v>0.01943683624267578</v>
+      </c>
+      <c r="AB99" t="n">
+        <v>0.00141717595152812</v>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>0.015089035034179688, 0.013850927352905273, 0.014113426208496094, 0.012748003005981445, 0.013571023941040039, 0.01359868049621582, 0.014022111892700195</t>
+        </is>
+      </c>
+      <c r="AD99" t="n">
+        <v>0.01385617256164551</v>
+      </c>
+      <c r="AE99" t="n">
+        <v>0.01385092735290527</v>
+      </c>
+      <c r="AF99" t="n">
+        <v>0.0006534900100340104</v>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.8301886792452831, 0.9056603773584906, 0.9056603773584906, 0.9245283018867925, 0.8867924528301887, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>0.9025641025641026, 0.8617216117216118, 0.9130036630036631, 0.9358974358974359, 0.9258241758241759, 0.8772893772893773, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="AI99" t="n">
+        <v>0.9056253270538986</v>
+      </c>
+      <c r="AJ99" t="n">
+        <v>0.9130036630036631</v>
+      </c>
+      <c r="AK99" t="n">
+        <v>0.02513740944440836</v>
+      </c>
+      <c r="AL99" t="n">
+        <v>0.8897873614854748</v>
+      </c>
+      <c r="AM99" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="AN99" t="n">
+        <v>0.02746839050685379</v>
+      </c>
+      <c r="AO99" t="inlineStr">
+        <is>
+          <t>0.8235294117647058, 0.742857142857143, 0.8387096774193549, 0.8484848484848484, 0.8666666666666666, 0.7999999999999999, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="AP99" t="inlineStr">
+        <is>
+          <t>0.9189189189189189, 0.8732394366197183, 0.9333333333333333, 0.9315068493150686, 0.9473684210526315, 0.9210526315789475, 0.9166666666666666</t>
+        </is>
+      </c>
+      <c r="AQ99" t="n">
+        <v>0.9202980367836122</v>
+      </c>
+      <c r="AR99" t="n">
+        <v>0.9210526315789475</v>
+      </c>
+      <c r="AS99" t="n">
+        <v>0.02157555566799157</v>
+      </c>
+      <c r="AT99" t="inlineStr">
+        <is>
+          <t>0.8712241653418124, 0.8080482897384307, 0.886021505376344, 0.8899958488999584, 0.9070175438596491, 0.8605263157894737, 0.8700980392156863</t>
+        </is>
+      </c>
+      <c r="AU99" t="n">
+        <v>0.8704188154601934</v>
+      </c>
+      <c r="AV99" t="n">
+        <v>0.8712241653418124</v>
+      </c>
+      <c r="AW99" t="n">
+        <v>0.02916668012293056</v>
+      </c>
+      <c r="AX99" t="n">
+        <v>0.8205395941367748</v>
+      </c>
+      <c r="AY99" t="n">
+        <v>0.8235294117647058</v>
+      </c>
+      <c r="AZ99" t="n">
+        <v>0.03725033493668153</v>
+      </c>
+      <c r="BA99" t="inlineStr">
+        <is>
+          <t>0.7368421052631579, 0.6190476190476191, 0.7647058823529411, 0.7368421052631579, 0.8125, 0.75, 0.7</t>
+        </is>
+      </c>
+      <c r="BB99" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.96875, 0.9722222222222222, 1.0, 0.972972972972973, 0.9459459459459459, 1.0</t>
+        </is>
+      </c>
+      <c r="BC99" t="n">
+        <v>0.9759028160813875</v>
+      </c>
+      <c r="BD99" t="n">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="BE99" t="n">
+        <v>0.01753394670277403</v>
+      </c>
+      <c r="BF99" t="n">
+        <v>0.7314196731324109</v>
+      </c>
+      <c r="BG99" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+      <c r="BH99" t="n">
+        <v>0.0556785411538445</v>
+      </c>
+      <c r="BI99" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.9285714285714286, 0.9285714285714286, 1.0, 0.9285714285714286, 0.8571428571428571, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ99" t="inlineStr">
+        <is>
+          <t>0.8717948717948718, 0.7948717948717948, 0.8974358974358975, 0.8717948717948718, 0.9230769230769231, 0.8974358974358975, 0.8461538461538461</t>
+        </is>
+      </c>
+      <c r="BK99" t="n">
+        <v>0.8717948717948717</v>
+      </c>
+      <c r="BL99" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="BM99" t="n">
+        <v>0.03876558697530539</v>
+      </c>
+      <c r="BN99" t="n">
+        <v>0.9394557823129251</v>
+      </c>
+      <c r="BO99" t="n">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="BP99" t="n">
+        <v>0.04551218689436119</v>
+      </c>
+      <c r="BQ99" t="inlineStr">
+        <is>
+          <t>0.9743589743589743, 0.924908424908425, 0.978021978021978, 0.9505494505494506, 0.978021978021978, 0.9542124542124543, 0.9926739926739927</t>
+        </is>
+      </c>
+      <c r="BR99" t="n">
+        <v>0.9646781789638933</v>
+      </c>
+      <c r="BS99" t="n">
+        <v>0.9743589743589743</v>
+      </c>
+      <c r="BT99" t="n">
+        <v>0.02112677052662096</v>
+      </c>
+      <c r="BU99" t="inlineStr">
+        <is>
+          <t>0.9119496855345912, 0.9216300940438872, 0.896551724137931, 0.9059561128526645, 0.9059561128526645, 0.9122257053291536, 0.9090909090909091</t>
+        </is>
+      </c>
+      <c r="BV99" t="inlineStr">
+        <is>
+          <t>0.924908424908425, 0.9315987933634993, 0.9182503770739066, 0.9171694318753143, 0.9171694318753143, 0.9289341377576672, 0.9193061840120664</t>
+        </is>
+      </c>
+      <c r="BW99" t="n">
+        <v>0.9224766829808848</v>
+      </c>
+      <c r="BX99" t="n">
+        <v>0.9193061840120664</v>
+      </c>
+      <c r="BY99" t="n">
+        <v>0.00554298195603807</v>
+      </c>
+      <c r="BZ99" t="n">
+        <v>0.9090514776916859</v>
+      </c>
+      <c r="CA99" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="CB99" t="n">
+        <v>0.007092298437079058</v>
+      </c>
+      <c r="CC99" t="inlineStr">
+        <is>
+          <t>0.8510638297872339, 0.8663101604278074, 0.83248730964467, 0.8421052631578947, 0.8421052631578947, 0.8541666666666666, 0.8465608465608465</t>
+        </is>
+      </c>
+      <c r="CD99" t="inlineStr">
+        <is>
+          <t>0.9375, 0.9445676274944568, 0.9251700680272109, 0.9330357142857143, 0.9330357142857143, 0.937219730941704, 0.9354120267260579</t>
+        </is>
+      </c>
+      <c r="CE99" t="n">
+        <v>0.9351344116801227</v>
+      </c>
+      <c r="CF99" t="n">
+        <v>0.9354120267260579</v>
+      </c>
+      <c r="CG99" t="n">
+        <v>0.005439332957729684</v>
+      </c>
+      <c r="CH99" t="inlineStr">
+        <is>
+          <t>0.894281914893617, 0.9054388939611321, 0.8788286888359405, 0.8875704887218046, 0.8875704887218046, 0.8956931988041853, 0.8909864366434522</t>
+        </is>
+      </c>
+      <c r="CI99" t="n">
+        <v>0.891481444368848</v>
+      </c>
+      <c r="CJ99" t="n">
+        <v>0.8909864366434522</v>
+      </c>
+      <c r="CK99" t="n">
+        <v>0.007665510075981717</v>
+      </c>
+      <c r="CL99" t="n">
+        <v>0.8478284770575735</v>
+      </c>
+      <c r="CM99" t="n">
+        <v>0.8465608465608465</v>
+      </c>
+      <c r="CN99" t="n">
+        <v>0.009961937808863407</v>
+      </c>
+      <c r="CO99" t="inlineStr">
+        <is>
+          <t>0.7692307692307693, 0.7941176470588235, 0.7321428571428571, 0.7619047619047619, 0.7619047619047619, 0.7663551401869159, 0.7692307692307693</t>
+        </is>
+      </c>
+      <c r="CP99" t="inlineStr">
+        <is>
+          <t>0.9813084112149533, 0.9815668202764977, 0.9855072463768116, 0.9766355140186916, 0.9766355140186916, 0.9858490566037735, 0.9767441860465116</t>
+        </is>
+      </c>
+      <c r="CQ99" t="n">
+        <v>0.9806066783651329</v>
+      </c>
+      <c r="CR99" t="n">
+        <v>0.9813084112149533</v>
+      </c>
+      <c r="CS99" t="n">
+        <v>0.003767749183357525</v>
+      </c>
+      <c r="CT99" t="n">
+        <v>0.764983815237094</v>
+      </c>
+      <c r="CU99" t="n">
+        <v>0.7663551401869159</v>
+      </c>
+      <c r="CV99" t="n">
+        <v>0.01683628561249153</v>
+      </c>
+      <c r="CW99" t="inlineStr">
+        <is>
+          <t>0.9523809523809523, 0.9529411764705882, 0.9647058823529412, 0.9411764705882353, 0.9411764705882353, 0.9647058823529412, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="CX99" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.9102564102564102, 0.8717948717948718, 0.8931623931623932, 0.8931623931623932, 0.8931623931623932, 0.8974358974358975</t>
+        </is>
+      </c>
+      <c r="CY99" t="n">
+        <v>0.8937728937728939</v>
+      </c>
+      <c r="CZ99" t="n">
+        <v>0.8931623931623932</v>
+      </c>
+      <c r="DA99" t="n">
+        <v>0.01057418075438874</v>
+      </c>
+      <c r="DB99" t="n">
+        <v>0.9511804721888756</v>
+      </c>
+      <c r="DC99" t="n">
+        <v>0.9523809523809523</v>
+      </c>
+      <c r="DD99" t="n">
+        <v>0.009788147472095811</v>
+      </c>
+      <c r="DE99" t="inlineStr">
+        <is>
+          <t>0.9718152218152217, 0.9776772247360482, 0.969683257918552, 0.9755656108597285, 0.9685268979386626, 0.9729512317747612, 0.966817496229261</t>
+        </is>
+      </c>
+      <c r="DF99" t="n">
+        <v>0.971862420181748</v>
+      </c>
+      <c r="DG99" t="n">
+        <v>0.9718152218152217</v>
+      </c>
+      <c r="DH99" t="n">
+        <v>0.003586463161526487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] Study no_ensembles models with SMOTENC
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4.xlsx
+++ b/results/metrics_modelling4.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH99"/>
+  <dimension ref="A1:DH105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39208,6 +39208,2346 @@
       </c>
       <c r="DH99" t="n">
         <v>0.003586463161526487</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>LogisticRegression_splashing_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.15947545233607524, 'class_weight': None, 'penalty': 'l2'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.15947545233607524, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>0.7733333333333333</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0.8604651162790697</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.8131868131868132</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0.8927469135802469</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.7625256099832372</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0.7743055555555556</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0.65625</v>
+      </c>
+      <c r="M100" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0.711864406779661</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0.8249158249158249</v>
+      </c>
+      <c r="P100" t="n">
+        <v>0.9430379746835443</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0.7760416666666666</v>
+      </c>
+      <c r="R100" t="n">
+        <v>0.8514285714285714</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0.9124751984126984</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0.8191569086651054</v>
+      </c>
+      <c r="U100" t="n">
+        <v>0.8451636904761904</v>
+      </c>
+      <c r="V100" t="n">
+        <v>0.6906474820143885</v>
+      </c>
+      <c r="W100" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="X100" t="n">
+        <v>0.7868852459016393</v>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>0.025205612182617188, 0.02387094497680664, 0.023152828216552734, 0.022998571395874023, 0.022031307220458984, 0.02233409881591797, 0.02214360237121582</t>
+        </is>
+      </c>
+      <c r="Z100" t="n">
+        <v>0.02310528073992048</v>
+      </c>
+      <c r="AA100" t="n">
+        <v>0.02299857139587402</v>
+      </c>
+      <c r="AB100" t="n">
+        <v>0.001047735483569548</v>
+      </c>
+      <c r="AC100" t="inlineStr">
+        <is>
+          <t>0.018663406372070312, 0.014111042022705078, 0.015102386474609375, 0.015038013458251953, 0.016478776931762695, 0.01497507095336914, 0.01401066780090332</t>
+        </is>
+      </c>
+      <c r="AD100" t="n">
+        <v>0.01548276628766741</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>0.01503801345825195</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>0.001500355119744491</v>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.7924528301886793, 0.8301886792452831, 0.8113207547169812, 0.8113207547169812, 0.7547169811320755, 0.7358490566037735</t>
+        </is>
+      </c>
+      <c r="AH100" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.8158730158730159, 0.8560371517027863, 0.8413312693498451, 0.818111455108359, 0.7972136222910217, 0.7244582043343653</t>
+        </is>
+      </c>
+      <c r="AI100" t="n">
+        <v>0.8245459587343709</v>
+      </c>
+      <c r="AJ100" t="n">
+        <v>0.818111455108359</v>
+      </c>
+      <c r="AK100" t="n">
+        <v>0.05482170740612071</v>
+      </c>
+      <c r="AL100" t="n">
+        <v>0.8088249975042426</v>
+      </c>
+      <c r="AM100" t="n">
+        <v>0.8113207547169812</v>
+      </c>
+      <c r="AN100" t="n">
+        <v>0.05694948286674879</v>
+      </c>
+      <c r="AO100" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8253968253968255, 0.8524590163934426, 0.8333333333333333, 0.84375, 0.7719298245614036, 0.787878787878788</t>
+        </is>
+      </c>
+      <c r="AP100" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.7441860465116279, 0.7999999999999999, 0.782608695652174, 0.761904761904762, 0.7346938775510204, 0.6500000000000001</t>
+        </is>
+      </c>
+      <c r="AQ100" t="n">
+        <v>0.7668757462464068</v>
+      </c>
+      <c r="AR100" t="n">
+        <v>0.761904761904762</v>
+      </c>
+      <c r="AS100" t="n">
+        <v>0.06858607481606634</v>
+      </c>
+      <c r="AT100" t="inlineStr">
+        <is>
+          <t>0.918796992481203, 0.7847914359542267, 0.8262295081967213, 0.8079710144927537, 0.8028273809523809, 0.753311851056212, 0.718939393939394</t>
+        </is>
+      </c>
+      <c r="AU100" t="n">
+        <v>0.8018382252961275</v>
+      </c>
+      <c r="AV100" t="n">
+        <v>0.8028273809523809</v>
+      </c>
+      <c r="AW100" t="n">
+        <v>0.05834686391288818</v>
+      </c>
+      <c r="AX100" t="n">
+        <v>0.8368007043458479</v>
+      </c>
+      <c r="AY100" t="n">
+        <v>0.8333333333333333</v>
+      </c>
+      <c r="AZ100" t="n">
+        <v>0.05110926623786245</v>
+      </c>
+      <c r="BA100" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.9285714285714286, 0.9629629629629629, 0.9615384615384616, 0.9, 0.9565217391304348, 0.8125</t>
+        </is>
+      </c>
+      <c r="BB100" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.64, 0.6923076923076923, 0.6666666666666666, 0.6956521739130435, 0.6, 0.6190476190476191</t>
+        </is>
+      </c>
+      <c r="BC100" t="n">
+        <v>0.6869158562914693</v>
+      </c>
+      <c r="BD100" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="BE100" t="n">
+        <v>0.09107810481693945</v>
+      </c>
+      <c r="BF100" t="n">
+        <v>0.9235645335800615</v>
+      </c>
+      <c r="BG100" t="n">
+        <v>0.9428571428571428</v>
+      </c>
+      <c r="BH100" t="n">
+        <v>0.04981153692023844</v>
+      </c>
+      <c r="BI100" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.7428571428571429, 0.7647058823529411, 0.7352941176470589, 0.7941176470588235, 0.6470588235294118, 0.7647058823529411</t>
+        </is>
+      </c>
+      <c r="BJ100" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8888888888888888, 0.9473684210526315, 0.9473684210526315, 0.8421052631578947, 0.9473684210526315, 0.6842105263157895</t>
+        </is>
+      </c>
+      <c r="BK100" t="n">
+        <v>0.8788638262322472</v>
+      </c>
+      <c r="BL100" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM100" t="n">
+        <v>0.08756401101589893</v>
+      </c>
+      <c r="BN100" t="n">
+        <v>0.7702280912364946</v>
+      </c>
+      <c r="BO100" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="BP100" t="n">
+        <v>0.08243847035055155</v>
+      </c>
+      <c r="BQ100" t="inlineStr">
+        <is>
+          <t>0.9654135338345865, 0.8746031746031746, 0.9427244582043344, 0.869969040247678, 0.9334365325077401, 0.826625386996904, 0.8498452012383901</t>
+        </is>
+      </c>
+      <c r="BR100" t="n">
+        <v>0.8946596182332581</v>
+      </c>
+      <c r="BS100" t="n">
+        <v>0.8746031746031746</v>
+      </c>
+      <c r="BT100" t="n">
+        <v>0.04850459279855573</v>
+      </c>
+      <c r="BU100" t="inlineStr">
+        <is>
+          <t>0.8176100628930818, 0.8181818181818182, 0.8181818181818182, 0.8307210031347962, 0.8213166144200627, 0.8150470219435737, 0.8495297805642633</t>
+        </is>
+      </c>
+      <c r="BV100" t="inlineStr">
+        <is>
+          <t>0.8327217785452191, 0.8390671801454856, 0.8392473580204485, 0.8469585015894836, 0.8376793538963828, 0.8368201735544291, 0.857526419795515</t>
+        </is>
+      </c>
+      <c r="BW100" t="n">
+        <v>0.8414315379352805</v>
+      </c>
+      <c r="BX100" t="n">
+        <v>0.8390671801454856</v>
+      </c>
+      <c r="BY100" t="n">
+        <v>0.007663986785477481</v>
+      </c>
+      <c r="BZ100" t="n">
+        <v>0.8243697313313449</v>
+      </c>
+      <c r="CA100" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="CB100" t="n">
+        <v>0.0112876343201273</v>
+      </c>
+      <c r="CC100" t="inlineStr">
+        <is>
+          <t>0.8465608465608465, 0.8440860215053763, 0.8449197860962567, 0.8578947368421053, 0.8496042216358839, 0.841823056300268, 0.876923076923077</t>
+        </is>
+      </c>
+      <c r="CD100" t="inlineStr">
+        <is>
+          <t>0.7751937984496124, 0.7819548872180451, 0.7803030303030304, 0.7906976744186046, 0.7799227799227799, 0.7773584905660378, 0.8064516129032259</t>
+        </is>
+      </c>
+      <c r="CE100" t="n">
+        <v>0.7845546105401909</v>
+      </c>
+      <c r="CF100" t="n">
+        <v>0.7803030303030304</v>
+      </c>
+      <c r="CG100" t="n">
+        <v>0.01002078727098015</v>
+      </c>
+      <c r="CH100" t="inlineStr">
+        <is>
+          <t>0.8108773225052295, 0.8130204543617107, 0.8126114081996436, 0.8242962056303549, 0.8147635007793319, 0.8095907734331529, 0.8416873449131514</t>
+        </is>
+      </c>
+      <c r="CI100" t="n">
+        <v>0.818121001403225</v>
+      </c>
+      <c r="CJ100" t="n">
+        <v>0.8130204543617107</v>
+      </c>
+      <c r="CK100" t="n">
+        <v>0.01059909278263525</v>
+      </c>
+      <c r="CL100" t="n">
+        <v>0.8516873922662592</v>
+      </c>
+      <c r="CM100" t="n">
+        <v>0.8465608465608465</v>
+      </c>
+      <c r="CN100" t="n">
+        <v>0.01138218176608377</v>
+      </c>
+      <c r="CO100" t="inlineStr">
+        <is>
+          <t>0.9248554913294798, 0.9401197604790419, 0.9404761904761905, 0.9367816091954023, 0.930635838150289, 0.9401197604790419, 0.9293478260869565</t>
+        </is>
+      </c>
+      <c r="CP100" t="inlineStr">
+        <is>
+          <t>0.6896551724137931, 0.6842105263157895, 0.6821192052980133, 0.7034482758620689, 0.6917808219178082, 0.6776315789473685, 0.7407407407407407</t>
+        </is>
+      </c>
+      <c r="CQ100" t="n">
+        <v>0.6956551887850831</v>
+      </c>
+      <c r="CR100" t="n">
+        <v>0.6896551724137931</v>
+      </c>
+      <c r="CS100" t="n">
+        <v>0.01994099788301986</v>
+      </c>
+      <c r="CT100" t="n">
+        <v>0.934619496599486</v>
+      </c>
+      <c r="CU100" t="n">
+        <v>0.9367816091954023</v>
+      </c>
+      <c r="CV100" t="n">
+        <v>0.0058367951465262</v>
+      </c>
+      <c r="CW100" t="inlineStr">
+        <is>
+          <t>0.7804878048780488, 0.7658536585365854, 0.7669902912621359, 0.7912621359223301, 0.7815533980582524, 0.7621359223300971, 0.8300970873786407</t>
+        </is>
+      </c>
+      <c r="CX100" t="inlineStr">
+        <is>
+          <t>0.8849557522123894, 0.9122807017543859, 0.911504424778761, 0.9026548672566371, 0.8938053097345132, 0.911504424778761, 0.8849557522123894</t>
+        </is>
+      </c>
+      <c r="CY100" t="n">
+        <v>0.9002373189611197</v>
+      </c>
+      <c r="CZ100" t="n">
+        <v>0.9026548672566371</v>
+      </c>
+      <c r="DA100" t="n">
+        <v>0.01142182286653244</v>
+      </c>
+      <c r="DB100" t="n">
+        <v>0.7826257569094415</v>
+      </c>
+      <c r="DC100" t="n">
+        <v>0.7804878048780488</v>
+      </c>
+      <c r="DD100" t="n">
+        <v>0.02164466097906357</v>
+      </c>
+      <c r="DE100" t="inlineStr">
+        <is>
+          <t>0.8992661342542628, 0.9124946512623021, 0.9023326746284045, 0.9098934616375978, 0.9041799123636052, 0.9214709167454249, 0.9104519288598677</t>
+        </is>
+      </c>
+      <c r="DF100" t="n">
+        <v>0.9085842399644949</v>
+      </c>
+      <c r="DG100" t="n">
+        <v>0.9098934616375978</v>
+      </c>
+      <c r="DH100" t="n">
+        <v>0.006885464430521382</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>LogisticRegression_no_fragmentation_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'liblinear', 'C': 377.1313111077982, 'class_weight': None, 'penalty': 'l1'}, 'base_estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'liblinear', 'C': 377.1313111077982, 'class_weight': None, 'penalty': 'l1'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0.9581818181818181</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.8161764705882353</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0.8590909090909091</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0.9574468085106383</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0.8316498316498316</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0.6355140186915887</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0.8607594936708861</v>
+      </c>
+      <c r="R101" t="n">
+        <v>0.7311827956989247</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0.9419927999070956</v>
+      </c>
+      <c r="T101" t="n">
+        <v>0.8043168880455408</v>
+      </c>
+      <c r="U101" t="n">
+        <v>0.8409302055510394</v>
+      </c>
+      <c r="V101" t="n">
+        <v>0.9421052631578948</v>
+      </c>
+      <c r="W101" t="n">
+        <v>0.8211009174311926</v>
+      </c>
+      <c r="X101" t="n">
+        <v>0.8774509803921569</v>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>0.024035215377807617, 0.020569324493408203, 0.02002739906311035, 0.021613359451293945, 0.021079540252685547, 0.021424055099487305, 0.02055525779724121</t>
+        </is>
+      </c>
+      <c r="Z101" t="n">
+        <v>0.02132916450500488</v>
+      </c>
+      <c r="AA101" t="n">
+        <v>0.02107954025268555</v>
+      </c>
+      <c r="AB101" t="n">
+        <v>0.001215711213782499</v>
+      </c>
+      <c r="AC101" t="inlineStr">
+        <is>
+          <t>0.013138532638549805, 0.012949466705322266, 0.01444697380065918, 0.012259721755981445, 0.01354074478149414, 0.013348817825317383, 0.012997865676879883</t>
+        </is>
+      </c>
+      <c r="AD101" t="n">
+        <v>0.01324030331202916</v>
+      </c>
+      <c r="AE101" t="n">
+        <v>0.0131385326385498</v>
+      </c>
+      <c r="AF101" t="n">
+        <v>0.000617986770671858</v>
+      </c>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>0.8518518518518519, 0.7358490566037735, 0.8679245283018868, 0.7924528301886793, 0.7924528301886793, 0.8490566037735849, 0.9056603773584906</t>
+        </is>
+      </c>
+      <c r="AH101" t="inlineStr">
+        <is>
+          <t>0.8564102564102565, 0.728937728937729, 0.8873626373626373, 0.7902930402930403, 0.8131868131868132, 0.8287545787545787, 0.9358974358974359</t>
+        </is>
+      </c>
+      <c r="AI101" t="n">
+        <v>0.8344060701203558</v>
+      </c>
+      <c r="AJ101" t="n">
+        <v>0.8287545787545787</v>
+      </c>
+      <c r="AK101" t="n">
+        <v>0.06226763223318901</v>
+      </c>
+      <c r="AL101" t="n">
+        <v>0.8278925826095638</v>
+      </c>
+      <c r="AM101" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="AN101" t="n">
+        <v>0.05299098539693286</v>
+      </c>
+      <c r="AO101" t="inlineStr">
+        <is>
+          <t>0.7647058823529413, 0.588235294117647, 0.7878787878787878, 0.6666666666666667, 0.6857142857142857, 0.7333333333333334, 0.8484848484848484</t>
+        </is>
+      </c>
+      <c r="AP101" t="inlineStr">
+        <is>
+          <t>0.8918918918918919, 0.8055555555555556, 0.9041095890410958, 0.8493150684931507, 0.8450704225352113, 0.8947368421052632, 0.9315068493150686</t>
+        </is>
+      </c>
+      <c r="AQ101" t="n">
+        <v>0.8745980312767481</v>
+      </c>
+      <c r="AR101" t="n">
+        <v>0.8918918918918919</v>
+      </c>
+      <c r="AS101" t="n">
+        <v>0.0398069740257037</v>
+      </c>
+      <c r="AT101" t="inlineStr">
+        <is>
+          <t>0.8282988871224166, 0.6968954248366013, 0.8459941884599418, 0.7579908675799087, 0.7653923541247485, 0.8140350877192983, 0.8899958488999584</t>
+        </is>
+      </c>
+      <c r="AU101" t="n">
+        <v>0.7998003798204104</v>
+      </c>
+      <c r="AV101" t="n">
+        <v>0.8140350877192983</v>
+      </c>
+      <c r="AW101" t="n">
+        <v>0.05952821627813664</v>
+      </c>
+      <c r="AX101" t="n">
+        <v>0.725002728364073</v>
+      </c>
+      <c r="AY101" t="n">
+        <v>0.7333333333333334</v>
+      </c>
+      <c r="AZ101" t="n">
+        <v>0.07973078017929812</v>
+      </c>
+      <c r="BA101" t="inlineStr">
+        <is>
+          <t>0.6842105263157895, 0.5, 0.6842105263157895, 0.5789473684210527, 0.5714285714285714, 0.6875, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="BB101" t="inlineStr">
+        <is>
+          <t>0.9428571428571428, 0.8787878787878788, 0.9705882352941176, 0.9117647058823529, 0.9375, 0.918918918918919, 1.0</t>
+        </is>
+      </c>
+      <c r="BC101" t="n">
+        <v>0.9372024116772016</v>
+      </c>
+      <c r="BD101" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="BE101" t="n">
+        <v>0.03680806491108783</v>
+      </c>
+      <c r="BF101" t="n">
+        <v>0.634734156820623</v>
+      </c>
+      <c r="BG101" t="n">
+        <v>0.6842105263157895</v>
+      </c>
+      <c r="BH101" t="n">
+        <v>0.0787211584684933</v>
+      </c>
+      <c r="BI101" t="inlineStr">
+        <is>
+          <t>0.8666666666666667, 0.7142857142857143, 0.9285714285714286, 0.7857142857142857, 0.8571428571428571, 0.7857142857142857, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ101" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.7435897435897436, 0.8461538461538461, 0.7948717948717948, 0.7692307692307693, 0.8717948717948718, 0.8717948717948718</t>
+        </is>
+      </c>
+      <c r="BK101" t="n">
+        <v>0.8205128205128206</v>
+      </c>
+      <c r="BL101" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="BM101" t="n">
+        <v>0.04747795383448981</v>
+      </c>
+      <c r="BN101" t="n">
+        <v>0.8482993197278911</v>
+      </c>
+      <c r="BO101" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP101" t="n">
+        <v>0.08917534480638879</v>
+      </c>
+      <c r="BQ101" t="inlineStr">
+        <is>
+          <t>0.9521367521367521, 0.8974358974358975, 0.9670329670329672, 0.9304029304029304, 0.9175824175824175, 0.9304029304029304, 0.9981684981684982</t>
+        </is>
+      </c>
+      <c r="BR101" t="n">
+        <v>0.941880341880342</v>
+      </c>
+      <c r="BS101" t="n">
+        <v>0.9304029304029304</v>
+      </c>
+      <c r="BT101" t="n">
+        <v>0.03101926764665284</v>
+      </c>
+      <c r="BU101" t="inlineStr">
+        <is>
+          <t>0.8301886792452831, 0.8652037617554859, 0.8369905956112853, 0.8495297805642633, 0.8495297805642633, 0.8463949843260188, 0.8369905956112853</t>
+        </is>
+      </c>
+      <c r="BV101" t="inlineStr">
+        <is>
+          <t>0.8350122100122099, 0.8781548516842634, 0.8514328808446455, 0.8599798893916542, 0.8562342885872298, 0.857843137254902, 0.8514328808446455</t>
+        </is>
+      </c>
+      <c r="BW101" t="n">
+        <v>0.8557271626599355</v>
+      </c>
+      <c r="BX101" t="n">
+        <v>0.8562342885872298</v>
+      </c>
+      <c r="BY101" t="n">
+        <v>0.01190325538086766</v>
+      </c>
+      <c r="BZ101" t="n">
+        <v>0.8449754539539835</v>
+      </c>
+      <c r="CA101" t="n">
+        <v>0.8463949843260188</v>
+      </c>
+      <c r="CB101" t="n">
+        <v>0.0106827492216419</v>
+      </c>
+      <c r="CC101" t="inlineStr">
+        <is>
+          <t>0.7244897959183674, 0.7817258883248731, 0.7425742574257426, 0.7575757575757577, 0.7551020408163265, 0.7537688442211056, 0.7425742574257426</t>
+        </is>
+      </c>
+      <c r="CD101" t="inlineStr">
+        <is>
+          <t>0.8772727272727272, 0.9024943310657597, 0.8807339449541284, 0.8909090909090909, 0.8914027149321265, 0.8883826879271071, 0.8807339449541284</t>
+        </is>
+      </c>
+      <c r="CE101" t="n">
+        <v>0.8874184917164384</v>
+      </c>
+      <c r="CF101" t="n">
+        <v>0.8883826879271071</v>
+      </c>
+      <c r="CG101" t="n">
+        <v>0.00800510364667156</v>
+      </c>
+      <c r="CH101" t="inlineStr">
+        <is>
+          <t>0.8008812615955473, 0.8421101096953164, 0.8116541011899354, 0.8242424242424242, 0.8232523778742264, 0.8210757660741064, 0.8116541011899354</t>
+        </is>
+      </c>
+      <c r="CI101" t="n">
+        <v>0.8192671631230704</v>
+      </c>
+      <c r="CJ101" t="n">
+        <v>0.8210757660741064</v>
+      </c>
+      <c r="CK101" t="n">
+        <v>0.01206923604832221</v>
+      </c>
+      <c r="CL101" t="n">
+        <v>0.7511158345297021</v>
+      </c>
+      <c r="CM101" t="n">
+        <v>0.7537688442211056</v>
+      </c>
+      <c r="CN101" t="n">
+        <v>0.01628538920568498</v>
+      </c>
+      <c r="CO101" t="inlineStr">
+        <is>
+          <t>0.6339285714285714, 0.6875, 0.6410256410256411, 0.6637168141592921, 0.6666666666666666, 0.6578947368421053, 0.6410256410256411</t>
+        </is>
+      </c>
+      <c r="CP101" t="inlineStr">
+        <is>
+          <t>0.9368932038834952, 0.961352657004831, 0.9504950495049505, 0.9514563106796117, 0.9471153846153846, 0.9512195121951219, 0.9504950495049505</t>
+        </is>
+      </c>
+      <c r="CQ101" t="n">
+        <v>0.9498610239126207</v>
+      </c>
+      <c r="CR101" t="n">
+        <v>0.9504950495049505</v>
+      </c>
+      <c r="CS101" t="n">
+        <v>0.006686392682908714</v>
+      </c>
+      <c r="CT101" t="n">
+        <v>0.6559654387354168</v>
+      </c>
+      <c r="CU101" t="n">
+        <v>0.6578947368421053</v>
+      </c>
+      <c r="CV101" t="n">
+        <v>0.01734016591389645</v>
+      </c>
+      <c r="CW101" t="inlineStr">
+        <is>
+          <t>0.8452380952380952, 0.9058823529411765, 0.8823529411764706, 0.8823529411764706, 0.8705882352941177, 0.8823529411764706, 0.8823529411764706</t>
+        </is>
+      </c>
+      <c r="CX101" t="inlineStr">
+        <is>
+          <t>0.8247863247863247, 0.8504273504273504, 0.8205128205128205, 0.8376068376068376, 0.8418803418803419, 0.8333333333333334, 0.8205128205128205</t>
+        </is>
+      </c>
+      <c r="CY101" t="n">
+        <v>0.8327228327228327</v>
+      </c>
+      <c r="CZ101" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="DA101" t="n">
+        <v>0.01057418075438876</v>
+      </c>
+      <c r="DB101" t="n">
+        <v>0.8787314925970389</v>
+      </c>
+      <c r="DC101" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="DD101" t="n">
+        <v>0.01680879481881183</v>
+      </c>
+      <c r="DE101" t="inlineStr">
+        <is>
+          <t>0.9433760683760684, 0.9537456008044243, 0.9415786827551533, 0.9482151835093011, 0.945550527903469, 0.9516339869281046, 0.9359477124183007</t>
+        </is>
+      </c>
+      <c r="DF101" t="n">
+        <v>0.9457211089564032</v>
+      </c>
+      <c r="DG101" t="n">
+        <v>0.9455505279034691</v>
+      </c>
+      <c r="DH101" t="n">
+        <v>0.005654104591804274</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_splashing_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 1, 'weights': 'distance', 'p': 1}, 'base_estimator_params': {'n_neighbors': 1, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.8910891089108911</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0.8206018518518519</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0.8332996564962618</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0.8206018518518519</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0.8636363636363636</v>
+      </c>
+      <c r="M102" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0.7755102040816326</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P102" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0.9947916666666666</v>
+      </c>
+      <c r="R102" t="n">
+        <v>0.9973890339425587</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0.9973958333333333</v>
+      </c>
+      <c r="T102" t="n">
+        <v>0.996324848724834</v>
+      </c>
+      <c r="U102" t="n">
+        <v>0.9973958333333333</v>
+      </c>
+      <c r="V102" t="n">
+        <v>0.9905660377358491</v>
+      </c>
+      <c r="W102" t="n">
+        <v>1</v>
+      </c>
+      <c r="X102" t="n">
+        <v>0.9952606635071091</v>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>0.026993751525878906, 0.020168304443359375, 0.019930124282836914, 0.02133655548095703, 0.020959138870239258, 0.021331071853637695, 0.02089977264404297</t>
+        </is>
+      </c>
+      <c r="Z102" t="n">
+        <v>0.02165981701442174</v>
+      </c>
+      <c r="AA102" t="n">
+        <v>0.02095913887023926</v>
+      </c>
+      <c r="AB102" t="n">
+        <v>0.002234422033747832</v>
+      </c>
+      <c r="AC102" t="inlineStr">
+        <is>
+          <t>0.02968573570251465, 0.015359640121459961, 0.015287637710571289, 0.01620316505432129, 0.015335321426391602, 0.016111373901367188, 0.015524625778198242</t>
+        </is>
+      </c>
+      <c r="AD102" t="n">
+        <v>0.01764392852783203</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>0.01552462577819824</v>
+      </c>
+      <c r="AF102" t="n">
+        <v>0.004928355766586994</v>
+      </c>
+      <c r="AG102" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.8113207547169812, 0.9245283018867925, 0.9245283018867925, 0.9056603773584906, 0.9056603773584906, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH102" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8166666666666667, 0.9295665634674922, 0.9295665634674922, 0.891640866873065, 0.914860681114551, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AI102" t="n">
+        <v>0.8934247383163791</v>
+      </c>
+      <c r="AJ102" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="AK102" t="n">
+        <v>0.03633294461637566</v>
+      </c>
+      <c r="AL102" t="n">
+        <v>0.8977737845662374</v>
+      </c>
+      <c r="AM102" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="AN102" t="n">
+        <v>0.03768907413827519</v>
+      </c>
+      <c r="AO102" t="inlineStr">
+        <is>
+          <t>0.945945945945946, 0.8484848484848486, 0.9393939393939394, 0.9393939393939394, 0.9275362318840579, 0.923076923076923, 0.9117647058823528</t>
+        </is>
+      </c>
+      <c r="AP102" t="inlineStr">
+        <is>
+          <t>0.8823529411764706, 0.7499999999999999, 0.9, 0.9, 0.8648648648648649, 0.8780487804878049, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="AQ102" t="n">
+        <v>0.8596245499552906</v>
+      </c>
+      <c r="AR102" t="n">
+        <v>0.8780487804878049</v>
+      </c>
+      <c r="AS102" t="n">
+        <v>0.04850377633896862</v>
+      </c>
+      <c r="AT102" t="inlineStr">
+        <is>
+          <t>0.9141494435612083, 0.7992424242424243, 0.9196969696969697, 0.9196969696969697, 0.8962005483744614, 0.900562851782364, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="AU102" t="n">
+        <v>0.8894977416963601</v>
+      </c>
+      <c r="AV102" t="n">
+        <v>0.9005628517823639</v>
+      </c>
+      <c r="AW102" t="n">
+        <v>0.03946590322880562</v>
+      </c>
+      <c r="AX102" t="n">
+        <v>0.9193709334374296</v>
+      </c>
+      <c r="AY102" t="n">
+        <v>0.9275362318840579</v>
+      </c>
+      <c r="AZ102" t="n">
+        <v>0.03087109378494328</v>
+      </c>
+      <c r="BA102" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.9032258064516129, 0.96875, 0.96875, 0.9142857142857143, 0.967741935483871, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BB102" t="inlineStr">
+        <is>
+          <t>1.0, 0.6818181818181818, 0.8571428571428571, 0.8571428571428571, 0.8888888888888888, 0.8181818181818182, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BC102" t="n">
+        <v>0.8493256951903568</v>
+      </c>
+      <c r="BD102" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BE102" t="n">
+        <v>0.08739978033436586</v>
+      </c>
+      <c r="BF102" t="n">
+        <v>0.9331362942199213</v>
+      </c>
+      <c r="BG102" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="BH102" t="n">
+        <v>0.03097341543755244</v>
+      </c>
+      <c r="BI102" t="inlineStr">
+        <is>
+          <t>1.0, 0.8, 0.9117647058823529, 0.9117647058823529, 0.9411764705882353, 0.8823529411764706, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BJ102" t="inlineStr">
+        <is>
+          <t>0.7894736842105263, 0.8333333333333334, 0.9473684210526315, 0.9473684210526315, 0.8421052631578947, 0.9473684210526315, 0.8421052631578947</t>
+        </is>
+      </c>
+      <c r="BK102" t="n">
+        <v>0.8784461152882205</v>
+      </c>
+      <c r="BL102" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BM102" t="n">
+        <v>0.06192555940153299</v>
+      </c>
+      <c r="BN102" t="n">
+        <v>0.9084033613445379</v>
+      </c>
+      <c r="BO102" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BP102" t="n">
+        <v>0.0559691623709133</v>
+      </c>
+      <c r="BQ102" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8166666666666667, 0.9295665634674923, 0.9295665634674923, 0.891640866873065, 0.9148606811145512, 0.8769349845201238</t>
+        </is>
+      </c>
+      <c r="BR102" t="n">
+        <v>0.8934247383163791</v>
+      </c>
+      <c r="BS102" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BT102" t="n">
+        <v>0.03633294461637571</v>
+      </c>
+      <c r="BU102" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV102" t="inlineStr">
+        <is>
+          <t>0.995575221238938, 1.0, 0.9975728155339806, 0.995575221238938, 0.995575221238938, 1.0, 0.9975728155339806</t>
+        </is>
+      </c>
+      <c r="BW102" t="n">
+        <v>0.9974101849692536</v>
+      </c>
+      <c r="BX102" t="n">
+        <v>0.9975728155339806</v>
+      </c>
+      <c r="BY102" t="n">
+        <v>0.00183491754827791</v>
+      </c>
+      <c r="BZ102" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA102" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB102" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC102" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975669099756691, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975669099756691</t>
+        </is>
+      </c>
+      <c r="CD102" t="inlineStr">
+        <is>
+          <t>0.9955555555555555, 1.0, 0.9955947136563876, 0.9955555555555555, 0.9955555555555555, 1.0, 0.9955947136563876</t>
+        </is>
+      </c>
+      <c r="CE102" t="n">
+        <v>0.996836584854206</v>
+      </c>
+      <c r="CF102" t="n">
+        <v>0.9955947136563876</v>
+      </c>
+      <c r="CG102" t="n">
+        <v>0.002000785099662565</v>
+      </c>
+      <c r="CH102" t="inlineStr">
+        <is>
+          <t>0.9965612327656124, 1.0, 0.9965808118160284, 0.9965671240247511, 0.9965671240247511, 1.0, 0.9965808118160284</t>
+        </is>
+      </c>
+      <c r="CI102" t="n">
+        <v>0.9975510149210244</v>
+      </c>
+      <c r="CJ102" t="n">
+        <v>0.9965808118160284</v>
+      </c>
+      <c r="CK102" t="n">
+        <v>0.001548888784658625</v>
+      </c>
+      <c r="CL102" t="n">
+        <v>0.9982654449878429</v>
+      </c>
+      <c r="CM102" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="CN102" t="n">
+        <v>0.001097039760045307</v>
+      </c>
+      <c r="CO102" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 1.0, 0.9951690821256038, 0.9951690821256038, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP102" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 0.9912280701754386, 1.0, 1.0, 1.0, 0.9912280701754386</t>
+        </is>
+      </c>
+      <c r="CQ102" t="n">
+        <v>0.9974937343358395</v>
+      </c>
+      <c r="CR102" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS102" t="n">
+        <v>0.003962753960110764</v>
+      </c>
+      <c r="CT102" t="n">
+        <v>0.997926256474167</v>
+      </c>
+      <c r="CU102" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV102" t="n">
+        <v>0.002394563702285534</v>
+      </c>
+      <c r="CW102" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 0.9951456310679612, 1.0, 1.0, 1.0, 0.9951456310679612</t>
+        </is>
+      </c>
+      <c r="CX102" t="inlineStr">
+        <is>
+          <t>0.9911504424778761, 1.0, 1.0, 0.9911504424778761, 0.9911504424778761, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY102" t="n">
+        <v>0.9962073324905182</v>
+      </c>
+      <c r="CZ102" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA102" t="n">
+        <v>0.004379395215091984</v>
+      </c>
+      <c r="DB102" t="n">
+        <v>0.998613037447989</v>
+      </c>
+      <c r="DC102" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD102" t="n">
+        <v>0.002192980346857405</v>
+      </c>
+      <c r="DE102" t="inlineStr">
+        <is>
+          <t>0.995575221238938, 1.0, 0.9975728155339806, 0.995575221238938, 0.995575221238938, 1.0, 0.9975728155339806</t>
+        </is>
+      </c>
+      <c r="DF102" t="n">
+        <v>0.9974101849692536</v>
+      </c>
+      <c r="DG102" t="n">
+        <v>0.9975728155339806</v>
+      </c>
+      <c r="DH102" t="n">
+        <v>0.00183491754827791</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>KNeighborsClassifier_no_fragmentation_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'base_estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.6956521739130435</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.7441860465116279</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0.9027272727272728</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0.8206911540969355</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0.8363636363636364</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0.8727272727272727</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0.897196261682243</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.9427609427609428</v>
+      </c>
+      <c r="P103" t="n">
+        <v>0.8369565217391305</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0.9746835443037974</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0.9005847953216375</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0.9915515038903728</v>
+      </c>
+      <c r="T103" t="n">
+        <v>0.9301978350130646</v>
+      </c>
+      <c r="U103" t="n">
+        <v>0.9529381024271281</v>
+      </c>
+      <c r="V103" t="n">
+        <v>0.9902439024390244</v>
+      </c>
+      <c r="W103" t="n">
+        <v>0.9311926605504587</v>
+      </c>
+      <c r="X103" t="n">
+        <v>0.9598108747044918</v>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>0.024509429931640625, 0.020848751068115234, 0.020676612854003906, 0.01972341537475586, 0.019952058792114258, 0.021252870559692383, 0.020036697387695312</t>
+        </is>
+      </c>
+      <c r="Z103" t="n">
+        <v>0.02099997656685965</v>
+      </c>
+      <c r="AA103" t="n">
+        <v>0.02067661285400391</v>
+      </c>
+      <c r="AB103" t="n">
+        <v>0.001519553433003547</v>
+      </c>
+      <c r="AC103" t="inlineStr">
+        <is>
+          <t>0.018678665161132812, 0.015993595123291016, 0.015009641647338867, 0.016558170318603516, 0.015002727508544922, 0.015459299087524414, 0.017819881439208984</t>
+        </is>
+      </c>
+      <c r="AD103" t="n">
+        <v>0.01636028289794922</v>
+      </c>
+      <c r="AE103" t="n">
+        <v>0.01599359512329102</v>
+      </c>
+      <c r="AF103" t="n">
+        <v>0.001317893547891996</v>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>0.8703703703703703, 0.7358490566037735, 0.9245283018867925, 0.8867924528301887, 0.8867924528301887, 0.8867924528301887, 0.8490566037735849</t>
+        </is>
+      </c>
+      <c r="AH103" t="inlineStr">
+        <is>
+          <t>0.8487179487179488, 0.728937728937729, 0.9029304029304028, 0.9001831501831502, 0.8315018315018314, 0.8543956043956045, 0.8745421245421245</t>
+        </is>
+      </c>
+      <c r="AI103" t="n">
+        <v>0.8487441130298272</v>
+      </c>
+      <c r="AJ103" t="n">
+        <v>0.8543956043956045</v>
+      </c>
+      <c r="AK103" t="n">
+        <v>0.05468150893411447</v>
+      </c>
+      <c r="AL103" t="n">
+        <v>0.8628830987321555</v>
+      </c>
+      <c r="AM103" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN103" t="n">
+        <v>0.05593361086531986</v>
+      </c>
+      <c r="AO103" t="inlineStr">
+        <is>
+          <t>0.7741935483870969, 0.588235294117647, 0.8571428571428571, 0.8125000000000001, 0.7692307692307692, 0.7857142857142857, 0.7647058823529412</t>
+        </is>
+      </c>
+      <c r="AP103" t="inlineStr">
+        <is>
+          <t>0.9090909090909091, 0.8055555555555556, 0.9487179487179487, 0.9189189189189189, 0.9249999999999999, 0.9230769230769231, 0.8888888888888888</t>
+        </is>
+      </c>
+      <c r="AQ103" t="n">
+        <v>0.9027498777498779</v>
+      </c>
+      <c r="AR103" t="n">
+        <v>0.9189189189189189</v>
+      </c>
+      <c r="AS103" t="n">
+        <v>0.04303126788446314</v>
+      </c>
+      <c r="AT103" t="inlineStr">
+        <is>
+          <t>0.841642228739003, 0.6968954248366013, 0.9029304029304028, 0.8657094594594594, 0.8471153846153845, 0.8543956043956045, 0.826797385620915</t>
+        </is>
+      </c>
+      <c r="AU103" t="n">
+        <v>0.8336408415139099</v>
+      </c>
+      <c r="AV103" t="n">
+        <v>0.8471153846153845</v>
+      </c>
+      <c r="AW103" t="n">
+        <v>0.06006178621176272</v>
+      </c>
+      <c r="AX103" t="n">
+        <v>0.7645318052779425</v>
+      </c>
+      <c r="AY103" t="n">
+        <v>0.7741935483870969</v>
+      </c>
+      <c r="AZ103" t="n">
+        <v>0.07793987774662568</v>
+      </c>
+      <c r="BA103" t="inlineStr">
+        <is>
+          <t>0.75, 0.5, 0.8571428571428571, 0.7222222222222222, 0.8333333333333334, 0.7857142857142857, 0.65</t>
+        </is>
+      </c>
+      <c r="BB103" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.8787878787878788, 0.9487179487179487, 0.9714285714285714, 0.9024390243902439, 0.9230769230769231, 0.9696969696969697</t>
+        </is>
+      </c>
+      <c r="BC103" t="n">
+        <v>0.9307428496682119</v>
+      </c>
+      <c r="BD103" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="BE103" t="n">
+        <v>0.03195744467231082</v>
+      </c>
+      <c r="BF103" t="n">
+        <v>0.7283446712018141</v>
+      </c>
+      <c r="BG103" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="BH103" t="n">
+        <v>0.1131929317366905</v>
+      </c>
+      <c r="BI103" t="inlineStr">
+        <is>
+          <t>0.8, 0.7142857142857143, 0.8571428571428571, 0.9285714285714286, 0.7142857142857143, 0.7857142857142857, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ103" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.7435897435897436, 0.9487179487179487, 0.8717948717948718, 0.9487179487179487, 0.9230769230769231, 0.8205128205128205</t>
+        </is>
+      </c>
+      <c r="BK103" t="n">
+        <v>0.879120879120879</v>
+      </c>
+      <c r="BL103" t="n">
+        <v>0.8974358974358975</v>
+      </c>
+      <c r="BM103" t="n">
+        <v>0.06950060791578855</v>
+      </c>
+      <c r="BN103" t="n">
+        <v>0.8183673469387756</v>
+      </c>
+      <c r="BO103" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BP103" t="n">
+        <v>0.08354893669574988</v>
+      </c>
+      <c r="BQ103" t="inlineStr">
+        <is>
+          <t>0.9034188034188034, 0.7701465201465201, 0.934981684981685, 0.9560439560439561, 0.9578754578754579, 0.8946886446886447, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="BR103" t="n">
+        <v>0.9094104308390023</v>
+      </c>
+      <c r="BS103" t="n">
+        <v>0.934981684981685</v>
+      </c>
+      <c r="BT103" t="n">
+        <v>0.06137656826844985</v>
+      </c>
+      <c r="BU103" t="inlineStr">
+        <is>
+          <t>0.9433962264150944, 0.9404388714733543, 0.9341692789968652, 0.9373040752351097, 0.9373040752351097, 0.9435736677115988, 0.9467084639498433</t>
+        </is>
+      </c>
+      <c r="BV103" t="inlineStr">
+        <is>
+          <t>0.9424603174603174, 0.944419306184012, 0.9326546003016591, 0.9385369532428356, 0.9235545500251383, 0.9465560583207642, 0.944947209653092</t>
+        </is>
+      </c>
+      <c r="BW103" t="n">
+        <v>0.9390184278839743</v>
+      </c>
+      <c r="BX103" t="n">
+        <v>0.9424603174603174</v>
+      </c>
+      <c r="BY103" t="n">
+        <v>0.007679695435697343</v>
+      </c>
+      <c r="BZ103" t="n">
+        <v>0.9404135227167106</v>
+      </c>
+      <c r="CA103" t="n">
+        <v>0.9404388714733543</v>
+      </c>
+      <c r="CB103" t="n">
+        <v>0.004085477281850636</v>
+      </c>
+      <c r="CC103" t="inlineStr">
+        <is>
+          <t>0.8977272727272727, 0.8950276243093922, 0.8826815642458101, 0.8888888888888888, 0.8837209302325582, 0.9, 0.903954802259887</t>
+        </is>
+      </c>
+      <c r="CD103" t="inlineStr">
+        <is>
+          <t>0.9608695652173912, 0.9584245076586433, 0.954248366013072, 0.9563318777292577, 0.9570815450643777, 0.9606986899563319, 0.963123644251627</t>
+        </is>
+      </c>
+      <c r="CE103" t="n">
+        <v>0.9586825994129572</v>
+      </c>
+      <c r="CF103" t="n">
+        <v>0.9584245076586433</v>
+      </c>
+      <c r="CG103" t="n">
+        <v>0.002838224405392204</v>
+      </c>
+      <c r="CH103" t="inlineStr">
+        <is>
+          <t>0.9292984189723319, 0.9267260659840177, 0.918464965129441, 0.9226103833090733, 0.9204012376484679, 0.9303493449781659, 0.933539223255757</t>
+        </is>
+      </c>
+      <c r="CI103" t="n">
+        <v>0.9259128056110363</v>
+      </c>
+      <c r="CJ103" t="n">
+        <v>0.9267260659840177</v>
+      </c>
+      <c r="CK103" t="n">
+        <v>0.005164751414568978</v>
+      </c>
+      <c r="CL103" t="n">
+        <v>0.8931430118091156</v>
+      </c>
+      <c r="CM103" t="n">
+        <v>0.8950276243093922</v>
+      </c>
+      <c r="CN103" t="n">
+        <v>0.007604466548574816</v>
+      </c>
+      <c r="CO103" t="inlineStr">
+        <is>
+          <t>0.8586956521739131, 0.84375, 0.8404255319148937, 0.8421052631578947, 0.8735632183908046, 0.8526315789473684, 0.8695652173913043</t>
+        </is>
+      </c>
+      <c r="CP103" t="inlineStr">
+        <is>
+          <t>0.9778761061946902, 0.9820627802690582, 0.9733333333333334, 0.9776785714285714, 0.9612068965517241, 0.9821428571428571, 0.9779735682819384</t>
+        </is>
+      </c>
+      <c r="CQ103" t="n">
+        <v>0.9760391590288817</v>
+      </c>
+      <c r="CR103" t="n">
+        <v>0.9778761061946902</v>
+      </c>
+      <c r="CS103" t="n">
+        <v>0.006661838371995908</v>
+      </c>
+      <c r="CT103" t="n">
+        <v>0.8543909231394541</v>
+      </c>
+      <c r="CU103" t="n">
+        <v>0.8526315789473684</v>
+      </c>
+      <c r="CV103" t="n">
+        <v>0.01241347731753288</v>
+      </c>
+      <c r="CW103" t="inlineStr">
+        <is>
+          <t>0.9404761904761905, 0.9529411764705882, 0.9294117647058824, 0.9411764705882353, 0.8941176470588236, 0.9529411764705882, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="CX103" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.9358974358974359, 0.9358974358974359, 0.9358974358974359, 0.9529914529914529, 0.9401709401709402, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="CY103" t="n">
+        <v>0.9420024420024421</v>
+      </c>
+      <c r="CZ103" t="n">
+        <v>0.9401709401709402</v>
+      </c>
+      <c r="DA103" t="n">
+        <v>0.006402984421063173</v>
+      </c>
+      <c r="DB103" t="n">
+        <v>0.9360344137655063</v>
+      </c>
+      <c r="DC103" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="DD103" t="n">
+        <v>0.01868980982523908</v>
+      </c>
+      <c r="DE103" t="inlineStr">
+        <is>
+          <t>0.9907407407407407, 0.9920563097033686, 0.9874057315233786, 0.9886877828054299, 0.9866767219708397, 0.9913021618903971, 0.9913021618903972</t>
+        </is>
+      </c>
+      <c r="DF103" t="n">
+        <v>0.9897388015035073</v>
+      </c>
+      <c r="DG103" t="n">
+        <v>0.9907407407407407</v>
+      </c>
+      <c r="DH103" t="n">
+        <v>0.001970754199009418</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>SVC_splashing_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 26.972626232440984, 'class_weight': 'balanced', 'coef0': 0.08285683438096408, 'degree': 2, 'gamma': 'auto'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 26.972626232440984, 'class_weight': 'balanced', 'coef0': 0.08285683438096408, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0.8431372549019608</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.8686868686868686</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0.8896604938271604</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.8068924539512775</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0.7997685185185186</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="M104" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0.7450980392156864</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0.9158249158249159</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0.9417989417989417</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0.9270833333333334</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0.9343832020997376</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0.9550843253968253</v>
+      </c>
+      <c r="T104" t="n">
+        <v>0.9085061550404792</v>
+      </c>
+      <c r="U104" t="n">
+        <v>0.9111607142857143</v>
+      </c>
+      <c r="V104" t="n">
+        <v>0.8703703703703703</v>
+      </c>
+      <c r="W104" t="n">
+        <v>0.8952380952380953</v>
+      </c>
+      <c r="X104" t="n">
+        <v>0.8826291079812207</v>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>0.04044198989868164, 0.03241443634033203, 0.05623126029968262, 0.03369283676147461, 0.03164029121398926, 0.03268027305603027, 0.03355598449707031</t>
+        </is>
+      </c>
+      <c r="Z104" t="n">
+        <v>0.03723672458103725</v>
+      </c>
+      <c r="AA104" t="n">
+        <v>0.03355598449707031</v>
+      </c>
+      <c r="AB104" t="n">
+        <v>0.008215915583920414</v>
+      </c>
+      <c r="AC104" t="inlineStr">
+        <is>
+          <t>0.018276453018188477, 0.014851808547973633, 0.015522956848144531, 0.014258384704589844, 0.01596808433532715, 0.0160367488861084, 0.015537023544311523</t>
+        </is>
+      </c>
+      <c r="AD104" t="n">
+        <v>0.01577877998352051</v>
+      </c>
+      <c r="AE104" t="n">
+        <v>0.01553702354431152</v>
+      </c>
+      <c r="AF104" t="n">
+        <v>0.001173244839837054</v>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>0.9259259259259259, 0.7924528301886793, 0.9056603773584906, 0.8679245283018868, 0.9056603773584906, 0.8679245283018868, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="AH104" t="inlineStr">
+        <is>
+          <t>0.9067669172932331, 0.8023809523809524, 0.914860681114551, 0.8738390092879257, 0.903250773993808, 0.8738390092879257, 0.8738390092879257</t>
+        </is>
+      </c>
+      <c r="AI104" t="n">
+        <v>0.8783966218066173</v>
+      </c>
+      <c r="AJ104" t="n">
+        <v>0.8738390092879257</v>
+      </c>
+      <c r="AK104" t="n">
+        <v>0.03503656796221832</v>
+      </c>
+      <c r="AL104" t="n">
+        <v>0.8762104422481781</v>
+      </c>
+      <c r="AM104" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="AN104" t="n">
+        <v>0.04040426667887082</v>
+      </c>
+      <c r="AO104" t="inlineStr">
+        <is>
+          <t>0.9444444444444445, 0.8307692307692307, 0.923076923076923, 0.8923076923076922, 0.9253731343283583, 0.8923076923076922, 0.8923076923076922</t>
+        </is>
+      </c>
+      <c r="AP104" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7317073170731708, 0.8780487804878049, 0.8292682926829269, 0.8717948717948718, 0.8292682926829269, 0.8292682926829269</t>
+        </is>
+      </c>
+      <c r="AQ104" t="n">
+        <v>0.836892105184788</v>
+      </c>
+      <c r="AR104" t="n">
+        <v>0.8292682926829269</v>
+      </c>
+      <c r="AS104" t="n">
+        <v>0.0490683892365447</v>
+      </c>
+      <c r="AT104" t="inlineStr">
+        <is>
+          <t>0.9166666666666667, 0.7812382739212007, 0.900562851782364, 0.8607879924953096, 0.898584003061615, 0.8607879924953096, 0.8607879924953096</t>
+        </is>
+      </c>
+      <c r="AU104" t="n">
+        <v>0.8684879675596822</v>
+      </c>
+      <c r="AV104" t="n">
+        <v>0.8607879924953096</v>
+      </c>
+      <c r="AW104" t="n">
+        <v>0.04148344676142891</v>
+      </c>
+      <c r="AX104" t="n">
+        <v>0.9000838299345764</v>
+      </c>
+      <c r="AY104" t="n">
+        <v>0.8923076923076922</v>
+      </c>
+      <c r="AZ104" t="n">
+        <v>0.03406299620932701</v>
+      </c>
+      <c r="BA104" t="inlineStr">
+        <is>
+          <t>0.918918918918919, 0.9, 0.967741935483871, 0.9354838709677419, 0.9393939393939394, 0.9354838709677419, 0.9354838709677419</t>
+        </is>
+      </c>
+      <c r="BB104" t="inlineStr">
+        <is>
+          <t>0.9411764705882353, 0.6521739130434783, 0.8181818181818182, 0.7727272727272727, 0.85, 0.7727272727272727, 0.7727272727272727</t>
+        </is>
+      </c>
+      <c r="BC104" t="n">
+        <v>0.7971020028564785</v>
+      </c>
+      <c r="BD104" t="n">
+        <v>0.7727272727272727</v>
+      </c>
+      <c r="BE104" t="n">
+        <v>0.08175446042143104</v>
+      </c>
+      <c r="BF104" t="n">
+        <v>0.9332152009571365</v>
+      </c>
+      <c r="BG104" t="n">
+        <v>0.9354838709677419</v>
+      </c>
+      <c r="BH104" t="n">
+        <v>0.0190987884856617</v>
+      </c>
+      <c r="BI104" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.7714285714285715, 0.8823529411764706, 0.8529411764705882, 0.9117647058823529, 0.8529411764705882, 0.8529411764705882</t>
+        </is>
+      </c>
+      <c r="BJ104" t="inlineStr">
+        <is>
+          <t>0.8421052631578947, 0.8333333333333334, 0.9473684210526315, 0.8947368421052632, 0.8947368421052632, 0.8947368421052632, 0.8947368421052632</t>
+        </is>
+      </c>
+      <c r="BK104" t="n">
+        <v>0.8859649122807017</v>
+      </c>
+      <c r="BL104" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM104" t="n">
+        <v>0.03539961627023943</v>
+      </c>
+      <c r="BN104" t="n">
+        <v>0.870828331332533</v>
+      </c>
+      <c r="BO104" t="n">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="BP104" t="n">
+        <v>0.05703279119049408</v>
+      </c>
+      <c r="BQ104" t="inlineStr">
+        <is>
+          <t>0.981954887218045, 0.8682539682539683, 0.9489164086687307, 0.9272445820433437, 0.978328173374613, 0.9272445820433437, 0.9164086687306501</t>
+        </is>
+      </c>
+      <c r="BR104" t="n">
+        <v>0.9354787529046708</v>
+      </c>
+      <c r="BS104" t="n">
+        <v>0.9272445820433437</v>
+      </c>
+      <c r="BT104" t="n">
+        <v>0.03624345735842283</v>
+      </c>
+      <c r="BU104" t="inlineStr">
+        <is>
+          <t>0.889937106918239, 0.9153605015673981, 0.9184952978056427, 0.8996865203761756, 0.9090909090909091, 0.9153605015673981, 0.9059561128526645</t>
+        </is>
+      </c>
+      <c r="BV104" t="inlineStr">
+        <is>
+          <t>0.896762357004101, 0.9166238767650834, 0.9189148552281123, 0.9023541541369533, 0.9096357075350117, 0.9184852650571356, 0.9132013059541197</t>
+        </is>
+      </c>
+      <c r="BW104" t="n">
+        <v>0.9108539316686454</v>
+      </c>
+      <c r="BX104" t="n">
+        <v>0.9132013059541197</v>
+      </c>
+      <c r="BY104" t="n">
+        <v>0.0078769186780503</v>
+      </c>
+      <c r="BZ104" t="n">
+        <v>0.9076981357397752</v>
+      </c>
+      <c r="CA104" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="CB104" t="n">
+        <v>0.009400737020573018</v>
+      </c>
+      <c r="CC104" t="inlineStr">
+        <is>
+          <t>0.9109414758269719, 0.9326683291770573, 0.9356435643564357, 0.92, 0.9280397022332506, 0.9326683291770576, 0.9242424242424243</t>
+        </is>
+      </c>
+      <c r="CD104" t="inlineStr">
+        <is>
+          <t>0.8559670781893004, 0.8860759493670887, 0.888888888888889, 0.8655462184873949, 0.8765957446808511, 0.8860759493670886, 0.8760330578512397</t>
+        </is>
+      </c>
+      <c r="CE104" t="n">
+        <v>0.8764546981188361</v>
+      </c>
+      <c r="CF104" t="n">
+        <v>0.8765957446808511</v>
+      </c>
+      <c r="CG104" t="n">
+        <v>0.01120383368166361</v>
+      </c>
+      <c r="CH104" t="inlineStr">
+        <is>
+          <t>0.8834542770081362, 0.909372139272073, 0.9122662266226623, 0.8927731092436975, 0.9023177234570509, 0.909372139272073, 0.9001377410468321</t>
+        </is>
+      </c>
+      <c r="CI104" t="n">
+        <v>0.9013847651317892</v>
+      </c>
+      <c r="CJ104" t="n">
+        <v>0.9023177234570509</v>
+      </c>
+      <c r="CK104" t="n">
+        <v>0.009592340674305954</v>
+      </c>
+      <c r="CL104" t="n">
+        <v>0.9263148321447426</v>
+      </c>
+      <c r="CM104" t="n">
+        <v>0.9280397022332506</v>
+      </c>
+      <c r="CN104" t="n">
+        <v>0.008028932810974334</v>
+      </c>
+      <c r="CO104" t="inlineStr">
+        <is>
+          <t>0.9521276595744681, 0.9540816326530612, 0.9545454545454546, 0.9484536082474226, 0.949238578680203, 0.958974358974359, 0.9631578947368421</t>
+        </is>
+      </c>
+      <c r="CP104" t="inlineStr">
+        <is>
+          <t>0.8, 0.8536585365853658, 0.859504132231405, 0.824, 0.8442622950819673, 0.8467741935483871, 0.8217054263565892</t>
+        </is>
+      </c>
+      <c r="CQ104" t="n">
+        <v>0.8357006548291021</v>
+      </c>
+      <c r="CR104" t="n">
+        <v>0.8442622950819673</v>
+      </c>
+      <c r="CS104" t="n">
+        <v>0.01961167471487764</v>
+      </c>
+      <c r="CT104" t="n">
+        <v>0.9543684553445443</v>
+      </c>
+      <c r="CU104" t="n">
+        <v>0.9540816326530612</v>
+      </c>
+      <c r="CV104" t="n">
+        <v>0.004853634948724548</v>
+      </c>
+      <c r="CW104" t="inlineStr">
+        <is>
+          <t>0.8731707317073171, 0.9121951219512195, 0.9174757281553398, 0.8932038834951457, 0.9077669902912622, 0.9077669902912622, 0.8883495145631068</t>
+        </is>
+      </c>
+      <c r="CX104" t="inlineStr">
+        <is>
+          <t>0.9203539823008849, 0.9210526315789473, 0.9203539823008849, 0.911504424778761, 0.911504424778761, 0.9292035398230089, 0.9380530973451328</t>
+        </is>
+      </c>
+      <c r="CY104" t="n">
+        <v>0.9217180118437688</v>
+      </c>
+      <c r="CZ104" t="n">
+        <v>0.9203539823008849</v>
+      </c>
+      <c r="DA104" t="n">
+        <v>0.008747789541350907</v>
+      </c>
+      <c r="DB104" t="n">
+        <v>0.8999898514935218</v>
+      </c>
+      <c r="DC104" t="n">
+        <v>0.9077669902912622</v>
+      </c>
+      <c r="DD104" t="n">
+        <v>0.01452340120028887</v>
+      </c>
+      <c r="DE104" t="inlineStr">
+        <is>
+          <t>0.9524498165335635, 0.9647411210954215, 0.958866741128963, 0.9633774379242203, 0.9531961508720681, 0.967007474868975, 0.9659979379671794</t>
+        </is>
+      </c>
+      <c r="DF104" t="n">
+        <v>0.9608052400557702</v>
+      </c>
+      <c r="DG104" t="n">
+        <v>0.9633774379242203</v>
+      </c>
+      <c r="DH104" t="n">
+        <v>0.005593469511598041</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>SVC_no_fragmentation_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 27.620566418088167, 'class_weight': 'balanced', 'coef0': 0.48744430071806377, 'degree': 2, 'gamma': 'auto'}, 'base_estimator_params': {'probability': True, 'kernel': 'poly', 'C': 27.620566418088167, 'class_weight': 'balanced', 'coef0': 0.48744430071806377, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H105" t="n">
+        <v>0.8000000000000002</v>
+      </c>
+      <c r="I105" t="n">
+        <v>0.9190909090909092</v>
+      </c>
+      <c r="J105" t="n">
+        <v>0.8636363636363638</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0.8636363636363636</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.9272727272727272</v>
+      </c>
+      <c r="M105" t="n">
+        <v>0.9272727272727272</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0.9272727272727272</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0.9292929292929293</v>
+      </c>
+      <c r="P105" t="n">
+        <v>0.8372093023255814</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0.9113924050632911</v>
+      </c>
+      <c r="R105" t="n">
+        <v>0.8727272727272727</v>
+      </c>
+      <c r="S105" t="n">
+        <v>0.9693996051561956</v>
+      </c>
+      <c r="T105" t="n">
+        <v>0.9118881118881119</v>
+      </c>
+      <c r="U105" t="n">
+        <v>0.9235861107885264</v>
+      </c>
+      <c r="V105" t="n">
+        <v>0.966824644549763</v>
+      </c>
+      <c r="W105" t="n">
+        <v>0.9357798165137615</v>
+      </c>
+      <c r="X105" t="n">
+        <v>0.951048951048951</v>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>0.0368349552154541, 0.030502796173095703, 0.03272080421447754, 0.031003713607788086, 0.03106212615966797, 0.03137636184692383, 0.03338742256164551</t>
+        </is>
+      </c>
+      <c r="Z105" t="n">
+        <v>0.03241259711129325</v>
+      </c>
+      <c r="AA105" t="n">
+        <v>0.03137636184692383</v>
+      </c>
+      <c r="AB105" t="n">
+        <v>0.002040041146043053</v>
+      </c>
+      <c r="AC105" t="inlineStr">
+        <is>
+          <t>0.014758110046386719, 0.013398408889770508, 0.013259649276733398, 0.012997627258300781, 0.014047861099243164, 0.015001535415649414, 0.012931108474731445</t>
+        </is>
+      </c>
+      <c r="AD105" t="n">
+        <v>0.01377061435154506</v>
+      </c>
+      <c r="AE105" t="n">
+        <v>0.01339840888977051</v>
+      </c>
+      <c r="AF105" t="n">
+        <v>0.0007809409662593594</v>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.7924528301886793, 0.9622641509433962, 0.9245283018867925, 0.9245283018867925, 0.9056603773584906, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="AH105" t="inlineStr">
+        <is>
+          <t>0.9025641025641026, 0.7902930402930403, 0.9514652014652014, 0.9487179487179487, 0.9029304029304028, 0.8901098901098901, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="AI105" t="n">
+        <v>0.9049712192569336</v>
+      </c>
+      <c r="AJ105" t="n">
+        <v>0.9029304029304028</v>
+      </c>
+      <c r="AK105" t="n">
+        <v>0.05260519533712055</v>
+      </c>
+      <c r="AL105" t="n">
+        <v>0.9032644504342617</v>
+      </c>
+      <c r="AM105" t="n">
+        <v>0.9245283018867925</v>
+      </c>
+      <c r="AN105" t="n">
+        <v>0.04975515940651736</v>
+      </c>
+      <c r="AO105" t="inlineStr">
+        <is>
+          <t>0.8235294117647058, 0.6666666666666667, 0.9285714285714286, 0.8750000000000001, 0.8571428571428571, 0.8275862068965518, 0.8750000000000001</t>
+        </is>
+      </c>
+      <c r="AP105" t="inlineStr">
+        <is>
+          <t>0.9189189189189189, 0.8493150684931507, 0.9743589743589743, 0.945945945945946, 0.9487179487179487, 0.935064935064935, 0.945945945945946</t>
+        </is>
+      </c>
+      <c r="AQ105" t="n">
+        <v>0.9311811053494028</v>
+      </c>
+      <c r="AR105" t="n">
+        <v>0.9459459459459461</v>
+      </c>
+      <c r="AS105" t="n">
+        <v>0.03679162098531152</v>
+      </c>
+      <c r="AT105" t="inlineStr">
+        <is>
+          <t>0.8712241653418124, 0.7579908675799087, 0.9514652014652014, 0.910472972972973, 0.9029304029304028, 0.8813255709807435, 0.910472972972973</t>
+        </is>
+      </c>
+      <c r="AU105" t="n">
+        <v>0.8836974506062879</v>
+      </c>
+      <c r="AV105" t="n">
+        <v>0.9029304029304028</v>
+      </c>
+      <c r="AW105" t="n">
+        <v>0.05651748829472441</v>
+      </c>
+      <c r="AX105" t="n">
+        <v>0.8362137958631728</v>
+      </c>
+      <c r="AY105" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="AZ105" t="n">
+        <v>0.07649300163910447</v>
+      </c>
+      <c r="BA105" t="inlineStr">
+        <is>
+          <t>0.7368421052631579, 0.5789473684210527, 0.9285714285714286, 0.7777777777777778, 0.8571428571428571, 0.8, 0.7777777777777778</t>
+        </is>
+      </c>
+      <c r="BB105" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.9117647058823529, 0.9743589743589743, 1.0, 0.9487179487179487, 0.9473684210526315, 1.0</t>
+        </is>
+      </c>
+      <c r="BC105" t="n">
+        <v>0.9648055173486398</v>
+      </c>
+      <c r="BD105" t="n">
+        <v>0.9714285714285714</v>
+      </c>
+      <c r="BE105" t="n">
+        <v>0.02924924047139258</v>
+      </c>
+      <c r="BF105" t="n">
+        <v>0.7795799021362931</v>
+      </c>
+      <c r="BG105" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="BH105" t="n">
+        <v>0.1005114744739972</v>
+      </c>
+      <c r="BI105" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.7857142857142857, 0.9285714285714286, 1.0, 0.8571428571428571, 0.8571428571428571, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ105" t="inlineStr">
+        <is>
+          <t>0.8717948717948718, 0.7948717948717948, 0.9743589743589743, 0.8974358974358975, 0.9487179487179487, 0.9230769230769231, 0.8974358974358975</t>
+        </is>
+      </c>
+      <c r="BK105" t="n">
+        <v>0.9010989010989012</v>
+      </c>
+      <c r="BL105" t="n">
+        <v>0.8974358974358975</v>
+      </c>
+      <c r="BM105" t="n">
+        <v>0.05383493940182809</v>
+      </c>
+      <c r="BN105" t="n">
+        <v>0.9088435374149659</v>
+      </c>
+      <c r="BO105" t="n">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="BP105" t="n">
+        <v>0.073789928117601</v>
+      </c>
+      <c r="BQ105" t="inlineStr">
+        <is>
+          <t>0.9743589743589743, 0.9029304029304029, 0.9725274725274725, 0.9560439560439561, 0.9358974358974359, 0.9542124542124542, 0.9835164835164835</t>
+        </is>
+      </c>
+      <c r="BR105" t="n">
+        <v>0.9542124542124543</v>
+      </c>
+      <c r="BS105" t="n">
+        <v>0.9560439560439561</v>
+      </c>
+      <c r="BT105" t="n">
+        <v>0.02554741077704686</v>
+      </c>
+      <c r="BU105" t="inlineStr">
+        <is>
+          <t>0.9119496855345912, 0.9247648902821317, 0.8996865203761756, 0.9028213166144201, 0.9184952978056427, 0.9090909090909091, 0.9059561128526645</t>
+        </is>
+      </c>
+      <c r="BV105" t="inlineStr">
+        <is>
+          <t>0.924908424908425, 0.9262443438914028, 0.9166415284062343, 0.9150326797385621, 0.9182252388134741, 0.9267973856209151, 0.91342383107089</t>
+        </is>
+      </c>
+      <c r="BW105" t="n">
+        <v>0.9201819189214148</v>
+      </c>
+      <c r="BX105" t="n">
+        <v>0.9182252388134741</v>
+      </c>
+      <c r="BY105" t="n">
+        <v>0.005229130392284604</v>
+      </c>
+      <c r="BZ105" t="n">
+        <v>0.9103949617937906</v>
+      </c>
+      <c r="CA105" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="CB105" t="n">
+        <v>0.008176291566357985</v>
+      </c>
+      <c r="CC105" t="inlineStr">
+        <is>
+          <t>0.8510638297872339, 0.868131868131868, 0.8350515463917525, 0.837696335078534, 0.8571428571428571, 0.8497409326424871, 0.8404255319148938</t>
+        </is>
+      </c>
+      <c r="CD105" t="inlineStr">
+        <is>
+          <t>0.9375, 0.9473684210526315, 0.9279279279279279, 0.9306487695749441, 0.9429824561403509, 0.9348314606741573, 0.9333333333333333</t>
+        </is>
+      </c>
+      <c r="CE105" t="n">
+        <v>0.9363703383861922</v>
+      </c>
+      <c r="CF105" t="n">
+        <v>0.9348314606741573</v>
+      </c>
+      <c r="CG105" t="n">
+        <v>0.006342106986593089</v>
+      </c>
+      <c r="CH105" t="inlineStr">
+        <is>
+          <t>0.894281914893617, 0.9077501445922498, 0.8814897371598402, 0.8841725523267391, 0.900062656641604, 0.8922861966583222, 0.8868794326241136</t>
+        </is>
+      </c>
+      <c r="CI105" t="n">
+        <v>0.8924175192709266</v>
+      </c>
+      <c r="CJ105" t="n">
+        <v>0.8922861966583222</v>
+      </c>
+      <c r="CK105" t="n">
+        <v>0.008578187011358099</v>
+      </c>
+      <c r="CL105" t="n">
+        <v>0.848464700155661</v>
+      </c>
+      <c r="CM105" t="n">
+        <v>0.8497409326424871</v>
+      </c>
+      <c r="CN105" t="n">
+        <v>0.01089554794683732</v>
+      </c>
+      <c r="CO105" t="inlineStr">
+        <is>
+          <t>0.7692307692307693, 0.8144329896907216, 0.7431192660550459, 0.7547169811320755, 0.8041237113402062, 0.7592592592592593, 0.7669902912621359</t>
+        </is>
+      </c>
+      <c r="CP105" t="inlineStr">
+        <is>
+          <t>0.9813084112149533, 0.972972972972973, 0.9809523809523809, 0.9765258215962441, 0.9684684684684685, 0.985781990521327, 0.9722222222222222</t>
+        </is>
+      </c>
+      <c r="CQ105" t="n">
+        <v>0.9768903239926526</v>
+      </c>
+      <c r="CR105" t="n">
+        <v>0.9765258215962441</v>
+      </c>
+      <c r="CS105" t="n">
+        <v>0.005647741150517996</v>
+      </c>
+      <c r="CT105" t="n">
+        <v>0.7731247525671734</v>
+      </c>
+      <c r="CU105" t="n">
+        <v>0.7669902912621359</v>
+      </c>
+      <c r="CV105" t="n">
+        <v>0.02435313941540409</v>
+      </c>
+      <c r="CW105" t="inlineStr">
+        <is>
+          <t>0.9523809523809523, 0.9294117647058824, 0.9529411764705882, 0.9411764705882353, 0.9176470588235294, 0.9647058823529412, 0.9294117647058824</t>
+        </is>
+      </c>
+      <c r="CX105" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.9230769230769231, 0.8803418803418803, 0.8888888888888888, 0.9188034188034188, 0.8888888888888888, 0.8974358974358975</t>
+        </is>
+      </c>
+      <c r="CY105" t="n">
+        <v>0.8992673992673994</v>
+      </c>
+      <c r="CZ105" t="n">
+        <v>0.8974358974358975</v>
+      </c>
+      <c r="DA105" t="n">
+        <v>0.01477865499012237</v>
+      </c>
+      <c r="DB105" t="n">
+        <v>0.9410964385754302</v>
+      </c>
+      <c r="DC105" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="DD105" t="n">
+        <v>0.01534362094470151</v>
+      </c>
+      <c r="DE105" t="inlineStr">
+        <is>
+          <t>0.9712047212047212, 0.9768225238813475, 0.9673705379587731, 0.9739064856711916, 0.966365007541478, 0.9755153343388637, 0.9682755153343389</t>
+        </is>
+      </c>
+      <c r="DF105" t="n">
+        <v>0.9713514465615306</v>
+      </c>
+      <c r="DG105" t="n">
+        <v>0.9712047212047212</v>
+      </c>
+      <c r="DH105" t="n">
+        <v>0.003854384552734193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] Notebooks for ensembles optimisation for default SMOTE[NC]
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4.xlsx
+++ b/results/metrics_modelling4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vulf/Git/Hub/Drop_wall_impact/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E75BC0-FE5C-6D41-A0F5-54B43863D988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41A0F1E-4A10-6649-89DA-597B4D155740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5596,6 +5596,9 @@
     <t>LogisticRegression_splashing_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.552828000398145, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.010000228881835938, 0.009027719497680664, 0.007972478866577148, 0.008032798767089844, 0.00700831413269043, 0.0070002079010009766, 0.0069963932037353516</t>
   </si>
   <si>
@@ -5665,6 +5668,9 @@
     <t>LogisticRegression_no_fragmentation_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 3.6236985622991797, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.00800013542175293, 0.0069997310638427734, 0.0069997310638427734, 0.006999969482421875, 0.007001161575317383, 0.007002353668212891, 0.008000850677490234</t>
   </si>
   <si>
@@ -5731,6 +5737,9 @@
     <t>KNeighborsClassifier_splashing_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'distance', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.010028839111328125, 0.006996870040893555, 0.006000995635986328, 0.006015300750732422, 0.006010293960571289, 0.0059702396392822266, 0.006994485855102539</t>
   </si>
   <si>
@@ -5788,6 +5797,9 @@
     <t>KNeighborsClassifier_no_fragmentation_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 5, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.008001327514648438, 0.00699925422668457, 0.004000425338745117, 0.00500178337097168, 0.005002498626708984, 0.006001710891723633, 0.004999876022338867</t>
   </si>
   <si>
@@ -5827,6 +5839,9 @@
     <t>SVC_splashing_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 18.041415988066607, 'class_weight': None, 'coef0': 0.06653734510998605, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.03385305404663086, 0.016930818557739258, 0.015964508056640625, 0.018526554107666016, 0.016786813735961914, 0.014027833938598633, 0.014509916305541992</t>
   </si>
   <si>
@@ -5896,6 +5911,9 @@
     <t>SVC_no_fragmentation_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 5.737910803667096, 'class_weight': None, 'coef0': 0.8535469624679377, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.012425422668457031, 0.009999275207519531, 0.010129451751708984, 0.010998725891113281, 0.011511564254760742, 0.011305809020996094, 0.011202335357666016</t>
   </si>
   <si>
@@ -5965,6 +5983,9 @@
     <t>LogisticRegression_splashing_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 0.47129737561107793, 'class_weight': None, 'penalty': 'l2'}, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.011999845504760742, 0.011874675750732422, 0.011998891830444336, 0.011457443237304688, 0.010410308837890625, 0.01091313362121582, 0.01103830337524414</t>
   </si>
   <si>
@@ -6031,6 +6052,9 @@
     <t>LogisticRegression_no_fragmentation_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'newton-cholesky', 'C': 6.5706235157060515, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.009731769561767578, 0.010012388229370117, 0.009104728698730469, 0.009039163589477539, 0.010002613067626953, 0.008647680282592773, 0.008929014205932617</t>
   </si>
   <si>
@@ -6100,6 +6124,9 @@
     <t>KNeighborsClassifier_splashing_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 2, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.011987924575805664, 0.009905338287353516, 0.008966207504272461, 0.009542465209960938, 0.009782791137695312, 0.009510040283203125, 0.009002685546875</t>
   </si>
   <si>
@@ -6139,6 +6166,9 @@
     <t>KNeighborsClassifier_no_fragmentation_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.010000467300415039, 0.008997917175292969, 0.008598804473876953, 0.007999181747436523, 0.009029865264892578, 0.007953166961669922, 0.0070002079010009766</t>
   </si>
   <si>
@@ -6208,6 +6238,9 @@
     <t>SVC_splashing_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 8.080278139769582, 'class_weight': 'balanced', 'coef0': 0.48875906950513137, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.019130468368530273, 0.017958402633666992, 0.01714777946472168, 0.0182952880859375, 0.0179290771484375, 0.01857900619506836, 0.016715526580810547</t>
   </si>
   <si>
@@ -6277,6 +6310,9 @@
     <t>SVC_no_fragmentation_smote_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 28.682610859801468, 'class_weight': None, 'coef0': 0.49963292619423594, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.022585391998291016, 0.019678592681884766, 0.018721342086791992, 0.019030094146728516, 0.021327733993530273, 0.01943683624267578, 0.018349647521972656</t>
   </si>
   <si>
@@ -6346,6 +6382,9 @@
     <t>LogisticRegression_splashing_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.15947545233607524, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.025205612182617188, 0.02387094497680664, 0.023152828216552734, 0.022998571395874023, 0.022031307220458984, 0.02233409881591797, 0.02214360237121582</t>
   </si>
   <si>
@@ -6415,6 +6454,9 @@
     <t>LogisticRegression_no_fragmentation_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'liblinear', 'C': 377.1313111077982, 'class_weight': None, 'penalty': 'l1'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.024035215377807617, 0.020569324493408203, 0.02002739906311035, 0.021613359451293945, 0.021079540252685547, 0.021424055099487305, 0.02055525779724121</t>
   </si>
   <si>
@@ -6451,6 +6493,9 @@
     <t>KNeighborsClassifier_splashing_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 1, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.026993751525878906, 0.020168304443359375, 0.019930124282836914, 0.02133655548095703, 0.020959138870239258, 0.021331071853637695, 0.02089977264404297</t>
   </si>
   <si>
@@ -6511,6 +6556,9 @@
     <t>KNeighborsClassifier_no_fragmentation_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.024509429931640625, 0.020848751068115234, 0.020676612854003906, 0.01972341537475586, 0.019952058792114258, 0.021252870559692383, 0.020036697387695312</t>
   </si>
   <si>
@@ -6580,6 +6628,9 @@
     <t>SVC_splashing_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 26.972626232440984, 'class_weight': 'balanced', 'coef0': 0.08285683438096408, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.04044198989868164, 0.03241443634033203, 0.05623126029968262, 0.03369283676147461, 0.03164029121398926, 0.03268027305603027, 0.03355598449707031</t>
   </si>
   <si>
@@ -6649,6 +6700,9 @@
     <t>SVC_no_fragmentation_smotenc_opt-model</t>
   </si>
   <si>
+    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 27.620566418088167, 'class_weight': 'balanced', 'coef0': 0.48744430071806377, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+  </si>
+  <si>
     <t>0.0368349552154541, 0.030502796173095703, 0.03272080421447754, 0.031003713607788086, 0.03106212615966797, 0.03137636184692383, 0.03338742256164551</t>
   </si>
   <si>
@@ -6713,60 +6767,6 @@
   </si>
   <si>
     <t>0.9712047212047212, 0.9768225238813475, 0.9673705379587731, 0.9739064856711916, 0.966365007541478, 0.9755153343388637, 0.9682755153343389</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.552828000398145, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 3.6236985622991797, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 27.620566418088167, 'class_weight': 'balanced', 'coef0': 0.48744430071806377, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 26.972626232440984, 'class_weight': 'balanced', 'coef0': 0.08285683438096408, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 1, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'liblinear', 'C': 377.1313111077982, 'class_weight': None, 'penalty': 'l1'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'sag', 'C': 0.15947545233607524, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 28.682610859801468, 'class_weight': None, 'coef0': 0.49963292619423594, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 8.080278139769582, 'class_weight': 'balanced', 'coef0': 0.48875906950513137, 'degree': 2, 'gamma': 'auto'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'uniform', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 2, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'newton-cholesky', 'C': 6.5706235157060515, 'class_weight': 'balanced', 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'LogisticRegression', 'estimator_params': {'fit_intercept': False, 'max_iter': 1000, 'solver': 'lbfgs', 'C': 0.47129737561107793, 'class_weight': None, 'penalty': 'l2'}, 'class_weight': None, 'penalty': 'l2'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 5.737910803667096, 'class_weight': None, 'coef0': 0.8535469624679377, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'SVC', 'estimator_params': {'probability': True, 'kernel': 'poly', 'C': 18.041415988066607, 'class_weight': None, 'coef0': 0.06653734510998605, 'degree': 2, 'gamma': 'scale'}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 3, 'weights': 'distance', 'p': 2}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
-  </si>
-  <si>
-    <t>{'estimator': 'KNeighborsClassifier', 'estimator_params': {'n_neighbors': 5, 'weights': 'distance', 'p': 1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': False, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
   </si>
 </sst>
 </file>
@@ -36550,7 +36550,7 @@
         <v>1857</v>
       </c>
       <c r="D88" t="s">
-        <v>2231</v>
+        <v>1858</v>
       </c>
       <c r="E88">
         <v>0.78666666666666663</v>
@@ -36613,7 +36613,7 @@
         <v>0.79668049792531126</v>
       </c>
       <c r="Y88" t="s">
-        <v>1858</v>
+        <v>1859</v>
       </c>
       <c r="Z88">
         <v>8.0054487500871938E-3</v>
@@ -36625,7 +36625,7 @@
         <v>1.0723139197588111E-3</v>
       </c>
       <c r="AC88" t="s">
-        <v>1859</v>
+        <v>1860</v>
       </c>
       <c r="AD88">
         <v>1.646113395690918E-2</v>
@@ -36637,10 +36637,10 @@
         <v>1.56083659277844E-3</v>
       </c>
       <c r="AG88" t="s">
-        <v>1860</v>
+        <v>1861</v>
       </c>
       <c r="AH88" t="s">
-        <v>1861</v>
+        <v>1862</v>
       </c>
       <c r="AI88">
         <v>0.82886101809144708</v>
@@ -36661,10 +36661,10 @@
         <v>5.4442024745888183E-2</v>
       </c>
       <c r="AO88" t="s">
-        <v>1862</v>
+        <v>1863</v>
       </c>
       <c r="AP88" t="s">
-        <v>1863</v>
+        <v>1864</v>
       </c>
       <c r="AQ88">
         <v>0.77339474320449408</v>
@@ -36676,7 +36676,7 @@
         <v>6.3445713556925173E-2</v>
       </c>
       <c r="AT88" t="s">
-        <v>1864</v>
+        <v>1865</v>
       </c>
       <c r="AU88">
         <v>0.80948694899938711</v>
@@ -36697,10 +36697,10 @@
         <v>4.8832068757050838E-2</v>
       </c>
       <c r="BA88" t="s">
-        <v>1865</v>
+        <v>1866</v>
       </c>
       <c r="BB88" t="s">
-        <v>1866</v>
+        <v>1867</v>
       </c>
       <c r="BC88">
         <v>0.70034005114423548</v>
@@ -36721,10 +36721,10 @@
         <v>4.0507547092598691E-2</v>
       </c>
       <c r="BI88" t="s">
-        <v>1867</v>
+        <v>1868</v>
       </c>
       <c r="BJ88" t="s">
-        <v>1868</v>
+        <v>1869</v>
       </c>
       <c r="BK88">
         <v>0.87092731829573922</v>
@@ -36745,7 +36745,7 @@
         <v>7.554445485019097E-2</v>
       </c>
       <c r="BQ88" t="s">
-        <v>1869</v>
+        <v>1870</v>
       </c>
       <c r="BR88">
         <v>0.89732243774702858</v>
@@ -36757,10 +36757,10 @@
         <v>4.6350320653201889E-2</v>
       </c>
       <c r="BU88" t="s">
-        <v>1870</v>
+        <v>1871</v>
       </c>
       <c r="BV88" t="s">
-        <v>1871</v>
+        <v>1872</v>
       </c>
       <c r="BW88">
         <v>0.83751604529398749</v>
@@ -36781,10 +36781,10 @@
         <v>9.8321672312090651E-3</v>
       </c>
       <c r="CC88" t="s">
-        <v>1872</v>
+        <v>1873</v>
       </c>
       <c r="CD88" t="s">
-        <v>1873</v>
+        <v>1874</v>
       </c>
       <c r="CE88">
         <v>0.78129343692151554</v>
@@ -36796,7 +36796,7 @@
         <v>9.4179777766895886E-3</v>
       </c>
       <c r="CH88" t="s">
-        <v>1874</v>
+        <v>1875</v>
       </c>
       <c r="CI88">
         <v>0.81755999903193499</v>
@@ -36817,10 +36817,10 @@
         <v>9.6838309101750543E-3</v>
       </c>
       <c r="CO88" t="s">
-        <v>1875</v>
+        <v>1876</v>
       </c>
       <c r="CP88" t="s">
-        <v>1876</v>
+        <v>1877</v>
       </c>
       <c r="CQ88">
         <v>0.70202021846842677</v>
@@ -36841,10 +36841,10 @@
         <v>7.5910311155891466E-3</v>
       </c>
       <c r="CW88" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="CX88" t="s">
-        <v>1878</v>
+        <v>1879</v>
       </c>
       <c r="CY88">
         <v>0.88130725042695235</v>
@@ -36865,7 +36865,7 @@
         <v>1.8071534642519649E-2</v>
       </c>
       <c r="DE88" t="s">
-        <v>1879</v>
+        <v>1880</v>
       </c>
       <c r="DF88">
         <v>0.90969531996605446</v>
@@ -36885,10 +36885,10 @@
         <v>138</v>
       </c>
       <c r="C89" t="s">
-        <v>1880</v>
+        <v>1881</v>
       </c>
       <c r="D89" t="s">
-        <v>2232</v>
+        <v>1882</v>
       </c>
       <c r="E89">
         <v>0.82666666666666666</v>
@@ -36951,7 +36951,7 @@
         <v>0.9033816425120772</v>
       </c>
       <c r="Y89" t="s">
-        <v>1881</v>
+        <v>1883</v>
       </c>
       <c r="Z89">
         <v>7.2862761361258367E-3</v>
@@ -36963,7 +36963,7 @@
         <v>4.5171131619771589E-4</v>
       </c>
       <c r="AC89" t="s">
-        <v>1882</v>
+        <v>1884</v>
       </c>
       <c r="AD89">
         <v>1.3425895145961221E-2</v>
@@ -36975,10 +36975,10 @@
         <v>4.9737836101214968E-4</v>
       </c>
       <c r="AG89" t="s">
-        <v>1883</v>
+        <v>1885</v>
       </c>
       <c r="AH89" t="s">
-        <v>1884</v>
+        <v>1886</v>
       </c>
       <c r="AI89">
         <v>0.8643642072213501</v>
@@ -36999,10 +36999,10 @@
         <v>5.8839094672646551E-2</v>
       </c>
       <c r="AO89" t="s">
-        <v>1885</v>
+        <v>1887</v>
       </c>
       <c r="AP89" t="s">
-        <v>1886</v>
+        <v>1888</v>
       </c>
       <c r="AQ89">
         <v>0.89660790605935159</v>
@@ -37014,7 +37014,7 @@
         <v>4.5344363618053538E-2</v>
       </c>
       <c r="AT89" t="s">
-        <v>1887</v>
+        <v>1889</v>
       </c>
       <c r="AU89">
         <v>0.83279524954828321</v>
@@ -37035,10 +37035,10 @@
         <v>8.2792754002689539E-2</v>
       </c>
       <c r="BA89" t="s">
-        <v>1888</v>
+        <v>1890</v>
       </c>
       <c r="BB89" t="s">
-        <v>1889</v>
+        <v>1891</v>
       </c>
       <c r="BC89">
         <v>0.95093956879671171</v>
@@ -37062,7 +37062,7 @@
         <v>198</v>
       </c>
       <c r="BJ89" t="s">
-        <v>1890</v>
+        <v>1892</v>
       </c>
       <c r="BK89">
         <v>0.84981684981684968</v>
@@ -37083,7 +37083,7 @@
         <v>9.1024373788722357E-2</v>
       </c>
       <c r="BQ89" t="s">
-        <v>1891</v>
+        <v>1893</v>
       </c>
       <c r="BR89">
         <v>0.93521716378859232</v>
@@ -37095,10 +37095,10 @@
         <v>3.6492377948779603E-2</v>
       </c>
       <c r="BU89" t="s">
-        <v>1892</v>
+        <v>1894</v>
       </c>
       <c r="BV89" t="s">
-        <v>1893</v>
+        <v>1895</v>
       </c>
       <c r="BW89">
         <v>0.86560059921404453</v>
@@ -37119,10 +37119,10 @@
         <v>9.6149545162086767E-3</v>
       </c>
       <c r="CC89" t="s">
-        <v>1894</v>
+        <v>1896</v>
       </c>
       <c r="CD89" t="s">
-        <v>1895</v>
+        <v>1897</v>
       </c>
       <c r="CE89">
         <v>0.89966608584924734</v>
@@ -37134,7 +37134,7 @@
         <v>7.0531262209585126E-3</v>
       </c>
       <c r="CH89" t="s">
-        <v>1896</v>
+        <v>1898</v>
       </c>
       <c r="CI89">
         <v>0.83463826574678879</v>
@@ -37155,10 +37155,10 @@
         <v>1.5189692595782581E-2</v>
       </c>
       <c r="CO89" t="s">
-        <v>1897</v>
+        <v>1899</v>
       </c>
       <c r="CP89" t="s">
-        <v>1898</v>
+        <v>1900</v>
       </c>
       <c r="CQ89">
         <v>0.95041134659786153</v>
@@ -37179,10 +37179,10 @@
         <v>1.575385788795243E-2</v>
       </c>
       <c r="CW89" t="s">
-        <v>1899</v>
+        <v>1901</v>
       </c>
       <c r="CX89" t="s">
-        <v>1900</v>
+        <v>1902</v>
       </c>
       <c r="CY89">
         <v>0.85409035409035394</v>
@@ -37203,7 +37203,7 @@
         <v>1.641310052344333E-2</v>
       </c>
       <c r="DE89" t="s">
-        <v>1901</v>
+        <v>1903</v>
       </c>
       <c r="DF89">
         <v>0.93937797341158702</v>
@@ -37223,10 +37223,10 @@
         <v>113</v>
       </c>
       <c r="C90" t="s">
-        <v>1902</v>
+        <v>1904</v>
       </c>
       <c r="D90" t="s">
-        <v>2247</v>
+        <v>1905</v>
       </c>
       <c r="E90">
         <v>0.85333333333333339</v>
@@ -37289,7 +37289,7 @@
         <v>0.99526066350710907</v>
       </c>
       <c r="Y90" t="s">
-        <v>1903</v>
+        <v>1906</v>
       </c>
       <c r="Z90">
         <v>6.8595749991280696E-3</v>
@@ -37301,7 +37301,7 @@
         <v>1.3650452150791559E-3</v>
       </c>
       <c r="AC90" t="s">
-        <v>1904</v>
+        <v>1907</v>
       </c>
       <c r="AD90">
         <v>1.597057070050921E-2</v>
@@ -37313,10 +37313,10 @@
         <v>9.229586112470226E-4</v>
       </c>
       <c r="AG90" t="s">
-        <v>1905</v>
+        <v>1908</v>
       </c>
       <c r="AH90" t="s">
-        <v>1906</v>
+        <v>1909</v>
       </c>
       <c r="AI90">
         <v>0.88584591731429396</v>
@@ -37337,10 +37337,10 @@
         <v>3.1678857770437968E-2</v>
       </c>
       <c r="AO90" t="s">
-        <v>1907</v>
+        <v>1910</v>
       </c>
       <c r="AP90" t="s">
-        <v>1908</v>
+        <v>1911</v>
       </c>
       <c r="AQ90">
         <v>0.85138227503897768</v>
@@ -37352,7 +37352,7 @@
         <v>4.1561792280754919E-2</v>
       </c>
       <c r="AT90" t="s">
-        <v>1909</v>
+        <v>1912</v>
       </c>
       <c r="AU90">
         <v>0.88342827512180488</v>
@@ -37373,10 +37373,10 @@
         <v>2.5532956825800021E-2</v>
       </c>
       <c r="BA90" t="s">
-        <v>1910</v>
+        <v>1913</v>
       </c>
       <c r="BB90" t="s">
-        <v>1911</v>
+        <v>1914</v>
       </c>
       <c r="BC90">
         <v>0.8441119031344595</v>
@@ -37397,10 +37397,10 @@
         <v>2.043371926778044E-2</v>
       </c>
       <c r="BI90" t="s">
-        <v>1912</v>
+        <v>1915</v>
       </c>
       <c r="BJ90" t="s">
-        <v>1913</v>
+        <v>1916</v>
       </c>
       <c r="BK90">
         <v>0.86340852130325807</v>
@@ -37421,7 +37421,7 @@
         <v>4.7036155944005412E-2</v>
       </c>
       <c r="BQ90" t="s">
-        <v>1914</v>
+        <v>1917</v>
       </c>
       <c r="BR90">
         <v>0.92486924594399178</v>
@@ -37436,7 +37436,7 @@
         <v>369</v>
       </c>
       <c r="BV90" t="s">
-        <v>1915</v>
+        <v>1918</v>
       </c>
       <c r="BW90">
         <v>0.99826460539223982</v>
@@ -37457,10 +37457,10 @@
         <v>1.417051170840857E-3</v>
       </c>
       <c r="CC90" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="CD90" t="s">
-        <v>1917</v>
+        <v>1920</v>
       </c>
       <c r="CE90">
         <v>0.99685336689741977</v>
@@ -37472,7 +37472,7 @@
         <v>1.9901055130071761E-3</v>
       </c>
       <c r="CH90" t="s">
-        <v>1918</v>
+        <v>1921</v>
       </c>
       <c r="CI90">
         <v>0.99755687288639661</v>
@@ -37496,7 +37496,7 @@
         <v>375</v>
       </c>
       <c r="CP90" t="s">
-        <v>1919</v>
+        <v>1922</v>
       </c>
       <c r="CQ90">
         <v>0.99373433583959891</v>
@@ -37517,7 +37517,7 @@
         <v>0</v>
       </c>
       <c r="CW90" t="s">
-        <v>1920</v>
+        <v>1923</v>
       </c>
       <c r="CX90" t="s">
         <v>375</v>
@@ -37561,10 +37561,10 @@
         <v>138</v>
       </c>
       <c r="C91" t="s">
-        <v>1921</v>
+        <v>1924</v>
       </c>
       <c r="D91" t="s">
-        <v>2248</v>
+        <v>1925</v>
       </c>
       <c r="E91">
         <v>0.92</v>
@@ -37627,7 +37627,7 @@
         <v>1</v>
       </c>
       <c r="Y91" t="s">
-        <v>1922</v>
+        <v>1926</v>
       </c>
       <c r="Z91">
         <v>5.7152679988316116E-3</v>
@@ -37639,7 +37639,7 @@
         <v>1.277626694582705E-3</v>
       </c>
       <c r="AC91" t="s">
-        <v>1923</v>
+        <v>1927</v>
       </c>
       <c r="AD91">
         <v>1.5026535306658061E-2</v>
@@ -37651,10 +37651,10 @@
         <v>2.1160577179123682E-3</v>
       </c>
       <c r="AG91" t="s">
-        <v>1924</v>
+        <v>1928</v>
       </c>
       <c r="AH91" t="s">
-        <v>1925</v>
+        <v>1929</v>
       </c>
       <c r="AI91">
         <v>0.82697540554683402</v>
@@ -37675,10 +37675,10 @@
         <v>3.1570371855296632E-2</v>
       </c>
       <c r="AO91" t="s">
-        <v>1926</v>
+        <v>1930</v>
       </c>
       <c r="AP91" t="s">
-        <v>1927</v>
+        <v>1931</v>
       </c>
       <c r="AQ91">
         <v>0.91459045625712299</v>
@@ -37690,7 +37690,7 @@
         <v>2.2537737450952271E-2</v>
       </c>
       <c r="AT91" t="s">
-        <v>1928</v>
+        <v>1932</v>
       </c>
       <c r="AU91">
         <v>0.8334743445786138</v>
@@ -37711,10 +37711,10 @@
         <v>6.5039747346654866E-2</v>
       </c>
       <c r="BA91" t="s">
-        <v>1929</v>
+        <v>1933</v>
       </c>
       <c r="BB91" t="s">
-        <v>1930</v>
+        <v>1934</v>
       </c>
       <c r="BC91">
         <v>0.90530303691866132</v>
@@ -37735,10 +37735,10 @@
         <v>0.10228865129620759</v>
       </c>
       <c r="BI91" t="s">
-        <v>1931</v>
+        <v>1935</v>
       </c>
       <c r="BJ91" t="s">
-        <v>1932</v>
+        <v>1936</v>
       </c>
       <c r="BK91">
         <v>0.92673992673992667</v>
@@ -37759,7 +37759,7 @@
         <v>0.10400824410131369</v>
       </c>
       <c r="BQ91" t="s">
-        <v>1933</v>
+        <v>1937</v>
       </c>
       <c r="BR91">
         <v>0.93168498168498182</v>
@@ -37899,10 +37899,10 @@
         <v>113</v>
       </c>
       <c r="C92" t="s">
-        <v>1934</v>
+        <v>1938</v>
       </c>
       <c r="D92" t="s">
-        <v>2246</v>
+        <v>1939</v>
       </c>
       <c r="E92">
         <v>0.84</v>
@@ -37965,7 +37965,7 @@
         <v>0.87081339712918659</v>
       </c>
       <c r="Y92" t="s">
-        <v>1935</v>
+        <v>1940</v>
       </c>
       <c r="Z92">
         <v>1.8657071249825609E-2</v>
@@ -37977,7 +37977,7 @@
         <v>6.3616189333841767E-3</v>
       </c>
       <c r="AC92" t="s">
-        <v>1936</v>
+        <v>1941</v>
       </c>
       <c r="AD92">
         <v>1.7291375568934848E-2</v>
@@ -37989,10 +37989,10 @@
         <v>4.9319890074851968E-3</v>
       </c>
       <c r="AG92" t="s">
-        <v>1937</v>
+        <v>1942</v>
       </c>
       <c r="AH92" t="s">
-        <v>1938</v>
+        <v>1943</v>
       </c>
       <c r="AI92">
         <v>0.86159551539914214</v>
@@ -38013,10 +38013,10 @@
         <v>3.6418220603683812E-2</v>
       </c>
       <c r="AO92" t="s">
-        <v>1939</v>
+        <v>1944</v>
       </c>
       <c r="AP92" t="s">
-        <v>1940</v>
+        <v>1945</v>
       </c>
       <c r="AQ92">
         <v>0.82329995593282934</v>
@@ -38028,7 +38028,7 @@
         <v>5.7501527766802042E-2</v>
       </c>
       <c r="AT92" t="s">
-        <v>1941</v>
+        <v>1946</v>
       </c>
       <c r="AU92">
         <v>0.8654576529983663</v>
@@ -38049,10 +38049,10 @@
         <v>2.7060612692675439E-2</v>
       </c>
       <c r="BA92" t="s">
-        <v>1942</v>
+        <v>1947</v>
       </c>
       <c r="BB92" t="s">
-        <v>1943</v>
+        <v>1948</v>
       </c>
       <c r="BC92">
         <v>0.85034734787056743</v>
@@ -38073,10 +38073,10 @@
         <v>3.7412677092296842E-2</v>
       </c>
       <c r="BI92" t="s">
-        <v>1944</v>
+        <v>1949</v>
       </c>
       <c r="BJ92" t="s">
-        <v>1945</v>
+        <v>1950</v>
       </c>
       <c r="BK92">
         <v>0.80242272347535504</v>
@@ -38097,7 +38097,7 @@
         <v>3.7275634884588717E-2</v>
       </c>
       <c r="BQ92" t="s">
-        <v>1946</v>
+        <v>1951</v>
       </c>
       <c r="BR92">
         <v>0.93525831385185643</v>
@@ -38109,10 +38109,10 @@
         <v>3.5829968492735793E-2</v>
       </c>
       <c r="BU92" t="s">
-        <v>1947</v>
+        <v>1952</v>
       </c>
       <c r="BV92" t="s">
-        <v>1948</v>
+        <v>1953</v>
       </c>
       <c r="BW92">
         <v>0.90049037196752579</v>
@@ -38133,10 +38133,10 @@
         <v>1.023858807929395E-2</v>
       </c>
       <c r="CC92" t="s">
-        <v>1949</v>
+        <v>1954</v>
       </c>
       <c r="CD92" t="s">
-        <v>1950</v>
+        <v>1955</v>
       </c>
       <c r="CE92">
         <v>0.87315400977137847</v>
@@ -38148,7 +38148,7 @@
         <v>1.453673088192685E-2</v>
       </c>
       <c r="CH92" t="s">
-        <v>1951</v>
+        <v>1956</v>
       </c>
       <c r="CI92">
         <v>0.90220448068119097</v>
@@ -38169,10 +38169,10 @@
         <v>7.9116326087036518E-3</v>
       </c>
       <c r="CO92" t="s">
-        <v>1952</v>
+        <v>1957</v>
       </c>
       <c r="CP92" t="s">
-        <v>1953</v>
+        <v>1958</v>
       </c>
       <c r="CQ92">
         <v>0.88163111580542775</v>
@@ -38193,10 +38193,10 @@
         <v>7.5736648416428838E-3</v>
       </c>
       <c r="CW92" t="s">
-        <v>1954</v>
+        <v>1959</v>
       </c>
       <c r="CX92" t="s">
-        <v>1955</v>
+        <v>1960</v>
       </c>
       <c r="CY92">
         <v>0.86487235788586503</v>
@@ -38217,7 +38217,7 @@
         <v>8.814516510296494E-3</v>
       </c>
       <c r="DE92" t="s">
-        <v>1956</v>
+        <v>1961</v>
       </c>
       <c r="DF92">
         <v>0.96498620518971279</v>
@@ -38237,10 +38237,10 @@
         <v>138</v>
       </c>
       <c r="C93" t="s">
-        <v>1957</v>
+        <v>1962</v>
       </c>
       <c r="D93" t="s">
-        <v>2245</v>
+        <v>1963</v>
       </c>
       <c r="E93">
         <v>0.8666666666666667</v>
@@ -38303,7 +38303,7 @@
         <v>0.94883720930232562</v>
       </c>
       <c r="Y93" t="s">
-        <v>1958</v>
+        <v>1964</v>
       </c>
       <c r="Z93">
         <v>1.1081797736031671E-2</v>
@@ -38315,7 +38315,7 @@
         <v>7.6908632468164495E-4</v>
       </c>
       <c r="AC93" t="s">
-        <v>1959</v>
+        <v>1965</v>
       </c>
       <c r="AD93">
         <v>1.463331495012556E-2</v>
@@ -38327,10 +38327,10 @@
         <v>1.312864857834909E-3</v>
       </c>
       <c r="AG93" t="s">
-        <v>1960</v>
+        <v>1966</v>
       </c>
       <c r="AH93" t="s">
-        <v>1961</v>
+        <v>1967</v>
       </c>
       <c r="AI93">
         <v>0.88529565672422816</v>
@@ -38351,10 +38351,10 @@
         <v>5.2308260995201229E-2</v>
       </c>
       <c r="AO93" t="s">
-        <v>1962</v>
+        <v>1968</v>
       </c>
       <c r="AP93" t="s">
-        <v>1963</v>
+        <v>1969</v>
       </c>
       <c r="AQ93">
         <v>0.92857375031163947</v>
@@ -38366,7 +38366,7 @@
         <v>3.8092925665618102E-2</v>
       </c>
       <c r="AT93" t="s">
-        <v>1964</v>
+        <v>1970</v>
       </c>
       <c r="AU93">
         <v>0.87404875049055364</v>
@@ -38387,10 +38387,10 @@
         <v>8.3157645302476865E-2</v>
       </c>
       <c r="BA93" t="s">
-        <v>1965</v>
+        <v>1971</v>
       </c>
       <c r="BB93" t="s">
-        <v>1966</v>
+        <v>1972</v>
       </c>
       <c r="BC93">
         <v>0.94691772868464597</v>
@@ -38411,10 +38411,10 @@
         <v>0.1049407686566827</v>
       </c>
       <c r="BI93" t="s">
-        <v>1967</v>
+        <v>1973</v>
       </c>
       <c r="BJ93" t="s">
-        <v>1968</v>
+        <v>1974</v>
       </c>
       <c r="BK93">
         <v>0.91208791208791218</v>
@@ -38435,7 +38435,7 @@
         <v>8.5438493789503467E-2</v>
       </c>
       <c r="BQ93" t="s">
-        <v>1969</v>
+        <v>1975</v>
       </c>
       <c r="BR93">
         <v>0.95874760160474448</v>
@@ -38447,10 +38447,10 @@
         <v>1.9679551721959721E-2</v>
       </c>
       <c r="BU93" t="s">
-        <v>1970</v>
+        <v>1976</v>
       </c>
       <c r="BV93" t="s">
-        <v>1971</v>
+        <v>1977</v>
       </c>
       <c r="BW93">
         <v>0.90932398600465836</v>
@@ -38471,10 +38471,10 @@
         <v>5.9107130862048112E-3</v>
       </c>
       <c r="CC93" t="s">
-        <v>1972</v>
+        <v>1978</v>
       </c>
       <c r="CD93" t="s">
-        <v>1973</v>
+        <v>1979</v>
       </c>
       <c r="CE93">
         <v>0.94389976755300364</v>
@@ -38486,7 +38486,7 @@
         <v>4.2004318802550322E-3</v>
       </c>
       <c r="CH93" t="s">
-        <v>1974</v>
+        <v>1980</v>
       </c>
       <c r="CI93">
         <v>0.89878501048976223</v>
@@ -38507,10 +38507,10 @@
         <v>1.042945052687042E-2</v>
       </c>
       <c r="CO93" t="s">
-        <v>1975</v>
+        <v>1981</v>
       </c>
       <c r="CP93" t="s">
-        <v>1976</v>
+        <v>1982</v>
       </c>
       <c r="CQ93">
         <v>0.95854807561982036</v>
@@ -38531,10 +38531,10 @@
         <v>1.740622108788583E-2</v>
       </c>
       <c r="CW93" t="s">
-        <v>1977</v>
+        <v>1983</v>
       </c>
       <c r="CX93" t="s">
-        <v>1978</v>
+        <v>1984</v>
       </c>
       <c r="CY93">
         <v>0.92979242979242982</v>
@@ -38555,7 +38555,7 @@
         <v>1.9955734046635809E-2</v>
       </c>
       <c r="DE93" t="s">
-        <v>1979</v>
+        <v>1985</v>
       </c>
       <c r="DF93">
         <v>0.97052735624164199</v>
@@ -38575,10 +38575,10 @@
         <v>113</v>
       </c>
       <c r="C94" t="s">
-        <v>1980</v>
+        <v>1986</v>
       </c>
       <c r="D94" t="s">
-        <v>2244</v>
+        <v>1987</v>
       </c>
       <c r="E94">
         <v>0.77333333333333332</v>
@@ -38641,7 +38641,7 @@
         <v>0.8</v>
       </c>
       <c r="Y94" t="s">
-        <v>1981</v>
+        <v>1988</v>
       </c>
       <c r="Z94">
         <v>1.1384657451084679E-2</v>
@@ -38653,7 +38653,7 @@
         <v>5.7231447484966586E-4</v>
       </c>
       <c r="AC94" t="s">
-        <v>1982</v>
+        <v>1989</v>
       </c>
       <c r="AD94">
         <v>1.5223673411778041E-2</v>
@@ -38665,10 +38665,10 @@
         <v>8.97125378465606E-4</v>
       </c>
       <c r="AG94" t="s">
-        <v>1983</v>
+        <v>1990</v>
       </c>
       <c r="AH94" t="s">
-        <v>1984</v>
+        <v>1991</v>
       </c>
       <c r="AI94">
         <v>0.82886101809144708</v>
@@ -38689,10 +38689,10 @@
         <v>4.8514438936045408E-2</v>
       </c>
       <c r="AO94" t="s">
-        <v>1985</v>
+        <v>1992</v>
       </c>
       <c r="AP94" t="s">
-        <v>1986</v>
+        <v>1993</v>
       </c>
       <c r="AQ94">
         <v>0.77317102279508287</v>
@@ -38704,7 +38704,7 @@
         <v>5.6521888218575553E-2</v>
       </c>
       <c r="AT94" t="s">
-        <v>1987</v>
+        <v>1994</v>
       </c>
       <c r="AU94">
         <v>0.80933611177901665</v>
@@ -38725,10 +38725,10 @@
         <v>4.4235689348156623E-2</v>
       </c>
       <c r="BA94" t="s">
-        <v>1988</v>
+        <v>1995</v>
       </c>
       <c r="BB94" t="s">
-        <v>1989</v>
+        <v>1996</v>
       </c>
       <c r="BC94">
         <v>0.70081676654705927</v>
@@ -38752,7 +38752,7 @@
         <v>558</v>
       </c>
       <c r="BJ94" t="s">
-        <v>1990</v>
+        <v>1997</v>
       </c>
       <c r="BK94">
         <v>0.87092731829573933</v>
@@ -38773,7 +38773,7 @@
         <v>7.554445485019097E-2</v>
       </c>
       <c r="BQ94" t="s">
-        <v>1991</v>
+        <v>1998</v>
       </c>
       <c r="BR94">
         <v>0.897734532409455</v>
@@ -38785,10 +38785,10 @@
         <v>4.6250333929565193E-2</v>
       </c>
       <c r="BU94" t="s">
-        <v>1992</v>
+        <v>1999</v>
       </c>
       <c r="BV94" t="s">
-        <v>1993</v>
+        <v>2000</v>
       </c>
       <c r="BW94">
         <v>0.83760621616320907</v>
@@ -38809,10 +38809,10 @@
         <v>8.5821525732836454E-3</v>
       </c>
       <c r="CC94" t="s">
-        <v>1994</v>
+        <v>2001</v>
       </c>
       <c r="CD94" t="s">
-        <v>1995</v>
+        <v>2002</v>
       </c>
       <c r="CE94">
         <v>0.78097349016625317</v>
@@ -38824,7 +38824,7 @@
         <v>6.7801624782986604E-3</v>
       </c>
       <c r="CH94" t="s">
-        <v>1996</v>
+        <v>2003</v>
       </c>
       <c r="CI94">
         <v>0.81652679128772576</v>
@@ -38845,10 +38845,10 @@
         <v>9.0363374342491559E-3</v>
       </c>
       <c r="CO94" t="s">
-        <v>1997</v>
+        <v>2004</v>
       </c>
       <c r="CP94" t="s">
-        <v>1998</v>
+        <v>2005</v>
       </c>
       <c r="CQ94">
         <v>0.69847422693304684</v>
@@ -38869,10 +38869,10 @@
         <v>6.4336214947721578E-3</v>
       </c>
       <c r="CW94" t="s">
-        <v>1999</v>
+        <v>2006</v>
       </c>
       <c r="CX94" t="s">
-        <v>2000</v>
+        <v>2007</v>
       </c>
       <c r="CY94">
         <v>0.88634196109743379</v>
@@ -38893,7 +38893,7 @@
         <v>1.977086446669224E-2</v>
       </c>
       <c r="DE94" t="s">
-        <v>2001</v>
+        <v>2008</v>
       </c>
       <c r="DF94">
         <v>0.91073181214768406</v>
@@ -38913,10 +38913,10 @@
         <v>138</v>
       </c>
       <c r="C95" t="s">
-        <v>2002</v>
+        <v>2009</v>
       </c>
       <c r="D95" t="s">
-        <v>2243</v>
+        <v>2010</v>
       </c>
       <c r="E95">
         <v>0.82666666666666666</v>
@@ -38979,7 +38979,7 @@
         <v>0.875</v>
       </c>
       <c r="Y95" t="s">
-        <v>2003</v>
+        <v>2011</v>
       </c>
       <c r="Z95">
         <v>9.3524796622140062E-3</v>
@@ -38991,7 +38991,7 @@
         <v>5.1236513894784745E-4</v>
       </c>
       <c r="AC95" t="s">
-        <v>2004</v>
+        <v>2012</v>
       </c>
       <c r="AD95">
         <v>1.4224393027169361E-2</v>
@@ -39003,10 +39003,10 @@
         <v>1.1017711288096119E-3</v>
       </c>
       <c r="AG95" t="s">
-        <v>2005</v>
+        <v>2013</v>
       </c>
       <c r="AH95" t="s">
-        <v>2006</v>
+        <v>2014</v>
       </c>
       <c r="AI95">
         <v>0.85408163265306136</v>
@@ -39027,10 +39027,10 @@
         <v>5.3129038015935118E-2</v>
       </c>
       <c r="AO95" t="s">
-        <v>2007</v>
+        <v>2015</v>
       </c>
       <c r="AP95" t="s">
-        <v>2008</v>
+        <v>2016</v>
       </c>
       <c r="AQ95">
         <v>0.87642823047249596</v>
@@ -39042,7 +39042,7 @@
         <v>4.0658428646815868E-2</v>
       </c>
       <c r="AT95" t="s">
-        <v>2009</v>
+        <v>2017</v>
       </c>
       <c r="AU95">
         <v>0.80956674230858228</v>
@@ -39063,10 +39063,10 @@
         <v>7.6574942173962199E-2</v>
       </c>
       <c r="BA95" t="s">
-        <v>2010</v>
+        <v>2018</v>
       </c>
       <c r="BB95" t="s">
-        <v>2011</v>
+        <v>2019</v>
       </c>
       <c r="BC95">
         <v>0.95672313157912237</v>
@@ -39087,10 +39087,10 @@
         <v>7.9321056760163183E-2</v>
       </c>
       <c r="BI95" t="s">
-        <v>2012</v>
+        <v>2020</v>
       </c>
       <c r="BJ95" t="s">
-        <v>2013</v>
+        <v>2021</v>
       </c>
       <c r="BK95">
         <v>0.80952380952380953</v>
@@ -39111,7 +39111,7 @@
         <v>8.4408584322427746E-2</v>
       </c>
       <c r="BQ95" t="s">
-        <v>2014</v>
+        <v>2022</v>
       </c>
       <c r="BR95">
         <v>0.94681667538810399</v>
@@ -39123,10 +39123,10 @@
         <v>3.0782577013458021E-2</v>
       </c>
       <c r="BU95" t="s">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="BV95" t="s">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="BW95">
         <v>0.85722878895147814</v>
@@ -39147,10 +39147,10 @@
         <v>1.0847611032199609E-2</v>
       </c>
       <c r="CC95" t="s">
-        <v>2017</v>
+        <v>2025</v>
       </c>
       <c r="CD95" t="s">
-        <v>2018</v>
+        <v>2026</v>
       </c>
       <c r="CE95">
         <v>0.87979823730049567</v>
@@ -39162,7 +39162,7 @@
         <v>8.8166518431554951E-3</v>
       </c>
       <c r="CH95" t="s">
-        <v>2019</v>
+        <v>2027</v>
       </c>
       <c r="CI95">
         <v>0.8130634152597308</v>
@@ -39183,10 +39183,10 @@
         <v>1.3372804051122169E-2</v>
       </c>
       <c r="CO95" t="s">
-        <v>2020</v>
+        <v>2028</v>
       </c>
       <c r="CP95" t="s">
-        <v>2021</v>
+        <v>2029</v>
       </c>
       <c r="CQ95">
         <v>0.95763568236948893</v>
@@ -39207,10 +39207,10 @@
         <v>1.9157236468690279E-2</v>
       </c>
       <c r="CW95" t="s">
-        <v>2022</v>
+        <v>2030</v>
       </c>
       <c r="CX95" t="s">
-        <v>2023</v>
+        <v>2031</v>
       </c>
       <c r="CY95">
         <v>0.81379731379731368</v>
@@ -39231,7 +39231,7 @@
         <v>1.075183998923873E-2</v>
       </c>
       <c r="DE95" t="s">
-        <v>2024</v>
+        <v>2032</v>
       </c>
       <c r="DF95">
         <v>0.94716972258989074</v>
@@ -39251,10 +39251,10 @@
         <v>113</v>
       </c>
       <c r="C96" t="s">
-        <v>2025</v>
+        <v>2033</v>
       </c>
       <c r="D96" t="s">
-        <v>2242</v>
+        <v>2034</v>
       </c>
       <c r="E96">
         <v>0.85333333333333339</v>
@@ -39317,7 +39317,7 @@
         <v>0.99526066350710907</v>
       </c>
       <c r="Y96" t="s">
-        <v>2026</v>
+        <v>2035</v>
       </c>
       <c r="Z96">
         <v>9.8139217921665734E-3</v>
@@ -39329,7 +39329,7 @@
         <v>9.4705337031672293E-4</v>
       </c>
       <c r="AC96" t="s">
-        <v>2027</v>
+        <v>2036</v>
       </c>
       <c r="AD96">
         <v>1.6008002417428151E-2</v>
@@ -39341,10 +39341,10 @@
         <v>1.4631953176020591E-3</v>
       </c>
       <c r="AG96" t="s">
-        <v>2028</v>
+        <v>2037</v>
       </c>
       <c r="AH96" t="s">
-        <v>2029</v>
+        <v>2038</v>
       </c>
       <c r="AI96">
         <v>0.88590594132389799</v>
@@ -39365,10 +39365,10 @@
         <v>3.6143803771930168E-2</v>
       </c>
       <c r="AO96" t="s">
-        <v>2030</v>
+        <v>2039</v>
       </c>
       <c r="AP96" t="s">
-        <v>2031</v>
+        <v>2040</v>
       </c>
       <c r="AQ96">
         <v>0.85135387326356138</v>
@@ -39380,7 +39380,7 @@
         <v>4.5773095695721321E-2</v>
       </c>
       <c r="AT96" t="s">
-        <v>2032</v>
+        <v>2041</v>
       </c>
       <c r="AU96">
         <v>0.8833888866710965</v>
@@ -39401,10 +39401,10 @@
         <v>2.9806642222565741E-2</v>
       </c>
       <c r="BA96" t="s">
-        <v>2033</v>
+        <v>2042</v>
       </c>
       <c r="BB96" t="s">
-        <v>2034</v>
+        <v>2043</v>
       </c>
       <c r="BC96">
         <v>0.84717746747821931</v>
@@ -39425,10 +39425,10 @@
         <v>2.7877211900740991E-2</v>
       </c>
       <c r="BI96" t="s">
-        <v>2035</v>
+        <v>2044</v>
       </c>
       <c r="BJ96" t="s">
-        <v>2036</v>
+        <v>2045</v>
       </c>
       <c r="BK96">
         <v>0.86340852130325818</v>
@@ -39449,7 +39449,7 @@
         <v>5.5969162370913303E-2</v>
       </c>
       <c r="BQ96" t="s">
-        <v>2037</v>
+        <v>2046</v>
       </c>
       <c r="BR96">
         <v>0.91902936613241792</v>
@@ -39464,7 +39464,7 @@
         <v>369</v>
       </c>
       <c r="BV96" t="s">
-        <v>1915</v>
+        <v>1918</v>
       </c>
       <c r="BW96">
         <v>0.99826460539223982</v>
@@ -39485,10 +39485,10 @@
         <v>1.417051170840857E-3</v>
       </c>
       <c r="CC96" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="CD96" t="s">
-        <v>1917</v>
+        <v>1920</v>
       </c>
       <c r="CE96">
         <v>0.99685336689741977</v>
@@ -39500,7 +39500,7 @@
         <v>1.9901055130071761E-3</v>
       </c>
       <c r="CH96" t="s">
-        <v>1918</v>
+        <v>1921</v>
       </c>
       <c r="CI96">
         <v>0.99755687288639661</v>
@@ -39524,7 +39524,7 @@
         <v>375</v>
       </c>
       <c r="CP96" t="s">
-        <v>1919</v>
+        <v>1922</v>
       </c>
       <c r="CQ96">
         <v>0.99373433583959891</v>
@@ -39545,7 +39545,7 @@
         <v>0</v>
       </c>
       <c r="CW96" t="s">
-        <v>1920</v>
+        <v>1923</v>
       </c>
       <c r="CX96" t="s">
         <v>375</v>
@@ -39589,10 +39589,10 @@
         <v>138</v>
       </c>
       <c r="C97" t="s">
-        <v>2038</v>
+        <v>2047</v>
       </c>
       <c r="D97" t="s">
-        <v>2241</v>
+        <v>2048</v>
       </c>
       <c r="E97">
         <v>0.84</v>
@@ -39655,7 +39655,7 @@
         <v>0.95981087470449178</v>
       </c>
       <c r="Y97" t="s">
-        <v>2039</v>
+        <v>2049</v>
       </c>
       <c r="Z97">
         <v>8.5113729749407094E-3</v>
@@ -39667,7 +39667,7 @@
         <v>8.9348110366789751E-4</v>
       </c>
       <c r="AC97" t="s">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="AD97">
         <v>1.6461508614676341E-2</v>
@@ -39679,10 +39679,10 @@
         <v>1.1809220954667899E-3</v>
       </c>
       <c r="AG97" t="s">
-        <v>2041</v>
+        <v>2051</v>
       </c>
       <c r="AH97" t="s">
-        <v>2042</v>
+        <v>2052</v>
       </c>
       <c r="AI97">
         <v>0.86187859759288321</v>
@@ -39703,10 +39703,10 @@
         <v>5.8686965356105063E-2</v>
       </c>
       <c r="AO97" t="s">
-        <v>2043</v>
+        <v>2053</v>
       </c>
       <c r="AP97" t="s">
-        <v>2044</v>
+        <v>2054</v>
       </c>
       <c r="AQ97">
         <v>0.9058525285642629</v>
@@ -39718,7 +39718,7 @@
         <v>4.4834732615850942E-2</v>
       </c>
       <c r="AT97" t="s">
-        <v>2045</v>
+        <v>2055</v>
       </c>
       <c r="AU97">
         <v>0.84241653879667433</v>
@@ -39739,10 +39739,10 @@
         <v>8.2415499252061833E-2</v>
       </c>
       <c r="BA97" t="s">
-        <v>2046</v>
+        <v>2056</v>
       </c>
       <c r="BB97" t="s">
-        <v>2047</v>
+        <v>2057</v>
       </c>
       <c r="BC97">
         <v>0.94067831401975588</v>
@@ -39763,10 +39763,10 @@
         <v>0.11443901769543049</v>
       </c>
       <c r="BI97" t="s">
-        <v>2048</v>
+        <v>2058</v>
       </c>
       <c r="BJ97" t="s">
-        <v>2049</v>
+        <v>2059</v>
       </c>
       <c r="BK97">
         <v>0.87545787545787535</v>
@@ -39787,7 +39787,7 @@
         <v>7.0970347514258389E-2</v>
       </c>
       <c r="BQ97" t="s">
-        <v>2050</v>
+        <v>2060</v>
       </c>
       <c r="BR97">
         <v>0.91036106750392476</v>
@@ -39799,10 +39799,10 @@
         <v>5.3732196890561801E-2</v>
       </c>
       <c r="BU97" t="s">
-        <v>2051</v>
+        <v>2061</v>
       </c>
       <c r="BV97" t="s">
-        <v>2052</v>
+        <v>2062</v>
       </c>
       <c r="BW97">
         <v>0.95042247668298097</v>
@@ -39823,10 +39823,10 @@
         <v>5.241863005903344E-3</v>
       </c>
       <c r="CC97" t="s">
-        <v>2053</v>
+        <v>2063</v>
       </c>
       <c r="CD97" t="s">
-        <v>2054</v>
+        <v>2064</v>
       </c>
       <c r="CE97">
         <v>0.96187498057230314</v>
@@ -39838,7 +39838,7 @@
         <v>3.6640131249366221E-3</v>
       </c>
       <c r="CH97" t="s">
-        <v>2055</v>
+        <v>2065</v>
       </c>
       <c r="CI97">
         <v>0.93267837381665519</v>
@@ -39859,10 +39859,10 @@
         <v>9.2535578013054828E-3</v>
       </c>
       <c r="CO97" t="s">
-        <v>2056</v>
+        <v>2066</v>
       </c>
       <c r="CP97" t="s">
-        <v>2057</v>
+        <v>2067</v>
       </c>
       <c r="CQ97">
         <v>0.98529986432933259</v>
@@ -39883,10 +39883,10 @@
         <v>1.0211061853907291E-2</v>
       </c>
       <c r="CW97" t="s">
-        <v>2058</v>
+        <v>2068</v>
       </c>
       <c r="CX97" t="s">
-        <v>2059</v>
+        <v>2069</v>
       </c>
       <c r="CY97">
         <v>0.93956043956043966</v>
@@ -39907,7 +39907,7 @@
         <v>1.36398536179124E-2</v>
       </c>
       <c r="DE97" t="s">
-        <v>2060</v>
+        <v>2070</v>
       </c>
       <c r="DF97">
         <v>0.99214048867410221</v>
@@ -39927,10 +39927,10 @@
         <v>113</v>
       </c>
       <c r="C98" t="s">
-        <v>2061</v>
+        <v>2071</v>
       </c>
       <c r="D98" t="s">
-        <v>2240</v>
+        <v>2072</v>
       </c>
       <c r="E98">
         <v>0.82666666666666666</v>
@@ -39993,7 +39993,7 @@
         <v>0.87037037037037035</v>
       </c>
       <c r="Y98" t="s">
-        <v>2062</v>
+        <v>2073</v>
       </c>
       <c r="Z98">
         <v>1.7965078353881839E-2</v>
@@ -40005,7 +40005,7 @@
         <v>7.6296203869359092E-4</v>
       </c>
       <c r="AC98" t="s">
-        <v>2063</v>
+        <v>2074</v>
       </c>
       <c r="AD98">
         <v>1.4922244208199639E-2</v>
@@ -40017,10 +40017,10 @@
         <v>5.4791746153441017E-4</v>
       </c>
       <c r="AG98" t="s">
-        <v>2064</v>
+        <v>2075</v>
       </c>
       <c r="AH98" t="s">
-        <v>2065</v>
+        <v>2076</v>
       </c>
       <c r="AI98">
         <v>0.87818776633460394</v>
@@ -40041,10 +40041,10 @@
         <v>4.8420056979197192E-2</v>
       </c>
       <c r="AO98" t="s">
-        <v>2066</v>
+        <v>2077</v>
       </c>
       <c r="AP98" t="s">
-        <v>2067</v>
+        <v>2078</v>
       </c>
       <c r="AQ98">
         <v>0.83685393197588309</v>
@@ -40056,7 +40056,7 @@
         <v>6.0923346791577723E-2</v>
       </c>
       <c r="AT98" t="s">
-        <v>2068</v>
+        <v>2079</v>
       </c>
       <c r="AU98">
         <v>0.86840731517387559</v>
@@ -40077,10 +40077,10 @@
         <v>4.0340855897196118E-2</v>
       </c>
       <c r="BA98" t="s">
-        <v>2069</v>
+        <v>2080</v>
       </c>
       <c r="BB98" t="s">
-        <v>2070</v>
+        <v>2081</v>
       </c>
       <c r="BC98">
         <v>0.79834988540870899</v>
@@ -40101,10 +40101,10 @@
         <v>3.0038471158665689E-2</v>
       </c>
       <c r="BI98" t="s">
-        <v>2071</v>
+        <v>2082</v>
       </c>
       <c r="BJ98" t="s">
-        <v>2072</v>
+        <v>2083</v>
       </c>
       <c r="BK98">
         <v>0.88554720133667486</v>
@@ -40125,7 +40125,7 @@
         <v>6.5125801472186981E-2</v>
       </c>
       <c r="BQ98" t="s">
-        <v>2073</v>
+        <v>2084</v>
       </c>
       <c r="BR98">
         <v>0.93420947326298953</v>
@@ -40137,10 +40137,10 @@
         <v>3.2692277747609987E-2</v>
       </c>
       <c r="BU98" t="s">
-        <v>2074</v>
+        <v>2085</v>
       </c>
       <c r="BV98" t="s">
-        <v>2075</v>
+        <v>2086</v>
       </c>
       <c r="BW98">
         <v>0.90295281885652279</v>
@@ -40161,10 +40161,10 @@
         <v>3.5749186921830499E-3</v>
       </c>
       <c r="CC98" t="s">
-        <v>2076</v>
+        <v>2087</v>
       </c>
       <c r="CD98" t="s">
-        <v>2077</v>
+        <v>2088</v>
       </c>
       <c r="CE98">
         <v>0.866330297705592</v>
@@ -40176,7 +40176,7 @@
         <v>5.723592902356963E-3</v>
       </c>
       <c r="CH98" t="s">
-        <v>2078</v>
+        <v>2089</v>
       </c>
       <c r="CI98">
         <v>0.89327129289729701</v>
@@ -40197,10 +40197,10 @@
         <v>2.753989329424617E-3</v>
       </c>
       <c r="CO98" t="s">
-        <v>2079</v>
+        <v>2090</v>
       </c>
       <c r="CP98" t="s">
-        <v>2080</v>
+        <v>2091</v>
       </c>
       <c r="CQ98">
         <v>0.82464067370751004</v>
@@ -40221,10 +40221,10 @@
         <v>9.674706604636844E-3</v>
       </c>
       <c r="CW98" t="s">
-        <v>2081</v>
+        <v>2092</v>
       </c>
       <c r="CX98" t="s">
-        <v>2082</v>
+        <v>2093</v>
       </c>
       <c r="CY98">
         <v>0.91285736465056455</v>
@@ -40245,7 +40245,7 @@
         <v>8.6966904373310706E-3</v>
       </c>
       <c r="DE98" t="s">
-        <v>2083</v>
+        <v>2094</v>
       </c>
       <c r="DF98">
         <v>0.96051483720523034</v>
@@ -40265,10 +40265,10 @@
         <v>138</v>
       </c>
       <c r="C99" t="s">
-        <v>2084</v>
+        <v>2095</v>
       </c>
       <c r="D99" t="s">
-        <v>2239</v>
+        <v>2096</v>
       </c>
       <c r="E99">
         <v>0.8666666666666667</v>
@@ -40331,7 +40331,7 @@
         <v>0.94033412887828161</v>
       </c>
       <c r="Y99" t="s">
-        <v>2085</v>
+        <v>2097</v>
       </c>
       <c r="Z99">
         <v>1.9875662667410719E-2</v>
@@ -40343,7 +40343,7 @@
         <v>1.4171759515281201E-3</v>
       </c>
       <c r="AC99" t="s">
-        <v>2086</v>
+        <v>2098</v>
       </c>
       <c r="AD99">
         <v>1.385617256164551E-2</v>
@@ -40355,10 +40355,10 @@
         <v>6.5349001003401036E-4</v>
       </c>
       <c r="AG99" t="s">
-        <v>2087</v>
+        <v>2099</v>
       </c>
       <c r="AH99" t="s">
-        <v>2088</v>
+        <v>2100</v>
       </c>
       <c r="AI99">
         <v>0.90562532705389864</v>
@@ -40379,10 +40379,10 @@
         <v>2.746839050685379E-2</v>
       </c>
       <c r="AO99" t="s">
-        <v>2089</v>
+        <v>2101</v>
       </c>
       <c r="AP99" t="s">
-        <v>2090</v>
+        <v>2102</v>
       </c>
       <c r="AQ99">
         <v>0.92029803678361222</v>
@@ -40394,7 +40394,7 @@
         <v>2.1575555667991572E-2</v>
       </c>
       <c r="AT99" t="s">
-        <v>2091</v>
+        <v>2103</v>
       </c>
       <c r="AU99">
         <v>0.8704188154601934</v>
@@ -40415,10 +40415,10 @@
         <v>3.7250334936681527E-2</v>
       </c>
       <c r="BA99" t="s">
-        <v>2092</v>
+        <v>2104</v>
       </c>
       <c r="BB99" t="s">
-        <v>2093</v>
+        <v>2105</v>
       </c>
       <c r="BC99">
         <v>0.97590281608138751</v>
@@ -40439,10 +40439,10 @@
         <v>5.5678541153844498E-2</v>
       </c>
       <c r="BI99" t="s">
-        <v>2094</v>
+        <v>2106</v>
       </c>
       <c r="BJ99" t="s">
-        <v>2095</v>
+        <v>2107</v>
       </c>
       <c r="BK99">
         <v>0.8717948717948717</v>
@@ -40463,7 +40463,7 @@
         <v>4.5512186894361192E-2</v>
       </c>
       <c r="BQ99" t="s">
-        <v>2096</v>
+        <v>2108</v>
       </c>
       <c r="BR99">
         <v>0.9646781789638933</v>
@@ -40475,10 +40475,10 @@
         <v>2.1126770526620962E-2</v>
       </c>
       <c r="BU99" t="s">
-        <v>2097</v>
+        <v>2109</v>
       </c>
       <c r="BV99" t="s">
-        <v>2098</v>
+        <v>2110</v>
       </c>
       <c r="BW99">
         <v>0.92247668298088481</v>
@@ -40499,10 +40499,10 @@
         <v>7.0922984370790582E-3</v>
       </c>
       <c r="CC99" t="s">
-        <v>2099</v>
+        <v>2111</v>
       </c>
       <c r="CD99" t="s">
-        <v>2100</v>
+        <v>2112</v>
       </c>
       <c r="CE99">
         <v>0.93513441168012268</v>
@@ -40514,7 +40514,7 @@
         <v>5.4393329577296836E-3</v>
       </c>
       <c r="CH99" t="s">
-        <v>2101</v>
+        <v>2113</v>
       </c>
       <c r="CI99">
         <v>0.89148144436884802</v>
@@ -40535,10 +40535,10 @@
         <v>9.9619378088634074E-3</v>
       </c>
       <c r="CO99" t="s">
-        <v>2102</v>
+        <v>2114</v>
       </c>
       <c r="CP99" t="s">
-        <v>2103</v>
+        <v>2115</v>
       </c>
       <c r="CQ99">
         <v>0.98060667836513293</v>
@@ -40559,10 +40559,10 @@
         <v>1.6836285612491529E-2</v>
       </c>
       <c r="CW99" t="s">
-        <v>2104</v>
+        <v>2116</v>
       </c>
       <c r="CX99" t="s">
-        <v>2105</v>
+        <v>2117</v>
       </c>
       <c r="CY99">
         <v>0.89377289377289393</v>
@@ -40583,7 +40583,7 @@
         <v>9.7881474720958109E-3</v>
       </c>
       <c r="DE99" t="s">
-        <v>2106</v>
+        <v>2118</v>
       </c>
       <c r="DF99">
         <v>0.97186242018174795</v>
@@ -40603,10 +40603,10 @@
         <v>113</v>
       </c>
       <c r="C100" t="s">
-        <v>2107</v>
+        <v>2119</v>
       </c>
       <c r="D100" t="s">
-        <v>2238</v>
+        <v>2120</v>
       </c>
       <c r="E100">
         <v>0.77333333333333332</v>
@@ -40669,7 +40669,7 @@
         <v>0.78688524590163933</v>
       </c>
       <c r="Y100" t="s">
-        <v>2108</v>
+        <v>2121</v>
       </c>
       <c r="Z100">
         <v>2.3105280739920481E-2</v>
@@ -40681,7 +40681,7 @@
         <v>1.0477354835695481E-3</v>
       </c>
       <c r="AC100" t="s">
-        <v>2109</v>
+        <v>2122</v>
       </c>
       <c r="AD100">
         <v>1.5482766287667409E-2</v>
@@ -40693,10 +40693,10 @@
         <v>1.5003551197444911E-3</v>
       </c>
       <c r="AG100" t="s">
-        <v>2110</v>
+        <v>2123</v>
       </c>
       <c r="AH100" t="s">
-        <v>2111</v>
+        <v>2124</v>
       </c>
       <c r="AI100">
         <v>0.82454595873437087</v>
@@ -40717,10 +40717,10 @@
         <v>5.6949482866748793E-2</v>
       </c>
       <c r="AO100" t="s">
-        <v>2112</v>
+        <v>2125</v>
       </c>
       <c r="AP100" t="s">
-        <v>2113</v>
+        <v>2126</v>
       </c>
       <c r="AQ100">
         <v>0.76687574624640675</v>
@@ -40732,7 +40732,7 @@
         <v>6.8586074816066336E-2</v>
       </c>
       <c r="AT100" t="s">
-        <v>2114</v>
+        <v>2127</v>
       </c>
       <c r="AU100">
         <v>0.80183822529612747</v>
@@ -40753,10 +40753,10 @@
         <v>5.1109266237862452E-2</v>
       </c>
       <c r="BA100" t="s">
-        <v>2115</v>
+        <v>2128</v>
       </c>
       <c r="BB100" t="s">
-        <v>2116</v>
+        <v>2129</v>
       </c>
       <c r="BC100">
         <v>0.68691585629146934</v>
@@ -40777,10 +40777,10 @@
         <v>4.9811536920238438E-2</v>
       </c>
       <c r="BI100" t="s">
-        <v>2117</v>
+        <v>2130</v>
       </c>
       <c r="BJ100" t="s">
-        <v>2118</v>
+        <v>2131</v>
       </c>
       <c r="BK100">
         <v>0.87886382623224724</v>
@@ -40801,7 +40801,7 @@
         <v>8.2438470350551546E-2</v>
       </c>
       <c r="BQ100" t="s">
-        <v>2119</v>
+        <v>2132</v>
       </c>
       <c r="BR100">
         <v>0.89465961823325812</v>
@@ -40813,10 +40813,10 @@
         <v>4.8504592798555728E-2</v>
       </c>
       <c r="BU100" t="s">
-        <v>2120</v>
+        <v>2133</v>
       </c>
       <c r="BV100" t="s">
-        <v>2121</v>
+        <v>2134</v>
       </c>
       <c r="BW100">
         <v>0.84143153793528047</v>
@@ -40837,10 +40837,10 @@
         <v>1.1287634320127299E-2</v>
       </c>
       <c r="CC100" t="s">
-        <v>2122</v>
+        <v>2135</v>
       </c>
       <c r="CD100" t="s">
-        <v>2123</v>
+        <v>2136</v>
       </c>
       <c r="CE100">
         <v>0.78455461054019093</v>
@@ -40852,7 +40852,7 @@
         <v>1.002078727098015E-2</v>
       </c>
       <c r="CH100" t="s">
-        <v>2124</v>
+        <v>2137</v>
       </c>
       <c r="CI100">
         <v>0.81812100140322497</v>
@@ -40873,10 +40873,10 @@
         <v>1.1382181766083769E-2</v>
       </c>
       <c r="CO100" t="s">
-        <v>2125</v>
+        <v>2138</v>
       </c>
       <c r="CP100" t="s">
-        <v>2126</v>
+        <v>2139</v>
       </c>
       <c r="CQ100">
         <v>0.69565518878508315</v>
@@ -40897,10 +40897,10 @@
         <v>5.8367951465261997E-3</v>
       </c>
       <c r="CW100" t="s">
-        <v>2127</v>
+        <v>2140</v>
       </c>
       <c r="CX100" t="s">
-        <v>2128</v>
+        <v>2141</v>
       </c>
       <c r="CY100">
         <v>0.90023731896111969</v>
@@ -40921,7 +40921,7 @@
         <v>2.1644660979063569E-2</v>
       </c>
       <c r="DE100" t="s">
-        <v>2129</v>
+        <v>2142</v>
       </c>
       <c r="DF100">
         <v>0.90858423996449489</v>
@@ -40941,10 +40941,10 @@
         <v>138</v>
       </c>
       <c r="C101" t="s">
-        <v>2130</v>
+        <v>2143</v>
       </c>
       <c r="D101" t="s">
-        <v>2237</v>
+        <v>2144</v>
       </c>
       <c r="E101">
         <v>0.84</v>
@@ -41007,7 +41007,7 @@
         <v>0.87745098039215685</v>
       </c>
       <c r="Y101" t="s">
-        <v>2131</v>
+        <v>2145</v>
       </c>
       <c r="Z101">
         <v>2.1329164505004879E-2</v>
@@ -41019,7 +41019,7 @@
         <v>1.215711213782499E-3</v>
       </c>
       <c r="AC101" t="s">
-        <v>2132</v>
+        <v>2146</v>
       </c>
       <c r="AD101">
         <v>1.324030331202916E-2</v>
@@ -41151,10 +41151,10 @@
         <v>3.1019267646652839E-2</v>
       </c>
       <c r="BU101" t="s">
-        <v>2133</v>
+        <v>2147</v>
       </c>
       <c r="BV101" t="s">
-        <v>2134</v>
+        <v>2148</v>
       </c>
       <c r="BW101">
         <v>0.85572716265993554</v>
@@ -41175,10 +41175,10 @@
         <v>1.0682749221641899E-2</v>
       </c>
       <c r="CC101" t="s">
-        <v>2135</v>
+        <v>2149</v>
       </c>
       <c r="CD101" t="s">
-        <v>2136</v>
+        <v>2150</v>
       </c>
       <c r="CE101">
         <v>0.88741849171643838</v>
@@ -41190,7 +41190,7 @@
         <v>8.0051036466715596E-3</v>
       </c>
       <c r="CH101" t="s">
-        <v>2137</v>
+        <v>2151</v>
       </c>
       <c r="CI101">
         <v>0.81926716312307035</v>
@@ -41211,10 +41211,10 @@
         <v>1.628538920568498E-2</v>
       </c>
       <c r="CO101" t="s">
-        <v>2138</v>
+        <v>2152</v>
       </c>
       <c r="CP101" t="s">
-        <v>2139</v>
+        <v>2153</v>
       </c>
       <c r="CQ101">
         <v>0.94986102391262073</v>
@@ -41235,7 +41235,7 @@
         <v>1.7340165913896449E-2</v>
       </c>
       <c r="CW101" t="s">
-        <v>2140</v>
+        <v>2154</v>
       </c>
       <c r="CX101" t="s">
         <v>918</v>
@@ -41259,7 +41259,7 @@
         <v>1.6808794818811829E-2</v>
       </c>
       <c r="DE101" t="s">
-        <v>2141</v>
+        <v>2155</v>
       </c>
       <c r="DF101">
         <v>0.94572110895640316</v>
@@ -41279,10 +41279,10 @@
         <v>113</v>
       </c>
       <c r="C102" t="s">
-        <v>2142</v>
+        <v>2156</v>
       </c>
       <c r="D102" t="s">
-        <v>2236</v>
+        <v>2157</v>
       </c>
       <c r="E102">
         <v>0.85333333333333339</v>
@@ -41345,7 +41345,7 @@
         <v>0.99526066350710907</v>
       </c>
       <c r="Y102" t="s">
-        <v>2143</v>
+        <v>2158</v>
       </c>
       <c r="Z102">
         <v>2.1659817014421739E-2</v>
@@ -41357,7 +41357,7 @@
         <v>2.234422033747832E-3</v>
       </c>
       <c r="AC102" t="s">
-        <v>2144</v>
+        <v>2159</v>
       </c>
       <c r="AD102">
         <v>1.7643928527832031E-2</v>
@@ -41369,10 +41369,10 @@
         <v>4.9283557665869941E-3</v>
       </c>
       <c r="AG102" t="s">
-        <v>2145</v>
+        <v>2160</v>
       </c>
       <c r="AH102" t="s">
-        <v>2146</v>
+        <v>2161</v>
       </c>
       <c r="AI102">
         <v>0.89342473831637914</v>
@@ -41393,10 +41393,10 @@
         <v>3.7689074138275193E-2</v>
       </c>
       <c r="AO102" t="s">
-        <v>2147</v>
+        <v>2162</v>
       </c>
       <c r="AP102" t="s">
-        <v>2148</v>
+        <v>2163</v>
       </c>
       <c r="AQ102">
         <v>0.85962454995529058</v>
@@ -41408,7 +41408,7 @@
         <v>4.8503776338968622E-2</v>
       </c>
       <c r="AT102" t="s">
-        <v>2149</v>
+        <v>2164</v>
       </c>
       <c r="AU102">
         <v>0.88949774169636009</v>
@@ -41429,10 +41429,10 @@
         <v>3.0871093784943279E-2</v>
       </c>
       <c r="BA102" t="s">
-        <v>2150</v>
+        <v>2165</v>
       </c>
       <c r="BB102" t="s">
-        <v>2151</v>
+        <v>2166</v>
       </c>
       <c r="BC102">
         <v>0.84932569519035683</v>
@@ -41453,10 +41453,10 @@
         <v>3.0973415437552439E-2</v>
       </c>
       <c r="BI102" t="s">
-        <v>2035</v>
+        <v>2044</v>
       </c>
       <c r="BJ102" t="s">
-        <v>2152</v>
+        <v>2167</v>
       </c>
       <c r="BK102">
         <v>0.87844611528822047</v>
@@ -41477,7 +41477,7 @@
         <v>5.5969162370913303E-2</v>
       </c>
       <c r="BQ102" t="s">
-        <v>2153</v>
+        <v>2168</v>
       </c>
       <c r="BR102">
         <v>0.89342473831637914</v>
@@ -41492,7 +41492,7 @@
         <v>369</v>
       </c>
       <c r="BV102" t="s">
-        <v>2154</v>
+        <v>2169</v>
       </c>
       <c r="BW102">
         <v>0.9974101849692536</v>
@@ -41513,10 +41513,10 @@
         <v>1.417051170840857E-3</v>
       </c>
       <c r="CC102" t="s">
-        <v>2155</v>
+        <v>2170</v>
       </c>
       <c r="CD102" t="s">
-        <v>2156</v>
+        <v>2171</v>
       </c>
       <c r="CE102">
         <v>0.99683658485420601</v>
@@ -41528,7 +41528,7 @@
         <v>2.0007850996625648E-3</v>
       </c>
       <c r="CH102" t="s">
-        <v>2157</v>
+        <v>2172</v>
       </c>
       <c r="CI102">
         <v>0.99755101492102438</v>
@@ -41549,10 +41549,10 @@
         <v>1.097039760045307E-3</v>
       </c>
       <c r="CO102" t="s">
-        <v>2158</v>
+        <v>2173</v>
       </c>
       <c r="CP102" t="s">
-        <v>2159</v>
+        <v>2174</v>
       </c>
       <c r="CQ102">
         <v>0.99749373433583954</v>
@@ -41573,10 +41573,10 @@
         <v>2.3945637022855341E-3</v>
       </c>
       <c r="CW102" t="s">
-        <v>2160</v>
+        <v>2175</v>
       </c>
       <c r="CX102" t="s">
-        <v>2161</v>
+        <v>2176</v>
       </c>
       <c r="CY102">
         <v>0.99620733249051818</v>
@@ -41597,7 +41597,7 @@
         <v>2.192980346857405E-3</v>
       </c>
       <c r="DE102" t="s">
-        <v>2154</v>
+        <v>2169</v>
       </c>
       <c r="DF102">
         <v>0.9974101849692536</v>
@@ -41617,10 +41617,10 @@
         <v>138</v>
       </c>
       <c r="C103" t="s">
-        <v>2162</v>
+        <v>2177</v>
       </c>
       <c r="D103" t="s">
-        <v>2235</v>
+        <v>2178</v>
       </c>
       <c r="E103">
         <v>0.85333333333333339</v>
@@ -41683,7 +41683,7 @@
         <v>0.95981087470449178</v>
       </c>
       <c r="Y103" t="s">
-        <v>2163</v>
+        <v>2179</v>
       </c>
       <c r="Z103">
         <v>2.099997656685965E-2</v>
@@ -41695,7 +41695,7 @@
         <v>1.519553433003547E-3</v>
       </c>
       <c r="AC103" t="s">
-        <v>2164</v>
+        <v>2180</v>
       </c>
       <c r="AD103">
         <v>1.6360282897949219E-2</v>
@@ -41707,10 +41707,10 @@
         <v>1.317893547891996E-3</v>
       </c>
       <c r="AG103" t="s">
-        <v>2165</v>
+        <v>2181</v>
       </c>
       <c r="AH103" t="s">
-        <v>2166</v>
+        <v>2182</v>
       </c>
       <c r="AI103">
         <v>0.84874411302982722</v>
@@ -41731,10 +41731,10 @@
         <v>5.5933610865319859E-2</v>
       </c>
       <c r="AO103" t="s">
-        <v>2167</v>
+        <v>2183</v>
       </c>
       <c r="AP103" t="s">
-        <v>2168</v>
+        <v>2184</v>
       </c>
       <c r="AQ103">
         <v>0.90274987774987792</v>
@@ -41746,7 +41746,7 @@
         <v>4.303126788446314E-2</v>
       </c>
       <c r="AT103" t="s">
-        <v>2169</v>
+        <v>2185</v>
       </c>
       <c r="AU103">
         <v>0.83364084151390994</v>
@@ -41767,10 +41767,10 @@
         <v>7.7939877746625683E-2</v>
       </c>
       <c r="BA103" t="s">
-        <v>2170</v>
+        <v>2186</v>
       </c>
       <c r="BB103" t="s">
-        <v>2171</v>
+        <v>2187</v>
       </c>
       <c r="BC103">
         <v>0.93074284966821186</v>
@@ -41791,10 +41791,10 @@
         <v>0.1131929317366905</v>
       </c>
       <c r="BI103" t="s">
-        <v>2172</v>
+        <v>2188</v>
       </c>
       <c r="BJ103" t="s">
-        <v>2173</v>
+        <v>2189</v>
       </c>
       <c r="BK103">
         <v>0.879120879120879</v>
@@ -41815,7 +41815,7 @@
         <v>8.3548936695749879E-2</v>
       </c>
       <c r="BQ103" t="s">
-        <v>2174</v>
+        <v>2190</v>
       </c>
       <c r="BR103">
         <v>0.9094104308390023</v>
@@ -41827,10 +41827,10 @@
         <v>6.1376568268449852E-2</v>
       </c>
       <c r="BU103" t="s">
-        <v>2175</v>
+        <v>2191</v>
       </c>
       <c r="BV103" t="s">
-        <v>2176</v>
+        <v>2192</v>
       </c>
       <c r="BW103">
         <v>0.93901842788397427</v>
@@ -41851,10 +41851,10 @@
         <v>4.0854772818506363E-3</v>
       </c>
       <c r="CC103" t="s">
-        <v>2177</v>
+        <v>2193</v>
       </c>
       <c r="CD103" t="s">
-        <v>2178</v>
+        <v>2194</v>
       </c>
       <c r="CE103">
         <v>0.95868259941295719</v>
@@ -41866,7 +41866,7 @@
         <v>2.838224405392204E-3</v>
       </c>
       <c r="CH103" t="s">
-        <v>2179</v>
+        <v>2195</v>
       </c>
       <c r="CI103">
         <v>0.92591280561103628</v>
@@ -41887,10 +41887,10 @@
         <v>7.6044665485748156E-3</v>
       </c>
       <c r="CO103" t="s">
-        <v>2180</v>
+        <v>2196</v>
       </c>
       <c r="CP103" t="s">
-        <v>2181</v>
+        <v>2197</v>
       </c>
       <c r="CQ103">
         <v>0.97603915902888172</v>
@@ -41911,10 +41911,10 @@
         <v>1.2413477317532879E-2</v>
       </c>
       <c r="CW103" t="s">
-        <v>2182</v>
+        <v>2198</v>
       </c>
       <c r="CX103" t="s">
-        <v>2183</v>
+        <v>2199</v>
       </c>
       <c r="CY103">
         <v>0.9420024420024421</v>
@@ -41935,7 +41935,7 @@
         <v>1.868980982523908E-2</v>
       </c>
       <c r="DE103" t="s">
-        <v>2184</v>
+        <v>2200</v>
       </c>
       <c r="DF103">
         <v>0.98973880150350735</v>
@@ -41955,10 +41955,10 @@
         <v>113</v>
       </c>
       <c r="C104" t="s">
-        <v>2185</v>
+        <v>2201</v>
       </c>
       <c r="D104" t="s">
-        <v>2234</v>
+        <v>2202</v>
       </c>
       <c r="E104">
         <v>0.82666666666666666</v>
@@ -42021,7 +42021,7 @@
         <v>0.88262910798122074</v>
       </c>
       <c r="Y104" t="s">
-        <v>2186</v>
+        <v>2203</v>
       </c>
       <c r="Z104">
         <v>3.7236724581037252E-2</v>
@@ -42033,7 +42033,7 @@
         <v>8.2159155839204145E-3</v>
       </c>
       <c r="AC104" t="s">
-        <v>2187</v>
+        <v>2204</v>
       </c>
       <c r="AD104">
         <v>1.5778779983520511E-2</v>
@@ -42045,10 +42045,10 @@
         <v>1.173244839837054E-3</v>
       </c>
       <c r="AG104" t="s">
-        <v>2188</v>
+        <v>2205</v>
       </c>
       <c r="AH104" t="s">
-        <v>2189</v>
+        <v>2206</v>
       </c>
       <c r="AI104">
         <v>0.87839662180661726</v>
@@ -42069,10 +42069,10 @@
         <v>4.0404266678870822E-2</v>
       </c>
       <c r="AO104" t="s">
-        <v>2190</v>
+        <v>2207</v>
       </c>
       <c r="AP104" t="s">
-        <v>2191</v>
+        <v>2208</v>
       </c>
       <c r="AQ104">
         <v>0.83689210518478796</v>
@@ -42084,7 +42084,7 @@
         <v>4.9068389236544697E-2</v>
       </c>
       <c r="AT104" t="s">
-        <v>2192</v>
+        <v>2209</v>
       </c>
       <c r="AU104">
         <v>0.86848796755968216</v>
@@ -42105,10 +42105,10 @@
         <v>3.4062996209327012E-2</v>
       </c>
       <c r="BA104" t="s">
-        <v>2193</v>
+        <v>2210</v>
       </c>
       <c r="BB104" t="s">
-        <v>2194</v>
+        <v>2211</v>
       </c>
       <c r="BC104">
         <v>0.79710200285647848</v>
@@ -42129,10 +42129,10 @@
         <v>1.90987884856617E-2</v>
       </c>
       <c r="BI104" t="s">
-        <v>2195</v>
+        <v>2212</v>
       </c>
       <c r="BJ104" t="s">
-        <v>2196</v>
+        <v>2213</v>
       </c>
       <c r="BK104">
         <v>0.88596491228070173</v>
@@ -42153,7 +42153,7 @@
         <v>5.7032791190494078E-2</v>
       </c>
       <c r="BQ104" t="s">
-        <v>2197</v>
+        <v>2214</v>
       </c>
       <c r="BR104">
         <v>0.93547875290467075</v>
@@ -42165,10 +42165,10 @@
         <v>3.6243457358422833E-2</v>
       </c>
       <c r="BU104" t="s">
-        <v>2198</v>
+        <v>2215</v>
       </c>
       <c r="BV104" t="s">
-        <v>2199</v>
+        <v>2216</v>
       </c>
       <c r="BW104">
         <v>0.91085393166864537</v>
@@ -42189,10 +42189,10 @@
         <v>9.4007370205730183E-3</v>
       </c>
       <c r="CC104" t="s">
-        <v>2200</v>
+        <v>2217</v>
       </c>
       <c r="CD104" t="s">
-        <v>2201</v>
+        <v>2218</v>
       </c>
       <c r="CE104">
         <v>0.87645469811883614</v>
@@ -42204,7 +42204,7 @@
         <v>1.1203833681663611E-2</v>
       </c>
       <c r="CH104" t="s">
-        <v>2202</v>
+        <v>2219</v>
       </c>
       <c r="CI104">
         <v>0.90138476513178922</v>
@@ -42225,10 +42225,10 @@
         <v>8.0289328109743336E-3</v>
       </c>
       <c r="CO104" t="s">
-        <v>2203</v>
+        <v>2220</v>
       </c>
       <c r="CP104" t="s">
-        <v>2204</v>
+        <v>2221</v>
       </c>
       <c r="CQ104">
         <v>0.83570065482910205</v>
@@ -42249,10 +42249,10 @@
         <v>4.8536349487245476E-3</v>
       </c>
       <c r="CW104" t="s">
-        <v>2205</v>
+        <v>2222</v>
       </c>
       <c r="CX104" t="s">
-        <v>2206</v>
+        <v>2223</v>
       </c>
       <c r="CY104">
         <v>0.92171801184376878</v>
@@ -42273,7 +42273,7 @@
         <v>1.4523401200288871E-2</v>
       </c>
       <c r="DE104" t="s">
-        <v>2207</v>
+        <v>2224</v>
       </c>
       <c r="DF104">
         <v>0.96080524005577017</v>
@@ -42293,10 +42293,10 @@
         <v>138</v>
       </c>
       <c r="C105" t="s">
-        <v>2208</v>
+        <v>2225</v>
       </c>
       <c r="D105" t="s">
-        <v>2233</v>
+        <v>2226</v>
       </c>
       <c r="E105">
         <v>0.89333333333333331</v>
@@ -42359,7 +42359,7 @@
         <v>0.95104895104895104</v>
       </c>
       <c r="Y105" t="s">
-        <v>2209</v>
+        <v>2227</v>
       </c>
       <c r="Z105">
         <v>3.2412597111293247E-2</v>
@@ -42371,7 +42371,7 @@
         <v>2.0400411460430529E-3</v>
       </c>
       <c r="AC105" t="s">
-        <v>2210</v>
+        <v>2228</v>
       </c>
       <c r="AD105">
         <v>1.3770614351545059E-2</v>
@@ -42383,10 +42383,10 @@
         <v>7.8094096625935935E-4</v>
       </c>
       <c r="AG105" t="s">
-        <v>2211</v>
+        <v>2229</v>
       </c>
       <c r="AH105" t="s">
-        <v>2212</v>
+        <v>2230</v>
       </c>
       <c r="AI105">
         <v>0.90497121925693358</v>
@@ -42407,10 +42407,10 @@
         <v>4.9755159406517362E-2</v>
       </c>
       <c r="AO105" t="s">
-        <v>2213</v>
+        <v>2231</v>
       </c>
       <c r="AP105" t="s">
-        <v>2214</v>
+        <v>2232</v>
       </c>
       <c r="AQ105">
         <v>0.93118110534940279</v>
@@ -42422,7 +42422,7 @@
         <v>3.6791620985311517E-2</v>
       </c>
       <c r="AT105" t="s">
-        <v>2215</v>
+        <v>2233</v>
       </c>
       <c r="AU105">
         <v>0.8836974506062879</v>
@@ -42443,10 +42443,10 @@
         <v>7.6493001639104469E-2</v>
       </c>
       <c r="BA105" t="s">
-        <v>2216</v>
+        <v>2234</v>
       </c>
       <c r="BB105" t="s">
-        <v>2217</v>
+        <v>2235</v>
       </c>
       <c r="BC105">
         <v>0.96480551734863984</v>
@@ -42467,10 +42467,10 @@
         <v>0.10051147447399721</v>
       </c>
       <c r="BI105" t="s">
-        <v>2218</v>
+        <v>2236</v>
       </c>
       <c r="BJ105" t="s">
-        <v>2219</v>
+        <v>2237</v>
       </c>
       <c r="BK105">
         <v>0.90109890109890123</v>
@@ -42491,7 +42491,7 @@
         <v>7.3789928117601003E-2</v>
       </c>
       <c r="BQ105" t="s">
-        <v>2220</v>
+        <v>2238</v>
       </c>
       <c r="BR105">
         <v>0.95421245421245426</v>
@@ -42503,10 +42503,10 @@
         <v>2.554741077704686E-2</v>
       </c>
       <c r="BU105" t="s">
-        <v>2221</v>
+        <v>2239</v>
       </c>
       <c r="BV105" t="s">
-        <v>2222</v>
+        <v>2240</v>
       </c>
       <c r="BW105">
         <v>0.92018191892141477</v>
@@ -42527,10 +42527,10 @@
         <v>8.1762915663579853E-3</v>
       </c>
       <c r="CC105" t="s">
-        <v>2223</v>
+        <v>2241</v>
       </c>
       <c r="CD105" t="s">
-        <v>2224</v>
+        <v>2242</v>
       </c>
       <c r="CE105">
         <v>0.93637033838619221</v>
@@ -42542,7 +42542,7 @@
         <v>6.3421069865930886E-3</v>
       </c>
       <c r="CH105" t="s">
-        <v>2225</v>
+        <v>2243</v>
       </c>
       <c r="CI105">
         <v>0.89241751927092661</v>
@@ -42563,10 +42563,10 @@
         <v>1.0895547946837321E-2</v>
       </c>
       <c r="CO105" t="s">
-        <v>2226</v>
+        <v>2244</v>
       </c>
       <c r="CP105" t="s">
-        <v>2227</v>
+        <v>2245</v>
       </c>
       <c r="CQ105">
         <v>0.97689032399265263</v>
@@ -42587,10 +42587,10 @@
         <v>2.4353139415404089E-2</v>
       </c>
       <c r="CW105" t="s">
-        <v>2228</v>
+        <v>2246</v>
       </c>
       <c r="CX105" t="s">
-        <v>2229</v>
+        <v>2247</v>
       </c>
       <c r="CY105">
         <v>0.8992673992673994</v>
@@ -42611,7 +42611,7 @@
         <v>1.534362094470151E-2</v>
       </c>
       <c r="DE105" t="s">
-        <v>2230</v>
+        <v>2248</v>
       </c>
       <c r="DF105">
         <v>0.97135144656153061</v>

</xml_diff>